<commit_message>
fix v307 spec[1] bug
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saran\Documents\Academia\repository_clones\Bioindustrial-Park\biorefineries\isobutanol\analyses\full\parameter_distributions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99F2905E-03D1-48B1-8849-2E58554BEF56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4E8C7A6-970B-48D3-885C-1315790FC9EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>

<commit_message>
change element annotations in param dists
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saran\Documents\Academia\repository_clones\Bioindustrial-Park\biorefineries\isobutanol\analyses\full\parameter_distributions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4E8C7A6-970B-48D3-885C-1315790FC9EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{282165B5-C9C4-4E9A-A06F-BB9F0F389DFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="160">
   <si>
     <t>Parameter name</t>
   </si>
@@ -209,9 +209,6 @@
     <t>V514.tau = x</t>
   </si>
   <si>
-    <t>Fermentation Kinetics</t>
-  </si>
-  <si>
     <t>V406.kinetic_reaction_system._te.k_2 = x</t>
   </si>
   <si>
@@ -486,6 +483,39 @@
   </si>
   <si>
     <t>._k_11</t>
+  </si>
+  <si>
+    <t>Kinetics: Glycolysis</t>
+  </si>
+  <si>
+    <t>Kinetics: TCA Cycle</t>
+  </si>
+  <si>
+    <t>Kinetics: Pyruvate-to-Acetaldehyde</t>
+  </si>
+  <si>
+    <t>Kinetics: Acetaldehyde-to-Acetate</t>
+  </si>
+  <si>
+    <t>Kinetics: Acetaldyhede-to-Ethanol</t>
+  </si>
+  <si>
+    <t>Kinetics: Glucose-to-Biomass</t>
+  </si>
+  <si>
+    <t>Kinetics: Acetate-to-Biomass</t>
+  </si>
+  <si>
+    <t>Kinetics: Acetalhdyde compartment formation</t>
+  </si>
+  <si>
+    <t>Kinetics: Acetate respiration</t>
+  </si>
+  <si>
+    <t>Kinetics: Active compartment degradation</t>
+  </si>
+  <si>
+    <t>Kinetics: Acetaldehyde compartment degradation</t>
   </si>
 </sst>
 </file>
@@ -509,7 +539,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -519,6 +549,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -550,7 +586,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -561,6 +597,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -955,70 +992,70 @@
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="6">
         <v>0.13900000000000001</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="6">
         <v>0.127</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="6">
         <f>E4</f>
         <v>0.13900000000000001</v>
       </c>
-      <c r="I4" s="3">
+      <c r="I4" s="6">
         <v>0.15</v>
       </c>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3" t="s">
+      <c r="J4" s="6"/>
+      <c r="K4" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="6">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="6">
         <v>6.7000000000000004E-2</v>
       </c>
-      <c r="H5" s="3">
+      <c r="H5" s="6">
         <f>E5</f>
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="I5" s="3">
+      <c r="I5" s="6">
         <v>7.3999999999999996E-2</v>
       </c>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3" t="s">
+      <c r="J5" s="6"/>
+      <c r="K5" s="6" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1217,76 +1254,76 @@
       </c>
       <c r="J11" s="4"/>
       <c r="K11" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E12" s="6">
         <v>0.28599999999999998</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G12" s="3">
+      <c r="G12" s="6">
         <v>0.17499999999999999</v>
       </c>
-      <c r="H12" s="3">
+      <c r="H12" s="6">
         <v>0.28599999999999998</v>
       </c>
-      <c r="I12" s="3">
+      <c r="I12" s="6">
         <v>0.315</v>
       </c>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3" t="s">
-        <v>87</v>
+      <c r="J12" s="6"/>
+      <c r="K12" s="6" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E13" s="3">
+      <c r="E13" s="6">
         <v>0.10355</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G13" s="3">
+      <c r="G13" s="6">
         <f>E13*0.9</f>
         <v>9.3195E-2</v>
       </c>
-      <c r="H13" s="3">
+      <c r="H13" s="6">
         <f>E13</f>
         <v>0.10355</v>
       </c>
-      <c r="I13" s="3">
+      <c r="I13" s="6">
         <f>E13*1.1</f>
         <v>0.11390500000000001</v>
       </c>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3" t="s">
-        <v>88</v>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
@@ -1463,22 +1500,22 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>57</v>
+        <v>149</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E19" s="3">
         <v>1.43</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G19" s="3">
         <v>1.1439999999999999</v>
@@ -1491,27 +1528,27 @@
       </c>
       <c r="J19" s="3"/>
       <c r="K19" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>57</v>
+        <v>149</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E20" s="3">
         <v>0.94</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G20" s="3">
         <v>0.752</v>
@@ -1524,27 +1561,27 @@
       </c>
       <c r="J20" s="3"/>
       <c r="K20" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>57</v>
+        <v>149</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E21" s="3">
         <v>0.58399999999999996</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G21" s="3">
         <v>0.4672</v>
@@ -1557,27 +1594,27 @@
       </c>
       <c r="J21" s="3"/>
       <c r="K21" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>57</v>
+        <v>149</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E22" s="3">
         <v>1.1599999999999999E-2</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G22" s="3">
         <v>9.2800000000000001E-3</v>
@@ -1590,27 +1627,27 @@
       </c>
       <c r="J22" s="3"/>
       <c r="K22" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>57</v>
+        <v>149</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E23" s="3">
         <v>47.1</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G23" s="3">
         <v>37.68</v>
@@ -1623,27 +1660,27 @@
       </c>
       <c r="J23" s="3"/>
       <c r="K23" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>57</v>
+        <v>149</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E24" s="3">
         <v>14.2</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G24" s="3">
         <v>11.36</v>
@@ -1656,27 +1693,27 @@
       </c>
       <c r="J24" s="3"/>
       <c r="K24" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>57</v>
+        <v>149</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E25" s="3">
         <v>0.12</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G25" s="3">
         <v>9.6000000000000002E-2</v>
@@ -1689,27 +1726,27 @@
       </c>
       <c r="J25" s="3"/>
       <c r="K25" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>57</v>
+        <v>149</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E26" s="3">
         <v>0.04</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G26" s="3">
         <v>3.2000000000000001E-2</v>
@@ -1722,27 +1759,27 @@
       </c>
       <c r="J26" s="3"/>
       <c r="K26" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>57</v>
+        <v>149</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E27" s="3">
         <v>0.12</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G27" s="3">
         <v>9.6000000000000002E-2</v>
@@ -1755,27 +1792,27 @@
       </c>
       <c r="J27" s="3"/>
       <c r="K27" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>57</v>
+        <v>149</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E28" s="3">
         <v>0.04</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G28" s="3">
         <v>3.2000000000000001E-2</v>
@@ -1788,27 +1825,27 @@
       </c>
       <c r="J28" s="3"/>
       <c r="K28" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>57</v>
+        <v>150</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E29" s="3">
         <v>0.501</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G29" s="3">
         <v>0.40079999999999999</v>
@@ -1821,27 +1858,27 @@
       </c>
       <c r="J29" s="3"/>
       <c r="K29" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>57</v>
+        <v>150</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E30" s="5">
         <v>2.0000000000000002E-5</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G30" s="5">
         <v>1.5999999999999999E-5</v>
@@ -1854,27 +1891,27 @@
       </c>
       <c r="J30" s="3"/>
       <c r="K30" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>57</v>
+        <v>150</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E31" s="3">
         <v>0.10100000000000001</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G31" s="3">
         <v>8.0799999999999997E-2</v>
@@ -1887,27 +1924,27 @@
       </c>
       <c r="J31" s="3"/>
       <c r="K31" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>57</v>
+        <v>151</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E32" s="3">
         <v>5.81</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G32" s="3">
         <v>4.6479999999999997</v>
@@ -1920,27 +1957,27 @@
       </c>
       <c r="J32" s="3"/>
       <c r="K32" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>57</v>
+        <v>151</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E33" s="5">
         <v>4.9999999999999998E-7</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G33" s="5">
         <v>3.9999999999999998E-7</v>
@@ -1953,27 +1990,27 @@
       </c>
       <c r="J33" s="3"/>
       <c r="K33" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>57</v>
+        <v>152</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E34" s="3">
         <v>4.8</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G34" s="3">
         <v>3.84</v>
@@ -1986,27 +2023,27 @@
       </c>
       <c r="J34" s="3"/>
       <c r="K34" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>57</v>
+        <v>152</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E35" s="3">
         <v>0.04</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G35" s="3">
         <v>3.2000000000000001E-2</v>
@@ -2019,27 +2056,27 @@
       </c>
       <c r="J35" s="3"/>
       <c r="K35" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>57</v>
+        <v>152</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E36" s="3">
         <v>0.12</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G36" s="3">
         <v>9.6000000000000002E-2</v>
@@ -2052,27 +2089,27 @@
       </c>
       <c r="J36" s="3"/>
       <c r="K36" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>57</v>
+        <v>152</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E37" s="3">
         <v>0.04</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G37" s="3">
         <v>3.2000000000000001E-2</v>
@@ -2085,27 +2122,27 @@
       </c>
       <c r="J37" s="3"/>
       <c r="K37" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>57</v>
+        <v>152</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E38" s="3">
         <v>2.6400000000000002E-4</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G38" s="3">
         <v>2.1120000000000001E-4</v>
@@ -2118,27 +2155,27 @@
       </c>
       <c r="J38" s="3"/>
       <c r="K38" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>57</v>
+        <v>157</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E39" s="3">
         <v>1.04E-2</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G39" s="3">
         <v>8.3199999999999993E-3</v>
@@ -2151,27 +2188,27 @@
       </c>
       <c r="J39" s="3"/>
       <c r="K39" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>57</v>
+        <v>157</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E40" s="3">
         <v>1.0200000000000001E-2</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G40" s="3">
         <v>8.1600000000000006E-3</v>
@@ -2184,27 +2221,27 @@
       </c>
       <c r="J40" s="3"/>
       <c r="K40" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>57</v>
+        <v>157</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E41" s="3">
         <v>0.77500000000000002</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G41" s="3">
         <v>0.62</v>
@@ -2217,27 +2254,27 @@
       </c>
       <c r="J41" s="3"/>
       <c r="K41" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>57</v>
+        <v>157</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E42" s="3">
         <v>0.1</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G42" s="3">
         <v>0.08</v>
@@ -2250,27 +2287,27 @@
       </c>
       <c r="J42" s="3"/>
       <c r="K42" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>57</v>
+        <v>157</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E43" s="3">
         <v>440</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G43" s="3">
         <v>352</v>
@@ -2283,27 +2320,27 @@
       </c>
       <c r="J43" s="3"/>
       <c r="K43" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>57</v>
+        <v>153</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E44" s="3">
         <v>2.82</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G44" s="3">
         <v>2.2559999999999998</v>
@@ -2316,27 +2353,27 @@
       </c>
       <c r="J44" s="3"/>
       <c r="K44" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>57</v>
+        <v>153</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E45" s="3">
         <v>1.2500000000000001E-2</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G45" s="3">
         <v>0.01</v>
@@ -2349,27 +2386,27 @@
       </c>
       <c r="J45" s="3"/>
       <c r="K45" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>57</v>
+        <v>153</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E46" s="3">
         <v>3.4000000000000002E-2</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G46" s="3">
         <v>2.7199999999999998E-2</v>
@@ -2382,27 +2419,27 @@
       </c>
       <c r="J46" s="3"/>
       <c r="K46" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>57</v>
+        <v>153</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E47" s="3">
         <v>5.7000000000000002E-2</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G47" s="3">
         <v>4.5600000000000002E-2</v>
@@ -2415,27 +2452,27 @@
       </c>
       <c r="J47" s="3"/>
       <c r="K47" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>57</v>
+        <v>154</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E48" s="3">
         <v>1.2030000000000001</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G48" s="3">
         <v>0.96240000000000003</v>
@@ -2448,27 +2485,27 @@
       </c>
       <c r="J48" s="3"/>
       <c r="K48" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>57</v>
+        <v>154</v>
       </c>
       <c r="C49" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E49" s="3">
         <v>0.04</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G49" s="3">
         <v>3.2000000000000001E-2</v>
@@ -2481,27 +2518,27 @@
       </c>
       <c r="J49" s="3"/>
       <c r="K49" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>57</v>
+        <v>154</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E50" s="3">
         <v>0.12</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G50" s="3">
         <v>9.6000000000000002E-2</v>
@@ -2514,27 +2551,27 @@
       </c>
       <c r="J50" s="3"/>
       <c r="K50" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>57</v>
+        <v>154</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E51" s="3">
         <v>0.04</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G51" s="3">
         <v>3.2000000000000001E-2</v>
@@ -2547,27 +2584,27 @@
       </c>
       <c r="J51" s="3"/>
       <c r="K51" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>57</v>
+        <v>154</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E52" s="3">
         <v>1.01E-2</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G52" s="3">
         <v>8.0800000000000004E-3</v>
@@ -2580,27 +2617,27 @@
       </c>
       <c r="J52" s="3"/>
       <c r="K52" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>57</v>
+        <v>155</v>
       </c>
       <c r="C53" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E53" s="3">
         <v>0.58899999999999997</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G53" s="3">
         <v>0.47120000000000001</v>
@@ -2613,27 +2650,27 @@
       </c>
       <c r="J53" s="3"/>
       <c r="K53" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>57</v>
+        <v>156</v>
       </c>
       <c r="C54" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E54" s="3">
         <v>8.0000000000000002E-3</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G54" s="3">
         <v>6.4000000000000003E-3</v>
@@ -2646,27 +2683,27 @@
       </c>
       <c r="J54" s="3"/>
       <c r="K54" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>57</v>
+        <v>156</v>
       </c>
       <c r="C55" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E55" s="5">
         <v>9.9999999999999995E-7</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G55" s="5">
         <v>7.9999999999999996E-7</v>
@@ -2679,27 +2716,27 @@
       </c>
       <c r="J55" s="3"/>
       <c r="K55" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>57</v>
+        <v>156</v>
       </c>
       <c r="C56" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E56" s="3">
         <v>7.51E-2</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G56" s="3">
         <v>6.0080000000000001E-2</v>
@@ -2712,27 +2749,27 @@
       </c>
       <c r="J56" s="3"/>
       <c r="K56" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>57</v>
+        <v>156</v>
       </c>
       <c r="C57" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E57" s="3">
         <v>13</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G57" s="3">
         <v>10.4</v>
@@ -2745,27 +2782,27 @@
       </c>
       <c r="J57" s="3"/>
       <c r="K57" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>57</v>
+        <v>156</v>
       </c>
       <c r="C58" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E58" s="3">
         <v>25</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G58" s="3">
         <v>20</v>
@@ -2778,27 +2815,27 @@
       </c>
       <c r="J58" s="3"/>
       <c r="K58" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>57</v>
+        <v>156</v>
       </c>
       <c r="C59" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E59" s="3">
         <v>3.9899999999999996E-3</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G59" s="3">
         <v>3.192E-3</v>
@@ -2811,27 +2848,27 @@
       </c>
       <c r="J59" s="3"/>
       <c r="K59" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>57</v>
+        <v>158</v>
       </c>
       <c r="C60" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E60" s="3">
         <v>0.06</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G60" s="3">
         <v>4.8000000000000001E-2</v>
@@ -2844,27 +2881,27 @@
       </c>
       <c r="J60" s="3"/>
       <c r="K60" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>57</v>
+        <v>159</v>
       </c>
       <c r="C61" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E61" s="3">
         <v>0.02</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G61" s="3">
         <v>1.6E-2</v>
@@ -2877,7 +2914,7 @@
       </c>
       <c r="J61" s="3"/>
       <c r="K61" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix unit group breakdowns
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saran\Documents\Academia\repository_clones\Bioindustrial-Park\biorefineries\isobutanol\analyses\full\parameter_distributions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{282165B5-C9C4-4E9A-A06F-BB9F0F389DFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73F6C879-74A0-4369-BA32-FCA612BBAF30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="163">
   <si>
     <t>Parameter name</t>
   </si>
@@ -516,6 +516,15 @@
   </si>
   <si>
     <t>Kinetics: Acetaldehyde compartment degradation</t>
+  </si>
+  <si>
+    <t>DDGS price</t>
+  </si>
+  <si>
+    <t>Isobutanol price</t>
+  </si>
+  <si>
+    <t>Isopentyl acetate price</t>
   </si>
 </sst>
 </file>
@@ -878,7 +887,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K61"/>
+  <dimension ref="A1:K64"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="40.81640625" customWidth="1"/>
@@ -1258,348 +1267,312 @@
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A13" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A14" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A15" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B15" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C15" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D15" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E15" s="6">
         <v>0.28599999999999998</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F15" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G12" s="6">
+      <c r="G15" s="6">
         <v>0.17499999999999999</v>
       </c>
-      <c r="H12" s="6">
+      <c r="H15" s="6">
         <v>0.28599999999999998</v>
       </c>
-      <c r="I12" s="6">
+      <c r="I15" s="6">
         <v>0.315</v>
       </c>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6" t="s">
+      <c r="J15" s="6"/>
+      <c r="K15" s="6" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A13" s="6" t="s">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A16" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B16" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C16" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D16" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E16" s="6">
         <v>0.10355</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="F16" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G13" s="6">
-        <f>E13*0.9</f>
+      <c r="G16" s="6">
+        <f>E16*0.9</f>
         <v>9.3195E-2</v>
       </c>
-      <c r="H13" s="6">
-        <f>E13</f>
+      <c r="H16" s="6">
+        <f>E16</f>
         <v>0.10355</v>
       </c>
-      <c r="I13" s="6">
-        <f>E13*1.1</f>
+      <c r="I16" s="6">
+        <f>E16*1.1</f>
         <v>0.11390500000000001</v>
       </c>
-      <c r="J13" s="6"/>
-      <c r="K13" s="6" t="s">
+      <c r="J16" s="6"/>
+      <c r="K16" s="6" t="s">
         <v>87</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A14" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E14" s="3">
-        <v>0.21</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G14" s="3">
-        <v>0.15</v>
-      </c>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3">
-        <v>0.28000000000000003</v>
-      </c>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A15" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E15" s="3">
-        <v>0.15</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G15" s="3">
-        <f>0.8*E15</f>
-        <v>0.12</v>
-      </c>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3">
-        <f>1.2*E15</f>
-        <v>0.18</v>
-      </c>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A16" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="E16" s="3">
-        <v>56972</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="G16" s="3">
-        <f>0.8*H16</f>
-        <v>45577.600000000006</v>
-      </c>
-      <c r="H16" s="3">
-        <f>E16</f>
-        <v>56972</v>
-      </c>
-      <c r="I16" s="3">
-        <f>1.2*H16</f>
-        <v>68366.399999999994</v>
-      </c>
-      <c r="J16" s="3"/>
-      <c r="K16" s="3" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="E17" s="3">
-        <v>156</v>
+        <v>0.21</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="G17" s="3">
-        <f>E17*0.8</f>
-        <v>124.80000000000001</v>
-      </c>
-      <c r="H17" s="3">
-        <f>E17</f>
-        <v>156</v>
-      </c>
+        <v>0.15</v>
+      </c>
+      <c r="H17" s="3"/>
       <c r="I17" s="3">
-        <f>E17*1.2</f>
-        <v>187.2</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="J17" s="3"/>
       <c r="K17" s="3" t="s">
-        <v>55</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="E18" s="3">
-        <v>156</v>
+        <v>0.15</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="G18" s="3">
-        <f>E18*0.8</f>
-        <v>124.80000000000001</v>
-      </c>
-      <c r="H18" s="3">
-        <f>E18</f>
-        <v>156</v>
-      </c>
+        <f>0.8*E18</f>
+        <v>0.12</v>
+      </c>
+      <c r="H18" s="3"/>
       <c r="I18" s="3">
-        <f>E18*1.2</f>
-        <v>187.2</v>
+        <f>1.2*E18</f>
+        <v>0.18</v>
       </c>
       <c r="J18" s="3"/>
       <c r="K18" s="3" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>123</v>
+        <v>38</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>149</v>
+        <v>39</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>66</v>
+        <v>40</v>
       </c>
       <c r="E19" s="3">
-        <v>1.43</v>
+        <v>56972</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>67</v>
+        <v>27</v>
       </c>
       <c r="G19" s="3">
-        <v>1.1439999999999999</v>
+        <f>0.8*H19</f>
+        <v>45577.600000000006</v>
       </c>
       <c r="H19" s="3">
-        <v>1.43</v>
+        <f>E19</f>
+        <v>56972</v>
       </c>
       <c r="I19" s="3">
-        <v>1.716</v>
+        <f>1.2*H19</f>
+        <v>68366.399999999994</v>
       </c>
       <c r="J19" s="3"/>
       <c r="K19" s="3" t="s">
-        <v>63</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>106</v>
+        <v>53</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>149</v>
+        <v>13</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>68</v>
+        <v>14</v>
       </c>
       <c r="E20" s="3">
-        <v>0.94</v>
+        <v>156</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>67</v>
+        <v>27</v>
       </c>
       <c r="G20" s="3">
-        <v>0.752</v>
+        <f>E20*0.8</f>
+        <v>124.80000000000001</v>
       </c>
       <c r="H20" s="3">
-        <v>0.94</v>
+        <f>E20</f>
+        <v>156</v>
       </c>
       <c r="I20" s="3">
-        <v>1.1279999999999999</v>
+        <f>E20*1.2</f>
+        <v>187.2</v>
       </c>
       <c r="J20" s="3"/>
       <c r="K20" s="3" t="s">
-        <v>88</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>124</v>
+        <v>54</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>149</v>
+        <v>13</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>66</v>
+        <v>14</v>
       </c>
       <c r="E21" s="3">
-        <v>0.58399999999999996</v>
+        <v>156</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>67</v>
+        <v>27</v>
       </c>
       <c r="G21" s="3">
-        <v>0.4672</v>
+        <f>E21*0.8</f>
+        <v>124.80000000000001</v>
       </c>
       <c r="H21" s="3">
-        <v>0.58399999999999996</v>
+        <f>E21</f>
+        <v>156</v>
       </c>
       <c r="I21" s="3">
-        <v>0.70079999999999998</v>
+        <f>E21*1.2</f>
+        <v>187.2</v>
       </c>
       <c r="J21" s="3"/>
       <c r="K21" s="3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>149</v>
@@ -1608,31 +1581,31 @@
         <v>21</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E22" s="3">
-        <v>1.1599999999999999E-2</v>
+        <v>1.43</v>
       </c>
       <c r="F22" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G22" s="3">
-        <v>9.2800000000000001E-3</v>
+        <v>1.1439999999999999</v>
       </c>
       <c r="H22" s="3">
-        <v>1.1599999999999999E-2</v>
+        <v>1.43</v>
       </c>
       <c r="I22" s="3">
-        <v>1.3919999999999899E-2</v>
+        <v>1.716</v>
       </c>
       <c r="J22" s="3"/>
       <c r="K22" s="3" t="s">
-        <v>89</v>
+        <v>63</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>125</v>
+        <v>106</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>149</v>
@@ -1641,31 +1614,31 @@
         <v>21</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E23" s="3">
-        <v>47.1</v>
+        <v>0.94</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G23" s="3">
-        <v>37.68</v>
+        <v>0.752</v>
       </c>
       <c r="H23" s="3">
-        <v>47.1</v>
+        <v>0.94</v>
       </c>
       <c r="I23" s="3">
-        <v>56.52</v>
+        <v>1.1279999999999999</v>
       </c>
       <c r="J23" s="3"/>
       <c r="K23" s="3" t="s">
-        <v>58</v>
+        <v>88</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>149</v>
@@ -1674,31 +1647,31 @@
         <v>21</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E24" s="3">
-        <v>14.2</v>
+        <v>0.58399999999999996</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G24" s="3">
-        <v>11.36</v>
+        <v>0.4672</v>
       </c>
       <c r="H24" s="3">
-        <v>14.2</v>
+        <v>0.58399999999999996</v>
       </c>
       <c r="I24" s="3">
-        <v>17.04</v>
+        <v>0.70079999999999998</v>
       </c>
       <c r="J24" s="3"/>
       <c r="K24" s="3" t="s">
-        <v>90</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>149</v>
@@ -1710,28 +1683,28 @@
         <v>68</v>
       </c>
       <c r="E25" s="3">
-        <v>0.12</v>
+        <v>1.1599999999999999E-2</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G25" s="3">
-        <v>9.6000000000000002E-2</v>
+        <v>9.2800000000000001E-3</v>
       </c>
       <c r="H25" s="3">
-        <v>0.12</v>
+        <v>1.1599999999999999E-2</v>
       </c>
       <c r="I25" s="3">
-        <v>0.14399999999999999</v>
+        <v>1.3919999999999899E-2</v>
       </c>
       <c r="J25" s="3"/>
       <c r="K25" s="3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>149</v>
@@ -1743,28 +1716,28 @@
         <v>66</v>
       </c>
       <c r="E26" s="3">
-        <v>0.04</v>
+        <v>47.1</v>
       </c>
       <c r="F26" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G26" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>37.68</v>
       </c>
       <c r="H26" s="3">
-        <v>0.04</v>
+        <v>47.1</v>
       </c>
       <c r="I26" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>56.52</v>
       </c>
       <c r="J26" s="3"/>
       <c r="K26" s="3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>149</v>
@@ -1773,31 +1746,31 @@
         <v>21</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E27" s="3">
-        <v>0.12</v>
+        <v>14.2</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G27" s="3">
-        <v>9.6000000000000002E-2</v>
+        <v>11.36</v>
       </c>
       <c r="H27" s="3">
-        <v>0.12</v>
+        <v>14.2</v>
       </c>
       <c r="I27" s="3">
-        <v>0.14399999999999999</v>
+        <v>17.04</v>
       </c>
       <c r="J27" s="3"/>
       <c r="K27" s="3" t="s">
-        <v>61</v>
+        <v>90</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>149</v>
@@ -1806,34 +1779,34 @@
         <v>21</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E28" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G28" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="H28" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="I28" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="J28" s="3"/>
       <c r="K28" s="3" t="s">
-        <v>62</v>
+        <v>91</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>21</v>
@@ -1842,97 +1815,97 @@
         <v>66</v>
       </c>
       <c r="E29" s="3">
-        <v>0.501</v>
+        <v>0.04</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G29" s="3">
-        <v>0.40079999999999999</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H29" s="3">
-        <v>0.501</v>
+        <v>0.04</v>
       </c>
       <c r="I29" s="3">
-        <v>0.60119999999999996</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J29" s="3"/>
       <c r="K29" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E30" s="5">
-        <v>2.0000000000000002E-5</v>
+        <v>66</v>
+      </c>
+      <c r="E30" s="3">
+        <v>0.12</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G30" s="5">
-        <v>1.5999999999999999E-5</v>
-      </c>
-      <c r="H30" s="5">
-        <v>2.0000000000000002E-5</v>
-      </c>
-      <c r="I30" s="5">
-        <v>2.4000000000000001E-5</v>
+      <c r="G30" s="3">
+        <v>9.6000000000000002E-2</v>
+      </c>
+      <c r="H30" s="3">
+        <v>0.12</v>
+      </c>
+      <c r="I30" s="3">
+        <v>0.14399999999999999</v>
       </c>
       <c r="J30" s="3"/>
       <c r="K30" s="3" t="s">
-        <v>92</v>
+        <v>61</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E31" s="3">
-        <v>0.10100000000000001</v>
+        <v>0.04</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G31" s="3">
-        <v>8.0799999999999997E-2</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H31" s="3">
-        <v>0.10100000000000001</v>
+        <v>0.04</v>
       </c>
       <c r="I31" s="3">
-        <v>0.1212</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J31" s="3"/>
       <c r="K31" s="3" t="s">
-        <v>93</v>
+        <v>62</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>21</v>
@@ -1941,31 +1914,31 @@
         <v>66</v>
       </c>
       <c r="E32" s="3">
-        <v>5.81</v>
+        <v>0.501</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G32" s="3">
-        <v>4.6479999999999997</v>
+        <v>0.40079999999999999</v>
       </c>
       <c r="H32" s="3">
-        <v>5.81</v>
+        <v>0.501</v>
       </c>
       <c r="I32" s="3">
-        <v>6.9719999999999898</v>
+        <v>0.60119999999999996</v>
       </c>
       <c r="J32" s="3"/>
       <c r="K32" s="3" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>21</v>
@@ -1974,64 +1947,64 @@
         <v>68</v>
       </c>
       <c r="E33" s="5">
-        <v>4.9999999999999998E-7</v>
+        <v>2.0000000000000002E-5</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G33" s="5">
-        <v>3.9999999999999998E-7</v>
+        <v>1.5999999999999999E-5</v>
       </c>
       <c r="H33" s="5">
-        <v>4.9999999999999998E-7</v>
+        <v>2.0000000000000002E-5</v>
       </c>
       <c r="I33" s="5">
-        <v>5.9999999999999997E-7</v>
+        <v>2.4000000000000001E-5</v>
       </c>
       <c r="J33" s="3"/>
       <c r="K33" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
-        <v>131</v>
+        <v>111</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E34" s="3">
-        <v>4.8</v>
+        <v>0.10100000000000001</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G34" s="3">
-        <v>3.84</v>
+        <v>8.0799999999999997E-2</v>
       </c>
       <c r="H34" s="3">
-        <v>4.8</v>
+        <v>0.10100000000000001</v>
       </c>
       <c r="I34" s="3">
-        <v>5.76</v>
+        <v>0.1212</v>
       </c>
       <c r="J34" s="3"/>
       <c r="K34" s="3" t="s">
-        <v>65</v>
+        <v>93</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>21</v>
@@ -2040,61 +2013,61 @@
         <v>66</v>
       </c>
       <c r="E35" s="3">
-        <v>0.04</v>
+        <v>5.81</v>
       </c>
       <c r="F35" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G35" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>4.6479999999999997</v>
       </c>
       <c r="H35" s="3">
-        <v>0.04</v>
+        <v>5.81</v>
       </c>
       <c r="I35" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>6.9719999999999898</v>
       </c>
       <c r="J35" s="3"/>
       <c r="K35" s="3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
-        <v>133</v>
+        <v>112</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="E36" s="3">
-        <v>0.12</v>
+        <v>68</v>
+      </c>
+      <c r="E36" s="5">
+        <v>4.9999999999999998E-7</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G36" s="3">
-        <v>9.6000000000000002E-2</v>
-      </c>
-      <c r="H36" s="3">
-        <v>0.12</v>
-      </c>
-      <c r="I36" s="3">
-        <v>0.14399999999999999</v>
+      <c r="G36" s="5">
+        <v>3.9999999999999998E-7</v>
+      </c>
+      <c r="H36" s="5">
+        <v>4.9999999999999998E-7</v>
+      </c>
+      <c r="I36" s="5">
+        <v>5.9999999999999997E-7</v>
       </c>
       <c r="J36" s="3"/>
       <c r="K36" s="3" t="s">
-        <v>70</v>
+        <v>94</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>152</v>
@@ -2106,28 +2079,28 @@
         <v>66</v>
       </c>
       <c r="E37" s="3">
-        <v>0.04</v>
+        <v>4.8</v>
       </c>
       <c r="F37" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G37" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>3.84</v>
       </c>
       <c r="H37" s="3">
-        <v>0.04</v>
+        <v>4.8</v>
       </c>
       <c r="I37" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>5.76</v>
       </c>
       <c r="J37" s="3"/>
       <c r="K37" s="3" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
-        <v>113</v>
+        <v>132</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>152</v>
@@ -2136,34 +2109,34 @@
         <v>21</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E38" s="3">
-        <v>2.6400000000000002E-4</v>
+        <v>0.04</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G38" s="3">
-        <v>2.1120000000000001E-4</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H38" s="3">
-        <v>2.6400000000000002E-4</v>
+        <v>0.04</v>
       </c>
       <c r="I38" s="3">
-        <v>3.168E-4</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J38" s="3"/>
       <c r="K38" s="3" t="s">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>21</v>
@@ -2172,94 +2145,94 @@
         <v>66</v>
       </c>
       <c r="E39" s="3">
-        <v>1.04E-2</v>
+        <v>0.12</v>
       </c>
       <c r="F39" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G39" s="3">
-        <v>8.3199999999999993E-3</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="H39" s="3">
-        <v>1.04E-2</v>
+        <v>0.12</v>
       </c>
       <c r="I39" s="3">
-        <v>1.248E-2</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="J39" s="3"/>
       <c r="K39" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
-        <v>114</v>
+        <v>134</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E40" s="3">
-        <v>1.0200000000000001E-2</v>
+        <v>0.04</v>
       </c>
       <c r="F40" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G40" s="3">
-        <v>8.1600000000000006E-3</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H40" s="3">
-        <v>1.0200000000000001E-2</v>
+        <v>0.04</v>
       </c>
       <c r="I40" s="3">
-        <v>1.2239999999999999E-2</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J40" s="3"/>
       <c r="K40" s="3" t="s">
-        <v>96</v>
+        <v>71</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
-        <v>136</v>
+        <v>113</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E41" s="3">
-        <v>0.77500000000000002</v>
+        <v>2.6400000000000002E-4</v>
       </c>
       <c r="F41" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G41" s="3">
-        <v>0.62</v>
+        <v>2.1120000000000001E-4</v>
       </c>
       <c r="H41" s="3">
-        <v>0.77500000000000002</v>
+        <v>2.6400000000000002E-4</v>
       </c>
       <c r="I41" s="3">
-        <v>0.92999999999999905</v>
+        <v>3.168E-4</v>
       </c>
       <c r="J41" s="3"/>
       <c r="K41" s="3" t="s">
-        <v>73</v>
+        <v>95</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
-        <v>115</v>
+        <v>135</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>157</v>
@@ -2268,31 +2241,31 @@
         <v>21</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E42" s="3">
-        <v>0.1</v>
+        <v>1.04E-2</v>
       </c>
       <c r="F42" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G42" s="3">
-        <v>0.08</v>
+        <v>8.3199999999999993E-3</v>
       </c>
       <c r="H42" s="3">
-        <v>0.1</v>
+        <v>1.04E-2</v>
       </c>
       <c r="I42" s="3">
-        <v>0.12</v>
+        <v>1.248E-2</v>
       </c>
       <c r="J42" s="3"/>
       <c r="K42" s="3" t="s">
-        <v>97</v>
+        <v>72</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>157</v>
@@ -2304,31 +2277,31 @@
         <v>68</v>
       </c>
       <c r="E43" s="3">
-        <v>440</v>
+        <v>1.0200000000000001E-2</v>
       </c>
       <c r="F43" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G43" s="3">
-        <v>352</v>
+        <v>8.1600000000000006E-3</v>
       </c>
       <c r="H43" s="3">
-        <v>440</v>
+        <v>1.0200000000000001E-2</v>
       </c>
       <c r="I43" s="3">
-        <v>528</v>
+        <v>1.2239999999999999E-2</v>
       </c>
       <c r="J43" s="3"/>
       <c r="K43" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>21</v>
@@ -2337,64 +2310,64 @@
         <v>66</v>
       </c>
       <c r="E44" s="3">
-        <v>2.82</v>
+        <v>0.77500000000000002</v>
       </c>
       <c r="F44" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G44" s="3">
-        <v>2.2559999999999998</v>
+        <v>0.62</v>
       </c>
       <c r="H44" s="3">
-        <v>2.82</v>
+        <v>0.77500000000000002</v>
       </c>
       <c r="I44" s="3">
-        <v>3.3839999999999999</v>
+        <v>0.92999999999999905</v>
       </c>
       <c r="J44" s="3"/>
       <c r="K44" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" s="3" t="s">
-        <v>138</v>
+        <v>115</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E45" s="3">
-        <v>1.2500000000000001E-2</v>
+        <v>0.1</v>
       </c>
       <c r="F45" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G45" s="3">
-        <v>0.01</v>
+        <v>0.08</v>
       </c>
       <c r="H45" s="3">
-        <v>1.2500000000000001E-2</v>
+        <v>0.1</v>
       </c>
       <c r="I45" s="3">
-        <v>1.4999999999999999E-2</v>
+        <v>0.12</v>
       </c>
       <c r="J45" s="3"/>
       <c r="K45" s="3" t="s">
-        <v>75</v>
+        <v>97</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>21</v>
@@ -2403,28 +2376,28 @@
         <v>68</v>
       </c>
       <c r="E46" s="3">
-        <v>3.4000000000000002E-2</v>
+        <v>440</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G46" s="3">
-        <v>2.7199999999999998E-2</v>
+        <v>352</v>
       </c>
       <c r="H46" s="3">
-        <v>3.4000000000000002E-2</v>
+        <v>440</v>
       </c>
       <c r="I46" s="3">
-        <v>4.0800000000000003E-2</v>
+        <v>528</v>
       </c>
       <c r="J46" s="3"/>
       <c r="K46" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" s="3" t="s">
-        <v>118</v>
+        <v>137</v>
       </c>
       <c r="B47" s="3" t="s">
         <v>153</v>
@@ -2433,34 +2406,34 @@
         <v>21</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E47" s="3">
-        <v>5.7000000000000002E-2</v>
+        <v>2.82</v>
       </c>
       <c r="F47" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G47" s="3">
-        <v>4.5600000000000002E-2</v>
+        <v>2.2559999999999998</v>
       </c>
       <c r="H47" s="3">
-        <v>5.7000000000000002E-2</v>
+        <v>2.82</v>
       </c>
       <c r="I47" s="3">
-        <v>6.8400000000000002E-2</v>
+        <v>3.3839999999999999</v>
       </c>
       <c r="J47" s="3"/>
       <c r="K47" s="3" t="s">
-        <v>100</v>
+        <v>74</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>21</v>
@@ -2469,94 +2442,94 @@
         <v>66</v>
       </c>
       <c r="E48" s="3">
-        <v>1.2030000000000001</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="F48" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G48" s="3">
-        <v>0.96240000000000003</v>
+        <v>0.01</v>
       </c>
       <c r="H48" s="3">
-        <v>1.2030000000000001</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="I48" s="3">
-        <v>1.4436</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="J48" s="3"/>
       <c r="K48" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" s="3" t="s">
-        <v>140</v>
+        <v>117</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C49" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E49" s="3">
-        <v>0.04</v>
+        <v>3.4000000000000002E-2</v>
       </c>
       <c r="F49" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G49" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>2.7199999999999998E-2</v>
       </c>
       <c r="H49" s="3">
-        <v>0.04</v>
+        <v>3.4000000000000002E-2</v>
       </c>
       <c r="I49" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>4.0800000000000003E-2</v>
       </c>
       <c r="J49" s="3"/>
       <c r="K49" s="3" t="s">
-        <v>77</v>
+        <v>99</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" s="3" t="s">
-        <v>141</v>
+        <v>118</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E50" s="3">
-        <v>0.12</v>
+        <v>5.7000000000000002E-2</v>
       </c>
       <c r="F50" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G50" s="3">
-        <v>9.6000000000000002E-2</v>
+        <v>4.5600000000000002E-2</v>
       </c>
       <c r="H50" s="3">
-        <v>0.12</v>
+        <v>5.7000000000000002E-2</v>
       </c>
       <c r="I50" s="3">
-        <v>0.14399999999999999</v>
+        <v>6.8400000000000002E-2</v>
       </c>
       <c r="J50" s="3"/>
       <c r="K50" s="3" t="s">
-        <v>78</v>
+        <v>100</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>154</v>
@@ -2568,28 +2541,28 @@
         <v>66</v>
       </c>
       <c r="E51" s="3">
-        <v>0.04</v>
+        <v>1.2030000000000001</v>
       </c>
       <c r="F51" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G51" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>0.96240000000000003</v>
       </c>
       <c r="H51" s="3">
-        <v>0.04</v>
+        <v>1.2030000000000001</v>
       </c>
       <c r="I51" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>1.4436</v>
       </c>
       <c r="J51" s="3"/>
       <c r="K51" s="3" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" s="3" t="s">
-        <v>119</v>
+        <v>140</v>
       </c>
       <c r="B52" s="3" t="s">
         <v>154</v>
@@ -2598,34 +2571,34 @@
         <v>21</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E52" s="3">
-        <v>1.01E-2</v>
+        <v>0.04</v>
       </c>
       <c r="F52" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G52" s="3">
-        <v>8.0800000000000004E-3</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H52" s="3">
-        <v>1.01E-2</v>
+        <v>0.04</v>
       </c>
       <c r="I52" s="3">
-        <v>1.21199999999999E-2</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J52" s="3"/>
       <c r="K52" s="3" t="s">
-        <v>101</v>
+        <v>77</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C53" s="3" t="s">
         <v>21</v>
@@ -2634,31 +2607,31 @@
         <v>66</v>
       </c>
       <c r="E53" s="3">
-        <v>0.58899999999999997</v>
+        <v>0.12</v>
       </c>
       <c r="F53" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G53" s="3">
-        <v>0.47120000000000001</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="H53" s="3">
-        <v>0.58899999999999997</v>
+        <v>0.12</v>
       </c>
       <c r="I53" s="3">
-        <v>0.70679999999999998</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="J53" s="3"/>
       <c r="K53" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C54" s="3" t="s">
         <v>21</v>
@@ -2667,31 +2640,31 @@
         <v>66</v>
       </c>
       <c r="E54" s="3">
-        <v>8.0000000000000002E-3</v>
+        <v>0.04</v>
       </c>
       <c r="F54" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G54" s="3">
-        <v>6.4000000000000003E-3</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H54" s="3">
-        <v>8.0000000000000002E-3</v>
+        <v>0.04</v>
       </c>
       <c r="I54" s="3">
-        <v>9.5999999999999992E-3</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J54" s="3"/>
       <c r="K54" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C55" s="3" t="s">
         <v>21</v>
@@ -2699,32 +2672,32 @@
       <c r="D55" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="E55" s="5">
-        <v>9.9999999999999995E-7</v>
+      <c r="E55" s="3">
+        <v>1.01E-2</v>
       </c>
       <c r="F55" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G55" s="5">
-        <v>7.9999999999999996E-7</v>
-      </c>
-      <c r="H55" s="5">
-        <v>9.9999999999999995E-7</v>
-      </c>
-      <c r="I55" s="5">
-        <v>1.1999999999999999E-6</v>
+      <c r="G55" s="3">
+        <v>8.0800000000000004E-3</v>
+      </c>
+      <c r="H55" s="3">
+        <v>1.01E-2</v>
+      </c>
+      <c r="I55" s="3">
+        <v>1.21199999999999E-2</v>
       </c>
       <c r="J55" s="3"/>
       <c r="K55" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C56" s="3" t="s">
         <v>21</v>
@@ -2733,28 +2706,28 @@
         <v>66</v>
       </c>
       <c r="E56" s="3">
-        <v>7.51E-2</v>
+        <v>0.58899999999999997</v>
       </c>
       <c r="F56" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G56" s="3">
-        <v>6.0080000000000001E-2</v>
+        <v>0.47120000000000001</v>
       </c>
       <c r="H56" s="3">
-        <v>7.51E-2</v>
+        <v>0.58899999999999997</v>
       </c>
       <c r="I56" s="3">
-        <v>9.0119999999999895E-2</v>
+        <v>0.70679999999999998</v>
       </c>
       <c r="J56" s="3"/>
       <c r="K56" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" s="3" t="s">
-        <v>121</v>
+        <v>144</v>
       </c>
       <c r="B57" s="3" t="s">
         <v>156</v>
@@ -2763,31 +2736,31 @@
         <v>21</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E57" s="3">
-        <v>13</v>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="F57" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G57" s="3">
-        <v>10.4</v>
+        <v>6.4000000000000003E-3</v>
       </c>
       <c r="H57" s="3">
-        <v>13</v>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="I57" s="3">
-        <v>15.6</v>
+        <v>9.5999999999999992E-3</v>
       </c>
       <c r="J57" s="3"/>
       <c r="K57" s="3" t="s">
-        <v>103</v>
+        <v>81</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B58" s="3" t="s">
         <v>156</v>
@@ -2798,29 +2771,29 @@
       <c r="D58" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="E58" s="3">
-        <v>25</v>
+      <c r="E58" s="5">
+        <v>9.9999999999999995E-7</v>
       </c>
       <c r="F58" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G58" s="3">
-        <v>20</v>
-      </c>
-      <c r="H58" s="3">
-        <v>25</v>
-      </c>
-      <c r="I58" s="3">
-        <v>30</v>
+      <c r="G58" s="5">
+        <v>7.9999999999999996E-7</v>
+      </c>
+      <c r="H58" s="5">
+        <v>9.9999999999999995E-7</v>
+      </c>
+      <c r="I58" s="5">
+        <v>1.1999999999999999E-6</v>
       </c>
       <c r="J58" s="3"/>
       <c r="K58" s="3" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B59" s="3" t="s">
         <v>156</v>
@@ -2832,88 +2805,187 @@
         <v>66</v>
       </c>
       <c r="E59" s="3">
-        <v>3.9899999999999996E-3</v>
+        <v>7.51E-2</v>
       </c>
       <c r="F59" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G59" s="3">
-        <v>3.192E-3</v>
+        <v>6.0080000000000001E-2</v>
       </c>
       <c r="H59" s="3">
-        <v>3.9899999999999996E-3</v>
+        <v>7.51E-2</v>
       </c>
       <c r="I59" s="3">
-        <v>4.7879999999999997E-3</v>
+        <v>9.0119999999999895E-2</v>
       </c>
       <c r="J59" s="3"/>
       <c r="K59" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" s="3" t="s">
-        <v>147</v>
+        <v>121</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C60" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E60" s="3">
-        <v>0.06</v>
+        <v>13</v>
       </c>
       <c r="F60" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G60" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>10.4</v>
       </c>
       <c r="H60" s="3">
-        <v>0.06</v>
+        <v>13</v>
       </c>
       <c r="I60" s="3">
-        <v>7.1999999999999995E-2</v>
+        <v>15.6</v>
       </c>
       <c r="J60" s="3"/>
       <c r="K60" s="3" t="s">
-        <v>84</v>
+        <v>103</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
-        <v>148</v>
+        <v>122</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C61" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E61" s="3">
-        <v>0.02</v>
+        <v>25</v>
       </c>
       <c r="F61" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G61" s="3">
-        <v>1.6E-2</v>
+        <v>20</v>
       </c>
       <c r="H61" s="3">
-        <v>0.02</v>
+        <v>25</v>
       </c>
       <c r="I61" s="3">
-        <v>2.4E-2</v>
+        <v>30</v>
       </c>
       <c r="J61" s="3"/>
       <c r="K61" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A62" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E62" s="3">
+        <v>3.9899999999999996E-3</v>
+      </c>
+      <c r="F62" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="G62" s="3">
+        <v>3.192E-3</v>
+      </c>
+      <c r="H62" s="3">
+        <v>3.9899999999999996E-3</v>
+      </c>
+      <c r="I62" s="3">
+        <v>4.7879999999999997E-3</v>
+      </c>
+      <c r="J62" s="3"/>
+      <c r="K62" s="3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A63" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E63" s="3">
+        <v>0.06</v>
+      </c>
+      <c r="F63" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="G63" s="3">
+        <v>4.8000000000000001E-2</v>
+      </c>
+      <c r="H63" s="3">
+        <v>0.06</v>
+      </c>
+      <c r="I63" s="3">
+        <v>7.1999999999999995E-2</v>
+      </c>
+      <c r="J63" s="3"/>
+      <c r="K63" s="3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A64" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E64" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="F64" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="G64" s="3">
+        <v>1.6E-2</v>
+      </c>
+      <c r="H64" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="I64" s="3">
+        <v>2.4E-2</v>
+      </c>
+      <c r="J64" s="3"/>
+      <c r="K64" s="3" t="s">
         <v>85</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add more uncertain params; other minor updates
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saran\Documents\Academia\repository_clones\Bioindustrial-Park\biorefineries\isobutanol\analyses\full\parameter_distributions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73F6C879-74A0-4369-BA32-FCA612BBAF30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57AE8EAF-8F0A-4FAC-A3CD-46F8DBE33160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="166">
   <si>
     <t>Parameter name</t>
   </si>
@@ -525,6 +525,15 @@
   </si>
   <si>
     <t>Isopentyl acetate price</t>
+  </si>
+  <si>
+    <t>V514.isobutanol_price = x</t>
+  </si>
+  <si>
+    <t>DDGS.price =x</t>
+  </si>
+  <si>
+    <t>makeup_isopentyl_acetate.price = x</t>
   </si>
 </sst>
 </file>
@@ -1088,12 +1097,12 @@
         <v>18</v>
       </c>
       <c r="G6" s="4">
-        <f t="shared" ref="G6:G11" si="0">E6*0.8</f>
+        <f t="shared" ref="G6:G14" si="0">E6*0.8</f>
         <v>0.35920000000000002</v>
       </c>
       <c r="H6" s="4"/>
       <c r="I6" s="4">
-        <f t="shared" ref="I6:I11" si="1">1.2*E6</f>
+        <f t="shared" ref="I6:I14" si="1">1.2*E6</f>
         <v>0.53879999999999995</v>
       </c>
       <c r="J6" s="4"/>
@@ -1279,13 +1288,25 @@
       <c r="D12" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
+      <c r="E12" s="4">
+        <v>0.12</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G12" s="4">
+        <f t="shared" si="0"/>
+        <v>9.6000000000000002E-2</v>
+      </c>
       <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
+      <c r="I12" s="4">
+        <f t="shared" si="1"/>
+        <v>0.14399999999999999</v>
+      </c>
       <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
+      <c r="K12" s="4" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
@@ -1300,13 +1321,25 @@
       <c r="D13" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
+      <c r="E13" s="4">
+        <v>1.43</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G13" s="4">
+        <f t="shared" si="0"/>
+        <v>1.1439999999999999</v>
+      </c>
       <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
+      <c r="I13" s="4">
+        <f t="shared" si="1"/>
+        <v>1.716</v>
+      </c>
       <c r="J13" s="4"/>
-      <c r="K13" s="4"/>
+      <c r="K13" s="4" t="s">
+        <v>163</v>
+      </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
@@ -1321,13 +1354,25 @@
       <c r="D14" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
+      <c r="E14" s="4">
+        <v>3.2</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" s="4">
+        <f t="shared" si="0"/>
+        <v>2.5600000000000005</v>
+      </c>
       <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
+      <c r="I14" s="4">
+        <f t="shared" si="1"/>
+        <v>3.84</v>
+      </c>
       <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
+      <c r="K14" s="4" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">

</xml_diff>

<commit_message>
add feedstock comp to uncertainty; add new metrics; update opt_feed_strategy
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saran\Documents\Academia\repository_clones\Bioindustrial-Park\biorefineries\isobutanol\analyses\full\parameter_distributions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9813AE1-7256-4BD2-93B6-008AD071876A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCE5CA20-560A-4500-9C5E-34F66AF315C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="169">
   <si>
     <t>Parameter name</t>
   </si>
@@ -534,6 +534,15 @@
   </si>
   <si>
     <t>makeup_isopentyl_acetate.price = x</t>
+  </si>
+  <si>
+    <t>Feedstock starch content</t>
+  </si>
+  <si>
+    <t>kg/kg-water</t>
+  </si>
+  <si>
+    <t>feedstock.imass['Starch'] =x * feedstock.imass['Water']</t>
   </si>
 </sst>
 </file>
@@ -896,7 +905,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K64"/>
+  <dimension ref="A1:K65"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="40.81640625" customWidth="1"/>
@@ -1509,7 +1518,7 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>38</v>
+        <v>166</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>39</v>
@@ -1518,70 +1527,70 @@
         <v>21</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>40</v>
+        <v>167</v>
       </c>
       <c r="E19" s="3">
-        <v>56972</v>
+        <v>4.08</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>27</v>
       </c>
       <c r="G19" s="3">
         <f>0.8*H19</f>
-        <v>45577.600000000006</v>
+        <v>3.2640000000000002</v>
       </c>
       <c r="H19" s="3">
         <f>E19</f>
-        <v>56972</v>
+        <v>4.08</v>
       </c>
       <c r="I19" s="3">
         <f>1.2*H19</f>
-        <v>68366.399999999994</v>
+        <v>4.8959999999999999</v>
       </c>
       <c r="J19" s="3"/>
       <c r="K19" s="3" t="s">
-        <v>41</v>
+        <v>168</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="E20" s="3">
-        <v>156</v>
+        <v>56972</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>27</v>
       </c>
       <c r="G20" s="3">
-        <f>E20*0.8</f>
-        <v>124.80000000000001</v>
+        <f>0.8*H20</f>
+        <v>45577.600000000006</v>
       </c>
       <c r="H20" s="3">
         <f>E20</f>
-        <v>156</v>
+        <v>56972</v>
       </c>
       <c r="I20" s="3">
-        <f>E20*1.2</f>
-        <v>187.2</v>
+        <f>1.2*H20</f>
+        <v>68366.399999999994</v>
       </c>
       <c r="J20" s="3"/>
       <c r="K20" s="3" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>13</v>
@@ -1612,45 +1621,48 @@
       </c>
       <c r="J21" s="3"/>
       <c r="K21" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>123</v>
+        <v>54</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>149</v>
+        <v>13</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>66</v>
+        <v>14</v>
       </c>
       <c r="E22" s="3">
-        <v>1.43</v>
+        <v>156</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>67</v>
+        <v>27</v>
       </c>
       <c r="G22" s="3">
-        <v>1.1439999999999999</v>
+        <f>E22*0.8</f>
+        <v>124.80000000000001</v>
       </c>
       <c r="H22" s="3">
-        <v>1.43</v>
+        <f>E22</f>
+        <v>156</v>
       </c>
       <c r="I22" s="3">
-        <v>1.716</v>
+        <f>E22*1.2</f>
+        <v>187.2</v>
       </c>
       <c r="J22" s="3"/>
       <c r="K22" s="3" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>106</v>
+        <v>123</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>149</v>
@@ -1659,31 +1671,31 @@
         <v>21</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E23" s="3">
-        <v>0.94</v>
+        <v>1.43</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G23" s="3">
-        <v>0.752</v>
+        <v>1.1439999999999999</v>
       </c>
       <c r="H23" s="3">
-        <v>0.94</v>
+        <v>1.43</v>
       </c>
       <c r="I23" s="3">
-        <v>1.1279999999999999</v>
+        <v>1.716</v>
       </c>
       <c r="J23" s="3"/>
       <c r="K23" s="3" t="s">
-        <v>88</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>149</v>
@@ -1692,31 +1704,31 @@
         <v>21</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E24" s="3">
-        <v>0.58399999999999996</v>
+        <v>0.94</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G24" s="3">
-        <v>0.4672</v>
+        <v>0.752</v>
       </c>
       <c r="H24" s="3">
-        <v>0.58399999999999996</v>
+        <v>0.94</v>
       </c>
       <c r="I24" s="3">
-        <v>0.70079999999999998</v>
+        <v>1.1279999999999999</v>
       </c>
       <c r="J24" s="3"/>
       <c r="K24" s="3" t="s">
-        <v>59</v>
+        <v>88</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>149</v>
@@ -1725,31 +1737,31 @@
         <v>21</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E25" s="3">
-        <v>1.1599999999999999E-2</v>
+        <v>0.58399999999999996</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G25" s="3">
-        <v>9.2800000000000001E-3</v>
+        <v>0.4672</v>
       </c>
       <c r="H25" s="3">
-        <v>1.1599999999999999E-2</v>
+        <v>0.58399999999999996</v>
       </c>
       <c r="I25" s="3">
-        <v>1.3919999999999899E-2</v>
+        <v>0.70079999999999998</v>
       </c>
       <c r="J25" s="3"/>
       <c r="K25" s="3" t="s">
-        <v>89</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
-        <v>125</v>
+        <v>107</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>149</v>
@@ -1758,31 +1770,31 @@
         <v>21</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E26" s="3">
-        <v>47.1</v>
+        <v>1.1599999999999999E-2</v>
       </c>
       <c r="F26" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G26" s="3">
-        <v>37.68</v>
+        <v>9.2800000000000001E-3</v>
       </c>
       <c r="H26" s="3">
-        <v>47.1</v>
+        <v>1.1599999999999999E-2</v>
       </c>
       <c r="I26" s="3">
-        <v>56.52</v>
+        <v>1.3919999999999899E-2</v>
       </c>
       <c r="J26" s="3"/>
       <c r="K26" s="3" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>108</v>
+        <v>125</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>149</v>
@@ -1791,31 +1803,31 @@
         <v>21</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E27" s="3">
-        <v>14.2</v>
+        <v>47.1</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G27" s="3">
-        <v>11.36</v>
+        <v>37.68</v>
       </c>
       <c r="H27" s="3">
-        <v>14.2</v>
+        <v>47.1</v>
       </c>
       <c r="I27" s="3">
-        <v>17.04</v>
+        <v>56.52</v>
       </c>
       <c r="J27" s="3"/>
       <c r="K27" s="3" t="s">
-        <v>90</v>
+        <v>58</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>149</v>
@@ -1827,28 +1839,28 @@
         <v>68</v>
       </c>
       <c r="E28" s="3">
-        <v>0.12</v>
+        <v>14.2</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G28" s="3">
-        <v>9.6000000000000002E-2</v>
+        <v>11.36</v>
       </c>
       <c r="H28" s="3">
-        <v>0.12</v>
+        <v>14.2</v>
       </c>
       <c r="I28" s="3">
-        <v>0.14399999999999999</v>
+        <v>17.04</v>
       </c>
       <c r="J28" s="3"/>
       <c r="K28" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>126</v>
+        <v>109</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>149</v>
@@ -1857,31 +1869,31 @@
         <v>21</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E29" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G29" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="H29" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="I29" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="J29" s="3"/>
       <c r="K29" s="3" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>149</v>
@@ -1893,28 +1905,28 @@
         <v>66</v>
       </c>
       <c r="E30" s="3">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G30" s="3">
-        <v>9.6000000000000002E-2</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H30" s="3">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="I30" s="3">
-        <v>0.14399999999999999</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J30" s="3"/>
       <c r="K30" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>149</v>
@@ -1926,31 +1938,31 @@
         <v>66</v>
       </c>
       <c r="E31" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G31" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="H31" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="I31" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="J31" s="3"/>
       <c r="K31" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>21</v>
@@ -1959,28 +1971,28 @@
         <v>66</v>
       </c>
       <c r="E32" s="3">
-        <v>0.501</v>
+        <v>0.04</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G32" s="3">
-        <v>0.40079999999999999</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H32" s="3">
-        <v>0.501</v>
+        <v>0.04</v>
       </c>
       <c r="I32" s="3">
-        <v>0.60119999999999996</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J32" s="3"/>
       <c r="K32" s="3" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
-        <v>110</v>
+        <v>129</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>150</v>
@@ -1989,31 +2001,31 @@
         <v>21</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E33" s="5">
-        <v>2.0000000000000002E-5</v>
+        <v>66</v>
+      </c>
+      <c r="E33" s="3">
+        <v>0.501</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G33" s="5">
-        <v>1.5999999999999999E-5</v>
-      </c>
-      <c r="H33" s="5">
-        <v>2.0000000000000002E-5</v>
-      </c>
-      <c r="I33" s="5">
-        <v>2.4000000000000001E-5</v>
+      <c r="G33" s="3">
+        <v>0.40079999999999999</v>
+      </c>
+      <c r="H33" s="3">
+        <v>0.501</v>
+      </c>
+      <c r="I33" s="3">
+        <v>0.60119999999999996</v>
       </c>
       <c r="J33" s="3"/>
       <c r="K33" s="3" t="s">
-        <v>92</v>
+        <v>57</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>150</v>
@@ -2024,62 +2036,62 @@
       <c r="D34" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="E34" s="3">
-        <v>0.10100000000000001</v>
+      <c r="E34" s="5">
+        <v>2.0000000000000002E-5</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G34" s="3">
-        <v>8.0799999999999997E-2</v>
-      </c>
-      <c r="H34" s="3">
-        <v>0.10100000000000001</v>
-      </c>
-      <c r="I34" s="3">
-        <v>0.1212</v>
+      <c r="G34" s="5">
+        <v>1.5999999999999999E-5</v>
+      </c>
+      <c r="H34" s="5">
+        <v>2.0000000000000002E-5</v>
+      </c>
+      <c r="I34" s="5">
+        <v>2.4000000000000001E-5</v>
       </c>
       <c r="J34" s="3"/>
       <c r="K34" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
-        <v>130</v>
+        <v>111</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E35" s="3">
-        <v>5.81</v>
+        <v>0.10100000000000001</v>
       </c>
       <c r="F35" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G35" s="3">
-        <v>4.6479999999999997</v>
+        <v>8.0799999999999997E-2</v>
       </c>
       <c r="H35" s="3">
-        <v>5.81</v>
+        <v>0.10100000000000001</v>
       </c>
       <c r="I35" s="3">
-        <v>6.9719999999999898</v>
+        <v>0.1212</v>
       </c>
       <c r="J35" s="3"/>
       <c r="K35" s="3" t="s">
-        <v>64</v>
+        <v>93</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
-        <v>112</v>
+        <v>130</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>151</v>
@@ -2088,64 +2100,64 @@
         <v>21</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E36" s="5">
-        <v>4.9999999999999998E-7</v>
+        <v>66</v>
+      </c>
+      <c r="E36" s="3">
+        <v>5.81</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G36" s="5">
-        <v>3.9999999999999998E-7</v>
-      </c>
-      <c r="H36" s="5">
-        <v>4.9999999999999998E-7</v>
-      </c>
-      <c r="I36" s="5">
-        <v>5.9999999999999997E-7</v>
+      <c r="G36" s="3">
+        <v>4.6479999999999997</v>
+      </c>
+      <c r="H36" s="3">
+        <v>5.81</v>
+      </c>
+      <c r="I36" s="3">
+        <v>6.9719999999999898</v>
       </c>
       <c r="J36" s="3"/>
       <c r="K36" s="3" t="s">
-        <v>94</v>
+        <v>64</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
-        <v>131</v>
+        <v>112</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="E37" s="3">
-        <v>4.8</v>
+        <v>68</v>
+      </c>
+      <c r="E37" s="5">
+        <v>4.9999999999999998E-7</v>
       </c>
       <c r="F37" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G37" s="3">
-        <v>3.84</v>
-      </c>
-      <c r="H37" s="3">
-        <v>4.8</v>
-      </c>
-      <c r="I37" s="3">
-        <v>5.76</v>
+      <c r="G37" s="5">
+        <v>3.9999999999999998E-7</v>
+      </c>
+      <c r="H37" s="5">
+        <v>4.9999999999999998E-7</v>
+      </c>
+      <c r="I37" s="5">
+        <v>5.9999999999999997E-7</v>
       </c>
       <c r="J37" s="3"/>
       <c r="K37" s="3" t="s">
-        <v>65</v>
+        <v>94</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>152</v>
@@ -2157,28 +2169,28 @@
         <v>66</v>
       </c>
       <c r="E38" s="3">
-        <v>0.04</v>
+        <v>4.8</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G38" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>3.84</v>
       </c>
       <c r="H38" s="3">
-        <v>0.04</v>
+        <v>4.8</v>
       </c>
       <c r="I38" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>5.76</v>
       </c>
       <c r="J38" s="3"/>
       <c r="K38" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>152</v>
@@ -2190,28 +2202,28 @@
         <v>66</v>
       </c>
       <c r="E39" s="3">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="F39" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G39" s="3">
-        <v>9.6000000000000002E-2</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H39" s="3">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="I39" s="3">
-        <v>0.14399999999999999</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J39" s="3"/>
       <c r="K39" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>152</v>
@@ -2223,28 +2235,28 @@
         <v>66</v>
       </c>
       <c r="E40" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="F40" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G40" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="H40" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="I40" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="J40" s="3"/>
       <c r="K40" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
-        <v>113</v>
+        <v>134</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>152</v>
@@ -2253,64 +2265,64 @@
         <v>21</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E41" s="3">
-        <v>2.6400000000000002E-4</v>
+        <v>0.04</v>
       </c>
       <c r="F41" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G41" s="3">
-        <v>2.1120000000000001E-4</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H41" s="3">
-        <v>2.6400000000000002E-4</v>
+        <v>0.04</v>
       </c>
       <c r="I41" s="3">
-        <v>3.168E-4</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J41" s="3"/>
       <c r="K41" s="3" t="s">
-        <v>95</v>
+        <v>71</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
-        <v>135</v>
+        <v>113</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E42" s="3">
-        <v>1.04E-2</v>
+        <v>2.6400000000000002E-4</v>
       </c>
       <c r="F42" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G42" s="3">
-        <v>8.3199999999999993E-3</v>
+        <v>2.1120000000000001E-4</v>
       </c>
       <c r="H42" s="3">
-        <v>1.04E-2</v>
+        <v>2.6400000000000002E-4</v>
       </c>
       <c r="I42" s="3">
-        <v>1.248E-2</v>
+        <v>3.168E-4</v>
       </c>
       <c r="J42" s="3"/>
       <c r="K42" s="3" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>157</v>
@@ -2319,31 +2331,31 @@
         <v>21</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E43" s="3">
-        <v>1.0200000000000001E-2</v>
+        <v>1.04E-2</v>
       </c>
       <c r="F43" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G43" s="3">
-        <v>8.1600000000000006E-3</v>
+        <v>8.3199999999999993E-3</v>
       </c>
       <c r="H43" s="3">
-        <v>1.0200000000000001E-2</v>
+        <v>1.04E-2</v>
       </c>
       <c r="I43" s="3">
-        <v>1.2239999999999999E-2</v>
+        <v>1.248E-2</v>
       </c>
       <c r="J43" s="3"/>
       <c r="K43" s="3" t="s">
-        <v>96</v>
+        <v>72</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
-        <v>136</v>
+        <v>114</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>157</v>
@@ -2352,31 +2364,31 @@
         <v>21</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E44" s="3">
-        <v>0.77500000000000002</v>
+        <v>1.0200000000000001E-2</v>
       </c>
       <c r="F44" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G44" s="3">
-        <v>0.62</v>
+        <v>8.1600000000000006E-3</v>
       </c>
       <c r="H44" s="3">
-        <v>0.77500000000000002</v>
+        <v>1.0200000000000001E-2</v>
       </c>
       <c r="I44" s="3">
-        <v>0.92999999999999905</v>
+        <v>1.2239999999999999E-2</v>
       </c>
       <c r="J44" s="3"/>
       <c r="K44" s="3" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" s="3" t="s">
-        <v>115</v>
+        <v>136</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>157</v>
@@ -2385,31 +2397,31 @@
         <v>21</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E45" s="3">
-        <v>0.1</v>
+        <v>0.77500000000000002</v>
       </c>
       <c r="F45" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G45" s="3">
-        <v>0.08</v>
+        <v>0.62</v>
       </c>
       <c r="H45" s="3">
-        <v>0.1</v>
+        <v>0.77500000000000002</v>
       </c>
       <c r="I45" s="3">
-        <v>0.12</v>
+        <v>0.92999999999999905</v>
       </c>
       <c r="J45" s="3"/>
       <c r="K45" s="3" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>157</v>
@@ -2421,61 +2433,61 @@
         <v>68</v>
       </c>
       <c r="E46" s="3">
-        <v>440</v>
+        <v>0.1</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G46" s="3">
-        <v>352</v>
+        <v>0.08</v>
       </c>
       <c r="H46" s="3">
-        <v>440</v>
+        <v>0.1</v>
       </c>
       <c r="I46" s="3">
-        <v>528</v>
+        <v>0.12</v>
       </c>
       <c r="J46" s="3"/>
       <c r="K46" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" s="3" t="s">
-        <v>137</v>
+        <v>116</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E47" s="3">
-        <v>2.82</v>
+        <v>440</v>
       </c>
       <c r="F47" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G47" s="3">
-        <v>2.2559999999999998</v>
+        <v>352</v>
       </c>
       <c r="H47" s="3">
-        <v>2.82</v>
+        <v>440</v>
       </c>
       <c r="I47" s="3">
-        <v>3.3839999999999999</v>
+        <v>528</v>
       </c>
       <c r="J47" s="3"/>
       <c r="K47" s="3" t="s">
-        <v>74</v>
+        <v>98</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B48" s="3" t="s">
         <v>153</v>
@@ -2487,28 +2499,28 @@
         <v>66</v>
       </c>
       <c r="E48" s="3">
-        <v>1.2500000000000001E-2</v>
+        <v>2.82</v>
       </c>
       <c r="F48" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G48" s="3">
-        <v>0.01</v>
+        <v>2.2559999999999998</v>
       </c>
       <c r="H48" s="3">
-        <v>1.2500000000000001E-2</v>
+        <v>2.82</v>
       </c>
       <c r="I48" s="3">
-        <v>1.4999999999999999E-2</v>
+        <v>3.3839999999999999</v>
       </c>
       <c r="J48" s="3"/>
       <c r="K48" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" s="3" t="s">
-        <v>117</v>
+        <v>138</v>
       </c>
       <c r="B49" s="3" t="s">
         <v>153</v>
@@ -2517,31 +2529,31 @@
         <v>21</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E49" s="3">
-        <v>3.4000000000000002E-2</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="F49" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G49" s="3">
-        <v>2.7199999999999998E-2</v>
+        <v>0.01</v>
       </c>
       <c r="H49" s="3">
-        <v>3.4000000000000002E-2</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="I49" s="3">
-        <v>4.0800000000000003E-2</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="J49" s="3"/>
       <c r="K49" s="3" t="s">
-        <v>99</v>
+        <v>75</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>153</v>
@@ -2553,61 +2565,61 @@
         <v>68</v>
       </c>
       <c r="E50" s="3">
-        <v>5.7000000000000002E-2</v>
+        <v>3.4000000000000002E-2</v>
       </c>
       <c r="F50" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G50" s="3">
-        <v>4.5600000000000002E-2</v>
+        <v>2.7199999999999998E-2</v>
       </c>
       <c r="H50" s="3">
-        <v>5.7000000000000002E-2</v>
+        <v>3.4000000000000002E-2</v>
       </c>
       <c r="I50" s="3">
-        <v>6.8400000000000002E-2</v>
+        <v>4.0800000000000003E-2</v>
       </c>
       <c r="J50" s="3"/>
       <c r="K50" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
-        <v>139</v>
+        <v>118</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E51" s="3">
-        <v>1.2030000000000001</v>
+        <v>5.7000000000000002E-2</v>
       </c>
       <c r="F51" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G51" s="3">
-        <v>0.96240000000000003</v>
+        <v>4.5600000000000002E-2</v>
       </c>
       <c r="H51" s="3">
-        <v>1.2030000000000001</v>
+        <v>5.7000000000000002E-2</v>
       </c>
       <c r="I51" s="3">
-        <v>1.4436</v>
+        <v>6.8400000000000002E-2</v>
       </c>
       <c r="J51" s="3"/>
       <c r="K51" s="3" t="s">
-        <v>76</v>
+        <v>100</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B52" s="3" t="s">
         <v>154</v>
@@ -2619,28 +2631,28 @@
         <v>66</v>
       </c>
       <c r="E52" s="3">
-        <v>0.04</v>
+        <v>1.2030000000000001</v>
       </c>
       <c r="F52" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G52" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>0.96240000000000003</v>
       </c>
       <c r="H52" s="3">
-        <v>0.04</v>
+        <v>1.2030000000000001</v>
       </c>
       <c r="I52" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>1.4436</v>
       </c>
       <c r="J52" s="3"/>
       <c r="K52" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>154</v>
@@ -2652,28 +2664,28 @@
         <v>66</v>
       </c>
       <c r="E53" s="3">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="F53" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G53" s="3">
-        <v>9.6000000000000002E-2</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H53" s="3">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="I53" s="3">
-        <v>0.14399999999999999</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J53" s="3"/>
       <c r="K53" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B54" s="3" t="s">
         <v>154</v>
@@ -2685,28 +2697,28 @@
         <v>66</v>
       </c>
       <c r="E54" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="F54" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G54" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="H54" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="I54" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="J54" s="3"/>
       <c r="K54" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" s="3" t="s">
-        <v>119</v>
+        <v>142</v>
       </c>
       <c r="B55" s="3" t="s">
         <v>154</v>
@@ -2715,67 +2727,67 @@
         <v>21</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E55" s="3">
-        <v>1.01E-2</v>
+        <v>0.04</v>
       </c>
       <c r="F55" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G55" s="3">
-        <v>8.0800000000000004E-3</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H55" s="3">
-        <v>1.01E-2</v>
+        <v>0.04</v>
       </c>
       <c r="I55" s="3">
-        <v>1.21199999999999E-2</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J55" s="3"/>
       <c r="K55" s="3" t="s">
-        <v>101</v>
+        <v>79</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
-        <v>143</v>
+        <v>119</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C56" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E56" s="3">
-        <v>0.58899999999999997</v>
+        <v>1.01E-2</v>
       </c>
       <c r="F56" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G56" s="3">
-        <v>0.47120000000000001</v>
+        <v>8.0800000000000004E-3</v>
       </c>
       <c r="H56" s="3">
-        <v>0.58899999999999997</v>
+        <v>1.01E-2</v>
       </c>
       <c r="I56" s="3">
-        <v>0.70679999999999998</v>
+        <v>1.21199999999999E-2</v>
       </c>
       <c r="J56" s="3"/>
       <c r="K56" s="3" t="s">
-        <v>80</v>
+        <v>101</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C57" s="3" t="s">
         <v>21</v>
@@ -2784,28 +2796,28 @@
         <v>66</v>
       </c>
       <c r="E57" s="3">
-        <v>8.0000000000000002E-3</v>
+        <v>0.58899999999999997</v>
       </c>
       <c r="F57" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G57" s="3">
-        <v>6.4000000000000003E-3</v>
+        <v>0.47120000000000001</v>
       </c>
       <c r="H57" s="3">
-        <v>8.0000000000000002E-3</v>
+        <v>0.58899999999999997</v>
       </c>
       <c r="I57" s="3">
-        <v>9.5999999999999992E-3</v>
+        <v>0.70679999999999998</v>
       </c>
       <c r="J57" s="3"/>
       <c r="K57" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
-        <v>120</v>
+        <v>144</v>
       </c>
       <c r="B58" s="3" t="s">
         <v>156</v>
@@ -2814,31 +2826,31 @@
         <v>21</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E58" s="5">
-        <v>9.9999999999999995E-7</v>
+        <v>66</v>
+      </c>
+      <c r="E58" s="3">
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="F58" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G58" s="5">
-        <v>7.9999999999999996E-7</v>
-      </c>
-      <c r="H58" s="5">
-        <v>9.9999999999999995E-7</v>
-      </c>
-      <c r="I58" s="5">
-        <v>1.1999999999999999E-6</v>
+      <c r="G58" s="3">
+        <v>6.4000000000000003E-3</v>
+      </c>
+      <c r="H58" s="3">
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="I58" s="3">
+        <v>9.5999999999999992E-3</v>
       </c>
       <c r="J58" s="3"/>
       <c r="K58" s="3" t="s">
-        <v>102</v>
+        <v>81</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" s="3" t="s">
-        <v>145</v>
+        <v>120</v>
       </c>
       <c r="B59" s="3" t="s">
         <v>156</v>
@@ -2847,31 +2859,31 @@
         <v>21</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="E59" s="3">
-        <v>7.51E-2</v>
+        <v>68</v>
+      </c>
+      <c r="E59" s="5">
+        <v>9.9999999999999995E-7</v>
       </c>
       <c r="F59" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G59" s="3">
-        <v>6.0080000000000001E-2</v>
-      </c>
-      <c r="H59" s="3">
-        <v>7.51E-2</v>
-      </c>
-      <c r="I59" s="3">
-        <v>9.0119999999999895E-2</v>
+      <c r="G59" s="5">
+        <v>7.9999999999999996E-7</v>
+      </c>
+      <c r="H59" s="5">
+        <v>9.9999999999999995E-7</v>
+      </c>
+      <c r="I59" s="5">
+        <v>1.1999999999999999E-6</v>
       </c>
       <c r="J59" s="3"/>
       <c r="K59" s="3" t="s">
-        <v>82</v>
+        <v>102</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" s="3" t="s">
-        <v>121</v>
+        <v>145</v>
       </c>
       <c r="B60" s="3" t="s">
         <v>156</v>
@@ -2880,31 +2892,31 @@
         <v>21</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E60" s="3">
-        <v>13</v>
+        <v>7.51E-2</v>
       </c>
       <c r="F60" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G60" s="3">
-        <v>10.4</v>
+        <v>6.0080000000000001E-2</v>
       </c>
       <c r="H60" s="3">
-        <v>13</v>
+        <v>7.51E-2</v>
       </c>
       <c r="I60" s="3">
-        <v>15.6</v>
+        <v>9.0119999999999895E-2</v>
       </c>
       <c r="J60" s="3"/>
       <c r="K60" s="3" t="s">
-        <v>103</v>
+        <v>82</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B61" s="3" t="s">
         <v>156</v>
@@ -2916,28 +2928,28 @@
         <v>68</v>
       </c>
       <c r="E61" s="3">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="F61" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G61" s="3">
-        <v>20</v>
+        <v>10.4</v>
       </c>
       <c r="H61" s="3">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="I61" s="3">
-        <v>30</v>
+        <v>15.6</v>
       </c>
       <c r="J61" s="3"/>
       <c r="K61" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" s="3" t="s">
-        <v>146</v>
+        <v>122</v>
       </c>
       <c r="B62" s="3" t="s">
         <v>156</v>
@@ -2946,34 +2958,34 @@
         <v>21</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E62" s="3">
-        <v>3.9899999999999996E-3</v>
+        <v>25</v>
       </c>
       <c r="F62" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G62" s="3">
-        <v>3.192E-3</v>
+        <v>20</v>
       </c>
       <c r="H62" s="3">
-        <v>3.9899999999999996E-3</v>
+        <v>25</v>
       </c>
       <c r="I62" s="3">
-        <v>4.7879999999999997E-3</v>
+        <v>30</v>
       </c>
       <c r="J62" s="3"/>
       <c r="K62" s="3" t="s">
-        <v>83</v>
+        <v>104</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C63" s="3" t="s">
         <v>21</v>
@@ -2982,31 +2994,31 @@
         <v>66</v>
       </c>
       <c r="E63" s="3">
-        <v>0.06</v>
+        <v>3.9899999999999996E-3</v>
       </c>
       <c r="F63" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G63" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>3.192E-3</v>
       </c>
       <c r="H63" s="3">
-        <v>0.06</v>
+        <v>3.9899999999999996E-3</v>
       </c>
       <c r="I63" s="3">
-        <v>7.1999999999999995E-2</v>
+        <v>4.7879999999999997E-3</v>
       </c>
       <c r="J63" s="3"/>
       <c r="K63" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A64" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C64" s="3" t="s">
         <v>21</v>
@@ -3015,22 +3027,55 @@
         <v>66</v>
       </c>
       <c r="E64" s="3">
-        <v>0.02</v>
+        <v>0.06</v>
       </c>
       <c r="F64" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G64" s="3">
-        <v>1.6E-2</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="H64" s="3">
-        <v>0.02</v>
+        <v>0.06</v>
       </c>
       <c r="I64" s="3">
-        <v>2.4E-2</v>
+        <v>7.1999999999999995E-2</v>
       </c>
       <c r="J64" s="3"/>
       <c r="K64" s="3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A65" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E65" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="F65" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="G65" s="3">
+        <v>1.6E-2</v>
+      </c>
+      <c r="H65" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="I65" s="3">
+        <v>2.4E-2</v>
+      </c>
+      <c r="J65" s="3"/>
+      <c r="K65" s="3" t="s">
         <v>85</v>
       </c>
     </row>

</xml_diff>

<commit_message>
further major updates including analyses across more kinetic params
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saran\Documents\Academia\repository_clones\Bioindustrial-Park\biorefineries\isobutanol\analyses\full\parameter_distributions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCE5CA20-560A-4500-9C5E-34F66AF315C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4D4B085-6EFB-44DB-8945-CEFCDC6F4E4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -518,15 +518,6 @@
     <t>Kinetics: Acetaldehyde compartment degradation</t>
   </si>
   <si>
-    <t>DDGS price</t>
-  </si>
-  <si>
-    <t>Isobutanol price</t>
-  </si>
-  <si>
-    <t>Isopentyl acetate price</t>
-  </si>
-  <si>
     <t>V514.isobutanol_price = x</t>
   </si>
   <si>
@@ -543,6 +534,15 @@
   </si>
   <si>
     <t>feedstock.imass['Starch'] =x * feedstock.imass['Water']</t>
+  </si>
+  <si>
+    <t>Isobutanol unit price</t>
+  </si>
+  <si>
+    <t>DDGS unit price</t>
+  </si>
+  <si>
+    <t>Isopentyl acetate unit price</t>
   </si>
 </sst>
 </file>
@@ -1286,7 +1286,7 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>7</v>
@@ -1314,12 +1314,12 @@
       </c>
       <c r="J12" s="4"/>
       <c r="K12" s="4" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>7</v>
@@ -1331,28 +1331,28 @@
         <v>10</v>
       </c>
       <c r="E13" s="4">
-        <v>1.43</v>
+        <v>1.49</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>18</v>
       </c>
       <c r="G13" s="4">
         <f t="shared" si="0"/>
-        <v>1.1439999999999999</v>
+        <v>1.1919999999999999</v>
       </c>
       <c r="H13" s="4"/>
       <c r="I13" s="4">
         <f t="shared" si="1"/>
-        <v>1.716</v>
+        <v>1.788</v>
       </c>
       <c r="J13" s="4"/>
       <c r="K13" s="4" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>7</v>
@@ -1380,7 +1380,7 @@
       </c>
       <c r="J14" s="4"/>
       <c r="K14" s="4" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
@@ -1518,7 +1518,7 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>39</v>
@@ -1527,7 +1527,7 @@
         <v>21</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E19" s="3">
         <v>4.08</v>
@@ -1549,7 +1549,7 @@
       </c>
       <c r="J19" s="3"/>
       <c r="K19" s="3" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
minor updates; add code for pub plots
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saran\Documents\Academia\repository_clones\Bioindustrial-Park\biorefineries\isobutanol\analyses\full\parameter_distributions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4D4B085-6EFB-44DB-8945-CEFCDC6F4E4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02BBAFC5-450C-4E79-BFEB-ABB145034426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1337,13 +1337,11 @@
         <v>18</v>
       </c>
       <c r="G13" s="4">
-        <f t="shared" si="0"/>
-        <v>1.1919999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="H13" s="4"/>
       <c r="I13" s="4">
-        <f t="shared" si="1"/>
-        <v>1.788</v>
+        <v>1.7250000000000001</v>
       </c>
       <c r="J13" s="4"/>
       <c r="K13" s="4" t="s">

</xml_diff>

<commit_message>
add aeration rate safety factor to param dists for uncertainty analyses
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saran\Documents\Academia\repository_clones\Bioindustrial-Park\biorefineries\isobutanol\analyses\full\parameter_distributions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02BBAFC5-450C-4E79-BFEB-ABB145034426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EAC69E3-624C-4D8A-BDDC-ED485D55ABE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3380" yWindow="0" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="172">
   <si>
     <t>Parameter name</t>
   </si>
@@ -543,6 +543,15 @@
   </si>
   <si>
     <t>Isopentyl acetate unit price</t>
+  </si>
+  <si>
+    <t>Aeration rate safety factor</t>
+  </si>
+  <si>
+    <t>Fermentation</t>
+  </si>
+  <si>
+    <t>V406.aeration_safety_factor = x</t>
   </si>
 </sst>
 </file>
@@ -905,7 +914,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K65"/>
+  <dimension ref="A1:K66"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="40.81640625" customWidth="1"/>
@@ -1588,43 +1597,38 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>53</v>
+        <v>169</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>13</v>
+        <v>170</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E21" s="3">
-        <v>156</v>
+        <v>2</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="G21" s="3">
-        <f>E21*0.8</f>
-        <v>124.80000000000001</v>
-      </c>
-      <c r="H21" s="3">
-        <f>E21</f>
-        <v>156</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H21" s="3"/>
       <c r="I21" s="3">
-        <f>E21*1.2</f>
-        <v>187.2</v>
+        <v>3</v>
       </c>
       <c r="J21" s="3"/>
       <c r="K21" s="3" t="s">
-        <v>55</v>
+        <v>171</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>13</v>
@@ -1655,45 +1659,48 @@
       </c>
       <c r="J22" s="3"/>
       <c r="K22" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>123</v>
+        <v>54</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>149</v>
+        <v>13</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>66</v>
+        <v>14</v>
       </c>
       <c r="E23" s="3">
-        <v>1.43</v>
+        <v>156</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>67</v>
+        <v>27</v>
       </c>
       <c r="G23" s="3">
-        <v>1.1439999999999999</v>
+        <f>E23*0.8</f>
+        <v>124.80000000000001</v>
       </c>
       <c r="H23" s="3">
-        <v>1.43</v>
+        <f>E23</f>
+        <v>156</v>
       </c>
       <c r="I23" s="3">
-        <v>1.716</v>
+        <f>E23*1.2</f>
+        <v>187.2</v>
       </c>
       <c r="J23" s="3"/>
       <c r="K23" s="3" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>106</v>
+        <v>123</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>149</v>
@@ -1702,31 +1709,31 @@
         <v>21</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E24" s="3">
-        <v>0.94</v>
+        <v>1.43</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G24" s="3">
-        <v>0.752</v>
+        <v>1.1439999999999999</v>
       </c>
       <c r="H24" s="3">
-        <v>0.94</v>
+        <v>1.43</v>
       </c>
       <c r="I24" s="3">
-        <v>1.1279999999999999</v>
+        <v>1.716</v>
       </c>
       <c r="J24" s="3"/>
       <c r="K24" s="3" t="s">
-        <v>88</v>
+        <v>63</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>149</v>
@@ -1735,31 +1742,31 @@
         <v>21</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E25" s="3">
-        <v>0.58399999999999996</v>
+        <v>0.94</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G25" s="3">
-        <v>0.4672</v>
+        <v>0.752</v>
       </c>
       <c r="H25" s="3">
-        <v>0.58399999999999996</v>
+        <v>0.94</v>
       </c>
       <c r="I25" s="3">
-        <v>0.70079999999999998</v>
+        <v>1.1279999999999999</v>
       </c>
       <c r="J25" s="3"/>
       <c r="K25" s="3" t="s">
-        <v>59</v>
+        <v>88</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>149</v>
@@ -1768,31 +1775,31 @@
         <v>21</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E26" s="3">
-        <v>1.1599999999999999E-2</v>
+        <v>0.58399999999999996</v>
       </c>
       <c r="F26" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G26" s="3">
-        <v>9.2800000000000001E-3</v>
+        <v>0.4672</v>
       </c>
       <c r="H26" s="3">
-        <v>1.1599999999999999E-2</v>
+        <v>0.58399999999999996</v>
       </c>
       <c r="I26" s="3">
-        <v>1.3919999999999899E-2</v>
+        <v>0.70079999999999998</v>
       </c>
       <c r="J26" s="3"/>
       <c r="K26" s="3" t="s">
-        <v>89</v>
+        <v>59</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>125</v>
+        <v>107</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>149</v>
@@ -1801,31 +1808,31 @@
         <v>21</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E27" s="3">
-        <v>47.1</v>
+        <v>1.1599999999999999E-2</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G27" s="3">
-        <v>37.68</v>
+        <v>9.2800000000000001E-3</v>
       </c>
       <c r="H27" s="3">
-        <v>47.1</v>
+        <v>1.1599999999999999E-2</v>
       </c>
       <c r="I27" s="3">
-        <v>56.52</v>
+        <v>1.3919999999999899E-2</v>
       </c>
       <c r="J27" s="3"/>
       <c r="K27" s="3" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>108</v>
+        <v>125</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>149</v>
@@ -1834,31 +1841,31 @@
         <v>21</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E28" s="3">
-        <v>14.2</v>
+        <v>47.1</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G28" s="3">
-        <v>11.36</v>
+        <v>37.68</v>
       </c>
       <c r="H28" s="3">
-        <v>14.2</v>
+        <v>47.1</v>
       </c>
       <c r="I28" s="3">
-        <v>17.04</v>
+        <v>56.52</v>
       </c>
       <c r="J28" s="3"/>
       <c r="K28" s="3" t="s">
-        <v>90</v>
+        <v>58</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>149</v>
@@ -1870,28 +1877,28 @@
         <v>68</v>
       </c>
       <c r="E29" s="3">
-        <v>0.12</v>
+        <v>14.2</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G29" s="3">
-        <v>9.6000000000000002E-2</v>
+        <v>11.36</v>
       </c>
       <c r="H29" s="3">
-        <v>0.12</v>
+        <v>14.2</v>
       </c>
       <c r="I29" s="3">
-        <v>0.14399999999999999</v>
+        <v>17.04</v>
       </c>
       <c r="J29" s="3"/>
       <c r="K29" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>126</v>
+        <v>109</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>149</v>
@@ -1900,31 +1907,31 @@
         <v>21</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E30" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G30" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="H30" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="I30" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="J30" s="3"/>
       <c r="K30" s="3" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>149</v>
@@ -1936,28 +1943,28 @@
         <v>66</v>
       </c>
       <c r="E31" s="3">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G31" s="3">
-        <v>9.6000000000000002E-2</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H31" s="3">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="I31" s="3">
-        <v>0.14399999999999999</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J31" s="3"/>
       <c r="K31" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>149</v>
@@ -1969,31 +1976,31 @@
         <v>66</v>
       </c>
       <c r="E32" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G32" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="H32" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="I32" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="J32" s="3"/>
       <c r="K32" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>21</v>
@@ -2002,28 +2009,28 @@
         <v>66</v>
       </c>
       <c r="E33" s="3">
-        <v>0.501</v>
+        <v>0.04</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G33" s="3">
-        <v>0.40079999999999999</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H33" s="3">
-        <v>0.501</v>
+        <v>0.04</v>
       </c>
       <c r="I33" s="3">
-        <v>0.60119999999999996</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J33" s="3"/>
       <c r="K33" s="3" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
-        <v>110</v>
+        <v>129</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>150</v>
@@ -2032,31 +2039,31 @@
         <v>21</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E34" s="5">
-        <v>2.0000000000000002E-5</v>
+        <v>66</v>
+      </c>
+      <c r="E34" s="3">
+        <v>0.501</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G34" s="5">
-        <v>1.5999999999999999E-5</v>
-      </c>
-      <c r="H34" s="5">
-        <v>2.0000000000000002E-5</v>
-      </c>
-      <c r="I34" s="5">
-        <v>2.4000000000000001E-5</v>
+      <c r="G34" s="3">
+        <v>0.40079999999999999</v>
+      </c>
+      <c r="H34" s="3">
+        <v>0.501</v>
+      </c>
+      <c r="I34" s="3">
+        <v>0.60119999999999996</v>
       </c>
       <c r="J34" s="3"/>
       <c r="K34" s="3" t="s">
-        <v>92</v>
+        <v>57</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>150</v>
@@ -2067,62 +2074,62 @@
       <c r="D35" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="E35" s="3">
-        <v>0.10100000000000001</v>
+      <c r="E35" s="5">
+        <v>2.0000000000000002E-5</v>
       </c>
       <c r="F35" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G35" s="3">
-        <v>8.0799999999999997E-2</v>
-      </c>
-      <c r="H35" s="3">
-        <v>0.10100000000000001</v>
-      </c>
-      <c r="I35" s="3">
-        <v>0.1212</v>
+      <c r="G35" s="5">
+        <v>1.5999999999999999E-5</v>
+      </c>
+      <c r="H35" s="5">
+        <v>2.0000000000000002E-5</v>
+      </c>
+      <c r="I35" s="5">
+        <v>2.4000000000000001E-5</v>
       </c>
       <c r="J35" s="3"/>
       <c r="K35" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
-        <v>130</v>
+        <v>111</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E36" s="3">
-        <v>5.81</v>
+        <v>0.10100000000000001</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G36" s="3">
-        <v>4.6479999999999997</v>
+        <v>8.0799999999999997E-2</v>
       </c>
       <c r="H36" s="3">
-        <v>5.81</v>
+        <v>0.10100000000000001</v>
       </c>
       <c r="I36" s="3">
-        <v>6.9719999999999898</v>
+        <v>0.1212</v>
       </c>
       <c r="J36" s="3"/>
       <c r="K36" s="3" t="s">
-        <v>64</v>
+        <v>93</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
-        <v>112</v>
+        <v>130</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>151</v>
@@ -2131,64 +2138,64 @@
         <v>21</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E37" s="5">
-        <v>4.9999999999999998E-7</v>
+        <v>66</v>
+      </c>
+      <c r="E37" s="3">
+        <v>5.81</v>
       </c>
       <c r="F37" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G37" s="5">
-        <v>3.9999999999999998E-7</v>
-      </c>
-      <c r="H37" s="5">
-        <v>4.9999999999999998E-7</v>
-      </c>
-      <c r="I37" s="5">
-        <v>5.9999999999999997E-7</v>
+      <c r="G37" s="3">
+        <v>4.6479999999999997</v>
+      </c>
+      <c r="H37" s="3">
+        <v>5.81</v>
+      </c>
+      <c r="I37" s="3">
+        <v>6.9719999999999898</v>
       </c>
       <c r="J37" s="3"/>
       <c r="K37" s="3" t="s">
-        <v>94</v>
+        <v>64</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
-        <v>131</v>
+        <v>112</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="E38" s="3">
-        <v>4.8</v>
+        <v>68</v>
+      </c>
+      <c r="E38" s="5">
+        <v>4.9999999999999998E-7</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G38" s="3">
-        <v>3.84</v>
-      </c>
-      <c r="H38" s="3">
-        <v>4.8</v>
-      </c>
-      <c r="I38" s="3">
-        <v>5.76</v>
+      <c r="G38" s="5">
+        <v>3.9999999999999998E-7</v>
+      </c>
+      <c r="H38" s="5">
+        <v>4.9999999999999998E-7</v>
+      </c>
+      <c r="I38" s="5">
+        <v>5.9999999999999997E-7</v>
       </c>
       <c r="J38" s="3"/>
       <c r="K38" s="3" t="s">
-        <v>65</v>
+        <v>94</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>152</v>
@@ -2200,28 +2207,28 @@
         <v>66</v>
       </c>
       <c r="E39" s="3">
-        <v>0.04</v>
+        <v>4.8</v>
       </c>
       <c r="F39" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G39" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>3.84</v>
       </c>
       <c r="H39" s="3">
-        <v>0.04</v>
+        <v>4.8</v>
       </c>
       <c r="I39" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>5.76</v>
       </c>
       <c r="J39" s="3"/>
       <c r="K39" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>152</v>
@@ -2233,28 +2240,28 @@
         <v>66</v>
       </c>
       <c r="E40" s="3">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="F40" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G40" s="3">
-        <v>9.6000000000000002E-2</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H40" s="3">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="I40" s="3">
-        <v>0.14399999999999999</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J40" s="3"/>
       <c r="K40" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>152</v>
@@ -2266,28 +2273,28 @@
         <v>66</v>
       </c>
       <c r="E41" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="F41" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G41" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="H41" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="I41" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="J41" s="3"/>
       <c r="K41" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
-        <v>113</v>
+        <v>134</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>152</v>
@@ -2296,64 +2303,64 @@
         <v>21</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E42" s="3">
-        <v>2.6400000000000002E-4</v>
+        <v>0.04</v>
       </c>
       <c r="F42" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G42" s="3">
-        <v>2.1120000000000001E-4</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H42" s="3">
-        <v>2.6400000000000002E-4</v>
+        <v>0.04</v>
       </c>
       <c r="I42" s="3">
-        <v>3.168E-4</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J42" s="3"/>
       <c r="K42" s="3" t="s">
-        <v>95</v>
+        <v>71</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
-        <v>135</v>
+        <v>113</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E43" s="3">
-        <v>1.04E-2</v>
+        <v>2.6400000000000002E-4</v>
       </c>
       <c r="F43" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G43" s="3">
-        <v>8.3199999999999993E-3</v>
+        <v>2.1120000000000001E-4</v>
       </c>
       <c r="H43" s="3">
-        <v>1.04E-2</v>
+        <v>2.6400000000000002E-4</v>
       </c>
       <c r="I43" s="3">
-        <v>1.248E-2</v>
+        <v>3.168E-4</v>
       </c>
       <c r="J43" s="3"/>
       <c r="K43" s="3" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>157</v>
@@ -2362,31 +2369,31 @@
         <v>21</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E44" s="3">
-        <v>1.0200000000000001E-2</v>
+        <v>1.04E-2</v>
       </c>
       <c r="F44" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G44" s="3">
-        <v>8.1600000000000006E-3</v>
+        <v>8.3199999999999993E-3</v>
       </c>
       <c r="H44" s="3">
-        <v>1.0200000000000001E-2</v>
+        <v>1.04E-2</v>
       </c>
       <c r="I44" s="3">
-        <v>1.2239999999999999E-2</v>
+        <v>1.248E-2</v>
       </c>
       <c r="J44" s="3"/>
       <c r="K44" s="3" t="s">
-        <v>96</v>
+        <v>72</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" s="3" t="s">
-        <v>136</v>
+        <v>114</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>157</v>
@@ -2395,31 +2402,31 @@
         <v>21</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E45" s="3">
-        <v>0.77500000000000002</v>
+        <v>1.0200000000000001E-2</v>
       </c>
       <c r="F45" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G45" s="3">
-        <v>0.62</v>
+        <v>8.1600000000000006E-3</v>
       </c>
       <c r="H45" s="3">
-        <v>0.77500000000000002</v>
+        <v>1.0200000000000001E-2</v>
       </c>
       <c r="I45" s="3">
-        <v>0.92999999999999905</v>
+        <v>1.2239999999999999E-2</v>
       </c>
       <c r="J45" s="3"/>
       <c r="K45" s="3" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
-        <v>115</v>
+        <v>136</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>157</v>
@@ -2428,31 +2435,31 @@
         <v>21</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E46" s="3">
-        <v>0.1</v>
+        <v>0.77500000000000002</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G46" s="3">
-        <v>0.08</v>
+        <v>0.62</v>
       </c>
       <c r="H46" s="3">
-        <v>0.1</v>
+        <v>0.77500000000000002</v>
       </c>
       <c r="I46" s="3">
-        <v>0.12</v>
+        <v>0.92999999999999905</v>
       </c>
       <c r="J46" s="3"/>
       <c r="K46" s="3" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B47" s="3" t="s">
         <v>157</v>
@@ -2464,61 +2471,61 @@
         <v>68</v>
       </c>
       <c r="E47" s="3">
-        <v>440</v>
+        <v>0.1</v>
       </c>
       <c r="F47" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G47" s="3">
-        <v>352</v>
+        <v>0.08</v>
       </c>
       <c r="H47" s="3">
-        <v>440</v>
+        <v>0.1</v>
       </c>
       <c r="I47" s="3">
-        <v>528</v>
+        <v>0.12</v>
       </c>
       <c r="J47" s="3"/>
       <c r="K47" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" s="3" t="s">
-        <v>137</v>
+        <v>116</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E48" s="3">
-        <v>2.82</v>
+        <v>440</v>
       </c>
       <c r="F48" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G48" s="3">
-        <v>2.2559999999999998</v>
+        <v>352</v>
       </c>
       <c r="H48" s="3">
-        <v>2.82</v>
+        <v>440</v>
       </c>
       <c r="I48" s="3">
-        <v>3.3839999999999999</v>
+        <v>528</v>
       </c>
       <c r="J48" s="3"/>
       <c r="K48" s="3" t="s">
-        <v>74</v>
+        <v>98</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B49" s="3" t="s">
         <v>153</v>
@@ -2530,28 +2537,28 @@
         <v>66</v>
       </c>
       <c r="E49" s="3">
-        <v>1.2500000000000001E-2</v>
+        <v>2.82</v>
       </c>
       <c r="F49" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G49" s="3">
-        <v>0.01</v>
+        <v>2.2559999999999998</v>
       </c>
       <c r="H49" s="3">
-        <v>1.2500000000000001E-2</v>
+        <v>2.82</v>
       </c>
       <c r="I49" s="3">
-        <v>1.4999999999999999E-2</v>
+        <v>3.3839999999999999</v>
       </c>
       <c r="J49" s="3"/>
       <c r="K49" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" s="3" t="s">
-        <v>117</v>
+        <v>138</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>153</v>
@@ -2560,31 +2567,31 @@
         <v>21</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E50" s="3">
-        <v>3.4000000000000002E-2</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="F50" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G50" s="3">
-        <v>2.7199999999999998E-2</v>
+        <v>0.01</v>
       </c>
       <c r="H50" s="3">
-        <v>3.4000000000000002E-2</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="I50" s="3">
-        <v>4.0800000000000003E-2</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="J50" s="3"/>
       <c r="K50" s="3" t="s">
-        <v>99</v>
+        <v>75</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>153</v>
@@ -2596,61 +2603,61 @@
         <v>68</v>
       </c>
       <c r="E51" s="3">
-        <v>5.7000000000000002E-2</v>
+        <v>3.4000000000000002E-2</v>
       </c>
       <c r="F51" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G51" s="3">
-        <v>4.5600000000000002E-2</v>
+        <v>2.7199999999999998E-2</v>
       </c>
       <c r="H51" s="3">
-        <v>5.7000000000000002E-2</v>
+        <v>3.4000000000000002E-2</v>
       </c>
       <c r="I51" s="3">
-        <v>6.8400000000000002E-2</v>
+        <v>4.0800000000000003E-2</v>
       </c>
       <c r="J51" s="3"/>
       <c r="K51" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" s="3" t="s">
-        <v>139</v>
+        <v>118</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E52" s="3">
-        <v>1.2030000000000001</v>
+        <v>5.7000000000000002E-2</v>
       </c>
       <c r="F52" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G52" s="3">
-        <v>0.96240000000000003</v>
+        <v>4.5600000000000002E-2</v>
       </c>
       <c r="H52" s="3">
-        <v>1.2030000000000001</v>
+        <v>5.7000000000000002E-2</v>
       </c>
       <c r="I52" s="3">
-        <v>1.4436</v>
+        <v>6.8400000000000002E-2</v>
       </c>
       <c r="J52" s="3"/>
       <c r="K52" s="3" t="s">
-        <v>76</v>
+        <v>100</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>154</v>
@@ -2662,28 +2669,28 @@
         <v>66</v>
       </c>
       <c r="E53" s="3">
-        <v>0.04</v>
+        <v>1.2030000000000001</v>
       </c>
       <c r="F53" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G53" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>0.96240000000000003</v>
       </c>
       <c r="H53" s="3">
-        <v>0.04</v>
+        <v>1.2030000000000001</v>
       </c>
       <c r="I53" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>1.4436</v>
       </c>
       <c r="J53" s="3"/>
       <c r="K53" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B54" s="3" t="s">
         <v>154</v>
@@ -2695,28 +2702,28 @@
         <v>66</v>
       </c>
       <c r="E54" s="3">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="F54" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G54" s="3">
-        <v>9.6000000000000002E-2</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H54" s="3">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="I54" s="3">
-        <v>0.14399999999999999</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J54" s="3"/>
       <c r="K54" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B55" s="3" t="s">
         <v>154</v>
@@ -2728,28 +2735,28 @@
         <v>66</v>
       </c>
       <c r="E55" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="F55" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G55" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="H55" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="I55" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="J55" s="3"/>
       <c r="K55" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
-        <v>119</v>
+        <v>142</v>
       </c>
       <c r="B56" s="3" t="s">
         <v>154</v>
@@ -2758,67 +2765,67 @@
         <v>21</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E56" s="3">
-        <v>1.01E-2</v>
+        <v>0.04</v>
       </c>
       <c r="F56" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G56" s="3">
-        <v>8.0800000000000004E-3</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H56" s="3">
-        <v>1.01E-2</v>
+        <v>0.04</v>
       </c>
       <c r="I56" s="3">
-        <v>1.21199999999999E-2</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J56" s="3"/>
       <c r="K56" s="3" t="s">
-        <v>101</v>
+        <v>79</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" s="3" t="s">
-        <v>143</v>
+        <v>119</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C57" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E57" s="3">
-        <v>0.58899999999999997</v>
+        <v>1.01E-2</v>
       </c>
       <c r="F57" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G57" s="3">
-        <v>0.47120000000000001</v>
+        <v>8.0800000000000004E-3</v>
       </c>
       <c r="H57" s="3">
-        <v>0.58899999999999997</v>
+        <v>1.01E-2</v>
       </c>
       <c r="I57" s="3">
-        <v>0.70679999999999998</v>
+        <v>1.21199999999999E-2</v>
       </c>
       <c r="J57" s="3"/>
       <c r="K57" s="3" t="s">
-        <v>80</v>
+        <v>101</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C58" s="3" t="s">
         <v>21</v>
@@ -2827,28 +2834,28 @@
         <v>66</v>
       </c>
       <c r="E58" s="3">
-        <v>8.0000000000000002E-3</v>
+        <v>0.58899999999999997</v>
       </c>
       <c r="F58" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G58" s="3">
-        <v>6.4000000000000003E-3</v>
+        <v>0.47120000000000001</v>
       </c>
       <c r="H58" s="3">
-        <v>8.0000000000000002E-3</v>
+        <v>0.58899999999999997</v>
       </c>
       <c r="I58" s="3">
-        <v>9.5999999999999992E-3</v>
+        <v>0.70679999999999998</v>
       </c>
       <c r="J58" s="3"/>
       <c r="K58" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" s="3" t="s">
-        <v>120</v>
+        <v>144</v>
       </c>
       <c r="B59" s="3" t="s">
         <v>156</v>
@@ -2857,31 +2864,31 @@
         <v>21</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E59" s="5">
-        <v>9.9999999999999995E-7</v>
+        <v>66</v>
+      </c>
+      <c r="E59" s="3">
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="F59" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G59" s="5">
-        <v>7.9999999999999996E-7</v>
-      </c>
-      <c r="H59" s="5">
-        <v>9.9999999999999995E-7</v>
-      </c>
-      <c r="I59" s="5">
-        <v>1.1999999999999999E-6</v>
+      <c r="G59" s="3">
+        <v>6.4000000000000003E-3</v>
+      </c>
+      <c r="H59" s="3">
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="I59" s="3">
+        <v>9.5999999999999992E-3</v>
       </c>
       <c r="J59" s="3"/>
       <c r="K59" s="3" t="s">
-        <v>102</v>
+        <v>81</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" s="3" t="s">
-        <v>145</v>
+        <v>120</v>
       </c>
       <c r="B60" s="3" t="s">
         <v>156</v>
@@ -2890,31 +2897,31 @@
         <v>21</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="E60" s="3">
-        <v>7.51E-2</v>
+        <v>68</v>
+      </c>
+      <c r="E60" s="5">
+        <v>9.9999999999999995E-7</v>
       </c>
       <c r="F60" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G60" s="3">
-        <v>6.0080000000000001E-2</v>
-      </c>
-      <c r="H60" s="3">
-        <v>7.51E-2</v>
-      </c>
-      <c r="I60" s="3">
-        <v>9.0119999999999895E-2</v>
+      <c r="G60" s="5">
+        <v>7.9999999999999996E-7</v>
+      </c>
+      <c r="H60" s="5">
+        <v>9.9999999999999995E-7</v>
+      </c>
+      <c r="I60" s="5">
+        <v>1.1999999999999999E-6</v>
       </c>
       <c r="J60" s="3"/>
       <c r="K60" s="3" t="s">
-        <v>82</v>
+        <v>102</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
-        <v>121</v>
+        <v>145</v>
       </c>
       <c r="B61" s="3" t="s">
         <v>156</v>
@@ -2923,31 +2930,31 @@
         <v>21</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E61" s="3">
-        <v>13</v>
+        <v>7.51E-2</v>
       </c>
       <c r="F61" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G61" s="3">
-        <v>10.4</v>
+        <v>6.0080000000000001E-2</v>
       </c>
       <c r="H61" s="3">
-        <v>13</v>
+        <v>7.51E-2</v>
       </c>
       <c r="I61" s="3">
-        <v>15.6</v>
+        <v>9.0119999999999895E-2</v>
       </c>
       <c r="J61" s="3"/>
       <c r="K61" s="3" t="s">
-        <v>103</v>
+        <v>82</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B62" s="3" t="s">
         <v>156</v>
@@ -2959,28 +2966,28 @@
         <v>68</v>
       </c>
       <c r="E62" s="3">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="F62" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G62" s="3">
-        <v>20</v>
+        <v>10.4</v>
       </c>
       <c r="H62" s="3">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="I62" s="3">
-        <v>30</v>
+        <v>15.6</v>
       </c>
       <c r="J62" s="3"/>
       <c r="K62" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" s="3" t="s">
-        <v>146</v>
+        <v>122</v>
       </c>
       <c r="B63" s="3" t="s">
         <v>156</v>
@@ -2989,34 +2996,34 @@
         <v>21</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E63" s="3">
-        <v>3.9899999999999996E-3</v>
+        <v>25</v>
       </c>
       <c r="F63" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G63" s="3">
-        <v>3.192E-3</v>
+        <v>20</v>
       </c>
       <c r="H63" s="3">
-        <v>3.9899999999999996E-3</v>
+        <v>25</v>
       </c>
       <c r="I63" s="3">
-        <v>4.7879999999999997E-3</v>
+        <v>30</v>
       </c>
       <c r="J63" s="3"/>
       <c r="K63" s="3" t="s">
-        <v>83</v>
+        <v>104</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A64" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C64" s="3" t="s">
         <v>21</v>
@@ -3025,31 +3032,31 @@
         <v>66</v>
       </c>
       <c r="E64" s="3">
-        <v>0.06</v>
+        <v>3.9899999999999996E-3</v>
       </c>
       <c r="F64" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G64" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>3.192E-3</v>
       </c>
       <c r="H64" s="3">
-        <v>0.06</v>
+        <v>3.9899999999999996E-3</v>
       </c>
       <c r="I64" s="3">
-        <v>7.1999999999999995E-2</v>
+        <v>4.7879999999999997E-3</v>
       </c>
       <c r="J64" s="3"/>
       <c r="K64" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A65" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C65" s="3" t="s">
         <v>21</v>
@@ -3058,22 +3065,55 @@
         <v>66</v>
       </c>
       <c r="E65" s="3">
-        <v>0.02</v>
+        <v>0.06</v>
       </c>
       <c r="F65" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G65" s="3">
-        <v>1.6E-2</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="H65" s="3">
-        <v>0.02</v>
+        <v>0.06</v>
       </c>
       <c r="I65" s="3">
-        <v>2.4E-2</v>
+        <v>7.1999999999999995E-2</v>
       </c>
       <c r="J65" s="3"/>
       <c r="K65" s="3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A66" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E66" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="F66" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="G66" s="3">
+        <v>1.6E-2</v>
+      </c>
+      <c r="H66" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="I66" s="3">
+        <v>2.4E-2</v>
+      </c>
+      <c r="J66" s="3"/>
+      <c r="K66" s="3" t="s">
         <v>85</v>
       </c>
     </row>

</xml_diff>

<commit_message>
major updates, includingoptional ethanol separation bypass, new unit groups, and plots
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saran\Documents\Academia\repository_clones\Bioindustrial-Park\biorefineries\isobutanol\analyses\full\parameter_distributions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EAC69E3-624C-4D8A-BDDC-ED485D55ABE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38C5CEFF-4B82-48F3-94B3-0E17AD8402FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3380" yWindow="0" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6100" yWindow="2720" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="170">
   <si>
     <t>Parameter name</t>
   </si>
@@ -194,9 +194,6 @@
     <t>denaturant.price = x</t>
   </si>
   <si>
-    <t>Steam jet cooking unit price</t>
-  </si>
-  <si>
     <t>Product ethanol storage time</t>
   </si>
   <si>
@@ -353,9 +350,6 @@
     <t>V406.kinetic_reaction_system._te.K_9i = x</t>
   </si>
   <si>
-    <t>steam.price = x</t>
-  </si>
-  <si>
     <t>K_1l</t>
   </si>
   <si>
@@ -536,12 +530,6 @@
     <t>feedstock.imass['Starch'] =x * feedstock.imass['Water']</t>
   </si>
   <si>
-    <t>Isobutanol unit price</t>
-  </si>
-  <si>
-    <t>DDGS unit price</t>
-  </si>
-  <si>
     <t>Isopentyl acetate unit price</t>
   </si>
   <si>
@@ -552,6 +540,12 @@
   </si>
   <si>
     <t>V406.aeration_safety_factor = x</t>
+  </si>
+  <si>
+    <t>DDGS unit price (sale)</t>
+  </si>
+  <si>
+    <t>Isobutanol selling unit price (sale)</t>
   </si>
 </sst>
 </file>
@@ -914,7 +908,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K66"/>
+  <dimension ref="A1:K65"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="40.81640625" customWidth="1"/>
@@ -1115,12 +1109,12 @@
         <v>18</v>
       </c>
       <c r="G6" s="4">
-        <f t="shared" ref="G6:G14" si="0">E6*0.8</f>
+        <f t="shared" ref="G6:G13" si="0">E6*0.8</f>
         <v>0.35920000000000002</v>
       </c>
       <c r="H6" s="4"/>
       <c r="I6" s="4">
-        <f t="shared" ref="I6:I14" si="1">1.2*E6</f>
+        <f t="shared" ref="I6:I13" si="1">1.2*E6</f>
         <v>0.53879999999999995</v>
       </c>
       <c r="J6" s="4"/>
@@ -1262,7 +1256,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
-        <v>52</v>
+        <v>168</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>7</v>
@@ -1274,28 +1268,28 @@
         <v>10</v>
       </c>
       <c r="E11" s="4">
-        <v>1.2999999999999999E-2</v>
+        <v>0.12</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>18</v>
       </c>
       <c r="G11" s="4">
         <f t="shared" si="0"/>
-        <v>1.04E-2</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="H11" s="4"/>
       <c r="I11" s="4">
         <f t="shared" si="1"/>
-        <v>1.5599999999999999E-2</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="J11" s="4"/>
       <c r="K11" s="4" t="s">
-        <v>105</v>
+        <v>159</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>7</v>
@@ -1307,28 +1301,29 @@
         <v>10</v>
       </c>
       <c r="E12" s="4">
-        <v>0.12</v>
+        <v>1.49</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="G12" s="4">
-        <f t="shared" si="0"/>
-        <v>9.6000000000000002E-2</v>
-      </c>
-      <c r="H12" s="4"/>
+        <v>0.95</v>
+      </c>
+      <c r="H12" s="4">
+        <f>E12</f>
+        <v>1.49</v>
+      </c>
       <c r="I12" s="4">
-        <f t="shared" si="1"/>
-        <v>0.14399999999999999</v>
+        <v>1.7250000000000001</v>
       </c>
       <c r="J12" s="4"/>
       <c r="K12" s="4" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>7</v>
@@ -1340,17 +1335,19 @@
         <v>10</v>
       </c>
       <c r="E13" s="4">
-        <v>1.49</v>
+        <v>3.2</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>18</v>
       </c>
       <c r="G13" s="4">
-        <v>0.95</v>
+        <f t="shared" si="0"/>
+        <v>2.5600000000000005</v>
       </c>
       <c r="H13" s="4"/>
       <c r="I13" s="4">
-        <v>1.7250000000000001</v>
+        <f t="shared" si="1"/>
+        <v>3.84</v>
       </c>
       <c r="J13" s="4"/>
       <c r="K13" s="4" t="s">
@@ -1358,41 +1355,41 @@
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A14" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="B14" s="4" t="s">
+      <c r="A14" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E14" s="4">
-        <v>3.2</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G14" s="4">
-        <f t="shared" si="0"/>
-        <v>2.5600000000000005</v>
-      </c>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4">
-        <f t="shared" si="1"/>
-        <v>3.84</v>
-      </c>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4" t="s">
-        <v>162</v>
+      <c r="E14" s="6">
+        <v>0.28599999999999998</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G14" s="6">
+        <v>0.17499999999999999</v>
+      </c>
+      <c r="H14" s="6">
+        <v>0.28599999999999998</v>
+      </c>
+      <c r="I14" s="6">
+        <v>0.315</v>
+      </c>
+      <c r="J14" s="6"/>
+      <c r="K14" s="6" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>7</v>
@@ -1404,19 +1401,22 @@
         <v>10</v>
       </c>
       <c r="E15" s="6">
-        <v>0.28599999999999998</v>
+        <v>0.10355</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>27</v>
       </c>
       <c r="G15" s="6">
-        <v>0.17499999999999999</v>
+        <f>E15*0.9</f>
+        <v>9.3195E-2</v>
       </c>
       <c r="H15" s="6">
-        <v>0.28599999999999998</v>
+        <f>E15</f>
+        <v>0.10355</v>
       </c>
       <c r="I15" s="6">
-        <v>0.315</v>
+        <f>E15*1.1</f>
+        <v>0.11390500000000001</v>
       </c>
       <c r="J15" s="6"/>
       <c r="K15" s="6" t="s">
@@ -1424,44 +1424,39 @@
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A16" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B16" s="6" t="s">
+      <c r="A16" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E16" s="6">
-        <v>0.10355</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="G16" s="6">
-        <f>E16*0.9</f>
-        <v>9.3195E-2</v>
-      </c>
-      <c r="H16" s="6">
-        <f>E16</f>
-        <v>0.10355</v>
-      </c>
-      <c r="I16" s="6">
-        <f>E16*1.1</f>
-        <v>0.11390500000000001</v>
-      </c>
-      <c r="J16" s="6"/>
-      <c r="K16" s="6" t="s">
-        <v>87</v>
+      <c r="D16" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E16" s="3">
+        <v>0.21</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G16" s="3">
+        <v>0.15</v>
+      </c>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>7</v>
@@ -1473,59 +1468,64 @@
         <v>8</v>
       </c>
       <c r="E17" s="3">
-        <v>0.21</v>
+        <v>0.15</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>18</v>
       </c>
       <c r="G17" s="3">
-        <v>0.15</v>
+        <f>0.8*E17</f>
+        <v>0.12</v>
       </c>
       <c r="H17" s="3"/>
       <c r="I17" s="3">
-        <v>0.28000000000000003</v>
+        <f>1.2*E17</f>
+        <v>0.18</v>
       </c>
       <c r="J17" s="3"/>
       <c r="K17" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>32</v>
+        <v>161</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>7</v>
+        <v>39</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>8</v>
+        <v>162</v>
       </c>
       <c r="E18" s="3">
-        <v>0.15</v>
+        <v>4.08</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="G18" s="3">
-        <f>0.8*E18</f>
-        <v>0.12</v>
-      </c>
-      <c r="H18" s="3"/>
+        <f>0.8*H18</f>
+        <v>3.2640000000000002</v>
+      </c>
+      <c r="H18" s="3">
+        <f>E18</f>
+        <v>4.08</v>
+      </c>
       <c r="I18" s="3">
-        <f>1.2*E18</f>
-        <v>0.18</v>
+        <f>1.2*H18</f>
+        <v>4.8959999999999999</v>
       </c>
       <c r="J18" s="3"/>
       <c r="K18" s="3" t="s">
-        <v>33</v>
+        <v>163</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>163</v>
+        <v>38</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>39</v>
@@ -1534,96 +1534,96 @@
         <v>21</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>164</v>
+        <v>40</v>
       </c>
       <c r="E19" s="3">
-        <v>4.08</v>
+        <v>56972</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>27</v>
       </c>
       <c r="G19" s="3">
         <f>0.8*H19</f>
-        <v>3.2640000000000002</v>
+        <v>45577.600000000006</v>
       </c>
       <c r="H19" s="3">
         <f>E19</f>
-        <v>4.08</v>
+        <v>56972</v>
       </c>
       <c r="I19" s="3">
         <f>1.2*H19</f>
-        <v>4.8959999999999999</v>
+        <v>68366.399999999994</v>
       </c>
       <c r="J19" s="3"/>
       <c r="K19" s="3" t="s">
-        <v>165</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>38</v>
+        <v>165</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>39</v>
+        <v>166</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="E20" s="3">
-        <v>56972</v>
+        <v>2</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="G20" s="3">
-        <f>0.8*H20</f>
-        <v>45577.600000000006</v>
-      </c>
-      <c r="H20" s="3">
-        <f>E20</f>
-        <v>56972</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H20" s="3"/>
       <c r="I20" s="3">
-        <f>1.2*H20</f>
-        <v>68366.399999999994</v>
+        <v>3</v>
       </c>
       <c r="J20" s="3"/>
       <c r="K20" s="3" t="s">
-        <v>41</v>
+        <v>167</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>169</v>
+        <v>52</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>170</v>
+        <v>13</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E21" s="3">
-        <v>2</v>
+        <v>156</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="G21" s="3">
-        <v>1</v>
-      </c>
-      <c r="H21" s="3"/>
+        <f>E21*0.8</f>
+        <v>124.80000000000001</v>
+      </c>
+      <c r="H21" s="3">
+        <f>E21</f>
+        <v>156</v>
+      </c>
       <c r="I21" s="3">
-        <v>3</v>
+        <f>E21*1.2</f>
+        <v>187.2</v>
       </c>
       <c r="J21" s="3"/>
       <c r="K21" s="3" t="s">
-        <v>171</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.35">
@@ -1664,232 +1664,229 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>54</v>
+        <v>121</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>13</v>
+        <v>147</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>14</v>
+        <v>65</v>
       </c>
       <c r="E23" s="3">
-        <v>156</v>
+        <v>1.43</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>27</v>
+        <v>66</v>
       </c>
       <c r="G23" s="3">
-        <f>E23*0.8</f>
-        <v>124.80000000000001</v>
+        <v>1.1439999999999999</v>
       </c>
       <c r="H23" s="3">
-        <f>E23</f>
-        <v>156</v>
+        <v>1.43</v>
       </c>
       <c r="I23" s="3">
-        <f>E23*1.2</f>
-        <v>187.2</v>
+        <v>1.716</v>
       </c>
       <c r="J23" s="3"/>
       <c r="K23" s="3" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>123</v>
+        <v>104</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E24" s="3">
-        <v>1.43</v>
+        <v>0.94</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G24" s="3">
-        <v>1.1439999999999999</v>
+        <v>0.752</v>
       </c>
       <c r="H24" s="3">
-        <v>1.43</v>
+        <v>0.94</v>
       </c>
       <c r="I24" s="3">
-        <v>1.716</v>
+        <v>1.1279999999999999</v>
       </c>
       <c r="J24" s="3"/>
       <c r="K24" s="3" t="s">
-        <v>63</v>
+        <v>87</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E25" s="3">
-        <v>0.94</v>
+        <v>0.58399999999999996</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G25" s="3">
-        <v>0.752</v>
+        <v>0.4672</v>
       </c>
       <c r="H25" s="3">
-        <v>0.94</v>
+        <v>0.58399999999999996</v>
       </c>
       <c r="I25" s="3">
-        <v>1.1279999999999999</v>
+        <v>0.70079999999999998</v>
       </c>
       <c r="J25" s="3"/>
       <c r="K25" s="3" t="s">
-        <v>88</v>
+        <v>58</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E26" s="3">
-        <v>0.58399999999999996</v>
+        <v>1.1599999999999999E-2</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G26" s="3">
-        <v>0.4672</v>
+        <v>9.2800000000000001E-3</v>
       </c>
       <c r="H26" s="3">
-        <v>0.58399999999999996</v>
+        <v>1.1599999999999999E-2</v>
       </c>
       <c r="I26" s="3">
-        <v>0.70079999999999998</v>
+        <v>1.3919999999999899E-2</v>
       </c>
       <c r="J26" s="3"/>
       <c r="K26" s="3" t="s">
-        <v>59</v>
+        <v>88</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E27" s="3">
-        <v>1.1599999999999999E-2</v>
+        <v>47.1</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G27" s="3">
-        <v>9.2800000000000001E-3</v>
+        <v>37.68</v>
       </c>
       <c r="H27" s="3">
-        <v>1.1599999999999999E-2</v>
+        <v>47.1</v>
       </c>
       <c r="I27" s="3">
-        <v>1.3919999999999899E-2</v>
+        <v>56.52</v>
       </c>
       <c r="J27" s="3"/>
       <c r="K27" s="3" t="s">
-        <v>89</v>
+        <v>57</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>125</v>
+        <v>106</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E28" s="3">
-        <v>47.1</v>
+        <v>14.2</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G28" s="3">
-        <v>37.68</v>
+        <v>11.36</v>
       </c>
       <c r="H28" s="3">
-        <v>47.1</v>
+        <v>14.2</v>
       </c>
       <c r="I28" s="3">
-        <v>56.52</v>
+        <v>17.04</v>
       </c>
       <c r="J28" s="3"/>
       <c r="K28" s="3" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E29" s="3">
-        <v>14.2</v>
+        <v>0.12</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G29" s="3">
-        <v>11.36</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="H29" s="3">
-        <v>14.2</v>
+        <v>0.12</v>
       </c>
       <c r="I29" s="3">
-        <v>17.04</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="J29" s="3"/>
       <c r="K29" s="3" t="s">
@@ -1898,64 +1895,64 @@
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E30" s="3">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G30" s="3">
-        <v>9.6000000000000002E-2</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H30" s="3">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="I30" s="3">
-        <v>0.14399999999999999</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J30" s="3"/>
       <c r="K30" s="3" t="s">
-        <v>91</v>
+        <v>59</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E31" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G31" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="H31" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="I31" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="J31" s="3"/>
       <c r="K31" s="3" t="s">
@@ -1964,31 +1961,31 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E32" s="3">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G32" s="3">
-        <v>9.6000000000000002E-2</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H32" s="3">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="I32" s="3">
-        <v>0.14399999999999999</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J32" s="3"/>
       <c r="K32" s="3" t="s">
@@ -1997,97 +1994,97 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E33" s="3">
-        <v>0.04</v>
+        <v>0.501</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G33" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>0.40079999999999999</v>
       </c>
       <c r="H33" s="3">
-        <v>0.04</v>
+        <v>0.501</v>
       </c>
       <c r="I33" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>0.60119999999999996</v>
       </c>
       <c r="J33" s="3"/>
       <c r="K33" s="3" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
-        <v>129</v>
+        <v>108</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="E34" s="3">
-        <v>0.501</v>
+        <v>67</v>
+      </c>
+      <c r="E34" s="5">
+        <v>2.0000000000000002E-5</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="G34" s="3">
-        <v>0.40079999999999999</v>
-      </c>
-      <c r="H34" s="3">
-        <v>0.501</v>
-      </c>
-      <c r="I34" s="3">
-        <v>0.60119999999999996</v>
+        <v>66</v>
+      </c>
+      <c r="G34" s="5">
+        <v>1.5999999999999999E-5</v>
+      </c>
+      <c r="H34" s="5">
+        <v>2.0000000000000002E-5</v>
+      </c>
+      <c r="I34" s="5">
+        <v>2.4000000000000001E-5</v>
       </c>
       <c r="J34" s="3"/>
       <c r="K34" s="3" t="s">
-        <v>57</v>
+        <v>91</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E35" s="5">
-        <v>2.0000000000000002E-5</v>
+        <v>67</v>
+      </c>
+      <c r="E35" s="3">
+        <v>0.10100000000000001</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="G35" s="5">
-        <v>1.5999999999999999E-5</v>
-      </c>
-      <c r="H35" s="5">
-        <v>2.0000000000000002E-5</v>
-      </c>
-      <c r="I35" s="5">
-        <v>2.4000000000000001E-5</v>
+        <v>66</v>
+      </c>
+      <c r="G35" s="3">
+        <v>8.0799999999999997E-2</v>
+      </c>
+      <c r="H35" s="3">
+        <v>0.10100000000000001</v>
+      </c>
+      <c r="I35" s="3">
+        <v>0.1212</v>
       </c>
       <c r="J35" s="3"/>
       <c r="K35" s="3" t="s">
@@ -2096,163 +2093,163 @@
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E36" s="3">
-        <v>0.10100000000000001</v>
+        <v>5.81</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G36" s="3">
-        <v>8.0799999999999997E-2</v>
+        <v>4.6479999999999997</v>
       </c>
       <c r="H36" s="3">
-        <v>0.10100000000000001</v>
+        <v>5.81</v>
       </c>
       <c r="I36" s="3">
-        <v>0.1212</v>
+        <v>6.9719999999999898</v>
       </c>
       <c r="J36" s="3"/>
       <c r="K36" s="3" t="s">
-        <v>93</v>
+        <v>63</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="E37" s="3">
-        <v>5.81</v>
+        <v>67</v>
+      </c>
+      <c r="E37" s="5">
+        <v>4.9999999999999998E-7</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="G37" s="3">
-        <v>4.6479999999999997</v>
-      </c>
-      <c r="H37" s="3">
-        <v>5.81</v>
-      </c>
-      <c r="I37" s="3">
-        <v>6.9719999999999898</v>
+        <v>66</v>
+      </c>
+      <c r="G37" s="5">
+        <v>3.9999999999999998E-7</v>
+      </c>
+      <c r="H37" s="5">
+        <v>4.9999999999999998E-7</v>
+      </c>
+      <c r="I37" s="5">
+        <v>5.9999999999999997E-7</v>
       </c>
       <c r="J37" s="3"/>
       <c r="K37" s="3" t="s">
-        <v>64</v>
+        <v>93</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E38" s="5">
-        <v>4.9999999999999998E-7</v>
+        <v>65</v>
+      </c>
+      <c r="E38" s="3">
+        <v>4.8</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="G38" s="5">
-        <v>3.9999999999999998E-7</v>
-      </c>
-      <c r="H38" s="5">
-        <v>4.9999999999999998E-7</v>
-      </c>
-      <c r="I38" s="5">
-        <v>5.9999999999999997E-7</v>
+        <v>66</v>
+      </c>
+      <c r="G38" s="3">
+        <v>3.84</v>
+      </c>
+      <c r="H38" s="3">
+        <v>4.8</v>
+      </c>
+      <c r="I38" s="3">
+        <v>5.76</v>
       </c>
       <c r="J38" s="3"/>
       <c r="K38" s="3" t="s">
-        <v>94</v>
+        <v>64</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E39" s="3">
-        <v>4.8</v>
+        <v>0.04</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G39" s="3">
-        <v>3.84</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H39" s="3">
-        <v>4.8</v>
+        <v>0.04</v>
       </c>
       <c r="I39" s="3">
-        <v>5.76</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J39" s="3"/>
       <c r="K39" s="3" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E40" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G40" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="H40" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="I40" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="J40" s="3"/>
       <c r="K40" s="3" t="s">
@@ -2261,31 +2258,31 @@
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E41" s="3">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G41" s="3">
-        <v>9.6000000000000002E-2</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H41" s="3">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="I41" s="3">
-        <v>0.14399999999999999</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J41" s="3"/>
       <c r="K41" s="3" t="s">
@@ -2294,196 +2291,196 @@
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
-        <v>134</v>
+        <v>111</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E42" s="3">
-        <v>0.04</v>
+        <v>2.6400000000000002E-4</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G42" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>2.1120000000000001E-4</v>
       </c>
       <c r="H42" s="3">
-        <v>0.04</v>
+        <v>2.6400000000000002E-4</v>
       </c>
       <c r="I42" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>3.168E-4</v>
       </c>
       <c r="J42" s="3"/>
       <c r="K42" s="3" t="s">
-        <v>71</v>
+        <v>94</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
-        <v>113</v>
+        <v>133</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E43" s="3">
-        <v>2.6400000000000002E-4</v>
+        <v>1.04E-2</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G43" s="3">
-        <v>2.1120000000000001E-4</v>
+        <v>8.3199999999999993E-3</v>
       </c>
       <c r="H43" s="3">
-        <v>2.6400000000000002E-4</v>
+        <v>1.04E-2</v>
       </c>
       <c r="I43" s="3">
-        <v>3.168E-4</v>
+        <v>1.248E-2</v>
       </c>
       <c r="J43" s="3"/>
       <c r="K43" s="3" t="s">
-        <v>95</v>
+        <v>71</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
-        <v>135</v>
+        <v>112</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E44" s="3">
-        <v>1.04E-2</v>
+        <v>1.0200000000000001E-2</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G44" s="3">
-        <v>8.3199999999999993E-3</v>
+        <v>8.1600000000000006E-3</v>
       </c>
       <c r="H44" s="3">
-        <v>1.04E-2</v>
+        <v>1.0200000000000001E-2</v>
       </c>
       <c r="I44" s="3">
-        <v>1.248E-2</v>
+        <v>1.2239999999999999E-2</v>
       </c>
       <c r="J44" s="3"/>
       <c r="K44" s="3" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" s="3" t="s">
-        <v>114</v>
+        <v>134</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E45" s="3">
-        <v>1.0200000000000001E-2</v>
+        <v>0.77500000000000002</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G45" s="3">
-        <v>8.1600000000000006E-3</v>
+        <v>0.62</v>
       </c>
       <c r="H45" s="3">
-        <v>1.0200000000000001E-2</v>
+        <v>0.77500000000000002</v>
       </c>
       <c r="I45" s="3">
-        <v>1.2239999999999999E-2</v>
+        <v>0.92999999999999905</v>
       </c>
       <c r="J45" s="3"/>
       <c r="K45" s="3" t="s">
-        <v>96</v>
+        <v>72</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
-        <v>136</v>
+        <v>113</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E46" s="3">
-        <v>0.77500000000000002</v>
+        <v>0.1</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G46" s="3">
-        <v>0.62</v>
+        <v>0.08</v>
       </c>
       <c r="H46" s="3">
-        <v>0.77500000000000002</v>
+        <v>0.1</v>
       </c>
       <c r="I46" s="3">
-        <v>0.92999999999999905</v>
+        <v>0.12</v>
       </c>
       <c r="J46" s="3"/>
       <c r="K46" s="3" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E47" s="3">
-        <v>0.1</v>
+        <v>440</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G47" s="3">
-        <v>0.08</v>
+        <v>352</v>
       </c>
       <c r="H47" s="3">
-        <v>0.1</v>
+        <v>440</v>
       </c>
       <c r="I47" s="3">
-        <v>0.12</v>
+        <v>528</v>
       </c>
       <c r="J47" s="3"/>
       <c r="K47" s="3" t="s">
@@ -2492,64 +2489,64 @@
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" s="3" t="s">
-        <v>116</v>
+        <v>135</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E48" s="3">
-        <v>440</v>
+        <v>2.82</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G48" s="3">
-        <v>352</v>
+        <v>2.2559999999999998</v>
       </c>
       <c r="H48" s="3">
-        <v>440</v>
+        <v>2.82</v>
       </c>
       <c r="I48" s="3">
-        <v>528</v>
+        <v>3.3839999999999999</v>
       </c>
       <c r="J48" s="3"/>
       <c r="K48" s="3" t="s">
-        <v>98</v>
+        <v>73</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C49" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E49" s="3">
-        <v>2.82</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G49" s="3">
-        <v>2.2559999999999998</v>
+        <v>0.01</v>
       </c>
       <c r="H49" s="3">
-        <v>2.82</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="I49" s="3">
-        <v>3.3839999999999999</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="J49" s="3"/>
       <c r="K49" s="3" t="s">
@@ -2558,64 +2555,64 @@
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" s="3" t="s">
-        <v>138</v>
+        <v>115</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E50" s="3">
-        <v>1.2500000000000001E-2</v>
+        <v>3.4000000000000002E-2</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G50" s="3">
-        <v>0.01</v>
+        <v>2.7199999999999998E-2</v>
       </c>
       <c r="H50" s="3">
-        <v>1.2500000000000001E-2</v>
+        <v>3.4000000000000002E-2</v>
       </c>
       <c r="I50" s="3">
-        <v>1.4999999999999999E-2</v>
+        <v>4.0800000000000003E-2</v>
       </c>
       <c r="J50" s="3"/>
       <c r="K50" s="3" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E51" s="3">
-        <v>3.4000000000000002E-2</v>
+        <v>5.7000000000000002E-2</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G51" s="3">
-        <v>2.7199999999999998E-2</v>
+        <v>4.5600000000000002E-2</v>
       </c>
       <c r="H51" s="3">
-        <v>3.4000000000000002E-2</v>
+        <v>5.7000000000000002E-2</v>
       </c>
       <c r="I51" s="3">
-        <v>4.0800000000000003E-2</v>
+        <v>6.8400000000000002E-2</v>
       </c>
       <c r="J51" s="3"/>
       <c r="K51" s="3" t="s">
@@ -2624,64 +2621,64 @@
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" s="3" t="s">
-        <v>118</v>
+        <v>137</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E52" s="3">
-        <v>5.7000000000000002E-2</v>
+        <v>1.2030000000000001</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G52" s="3">
-        <v>4.5600000000000002E-2</v>
+        <v>0.96240000000000003</v>
       </c>
       <c r="H52" s="3">
-        <v>5.7000000000000002E-2</v>
+        <v>1.2030000000000001</v>
       </c>
       <c r="I52" s="3">
-        <v>6.8400000000000002E-2</v>
+        <v>1.4436</v>
       </c>
       <c r="J52" s="3"/>
       <c r="K52" s="3" t="s">
-        <v>100</v>
+        <v>75</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C53" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E53" s="3">
-        <v>1.2030000000000001</v>
+        <v>0.04</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G53" s="3">
-        <v>0.96240000000000003</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H53" s="3">
-        <v>1.2030000000000001</v>
+        <v>0.04</v>
       </c>
       <c r="I53" s="3">
-        <v>1.4436</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J53" s="3"/>
       <c r="K53" s="3" t="s">
@@ -2690,31 +2687,31 @@
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C54" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E54" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G54" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="H54" s="3">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="I54" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="J54" s="3"/>
       <c r="K54" s="3" t="s">
@@ -2723,31 +2720,31 @@
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C55" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E55" s="3">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G55" s="3">
-        <v>9.6000000000000002E-2</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H55" s="3">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="I55" s="3">
-        <v>0.14399999999999999</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J55" s="3"/>
       <c r="K55" s="3" t="s">
@@ -2756,97 +2753,97 @@
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
-        <v>142</v>
+        <v>117</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C56" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E56" s="3">
-        <v>0.04</v>
+        <v>1.01E-2</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G56" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>8.0800000000000004E-3</v>
       </c>
       <c r="H56" s="3">
-        <v>0.04</v>
+        <v>1.01E-2</v>
       </c>
       <c r="I56" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>1.21199999999999E-2</v>
       </c>
       <c r="J56" s="3"/>
       <c r="K56" s="3" t="s">
-        <v>79</v>
+        <v>100</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" s="3" t="s">
-        <v>119</v>
+        <v>141</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C57" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E57" s="3">
-        <v>1.01E-2</v>
+        <v>0.58899999999999997</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G57" s="3">
-        <v>8.0800000000000004E-3</v>
+        <v>0.47120000000000001</v>
       </c>
       <c r="H57" s="3">
-        <v>1.01E-2</v>
+        <v>0.58899999999999997</v>
       </c>
       <c r="I57" s="3">
-        <v>1.21199999999999E-2</v>
+        <v>0.70679999999999998</v>
       </c>
       <c r="J57" s="3"/>
       <c r="K57" s="3" t="s">
-        <v>101</v>
+        <v>79</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C58" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E58" s="3">
-        <v>0.58899999999999997</v>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G58" s="3">
-        <v>0.47120000000000001</v>
+        <v>6.4000000000000003E-3</v>
       </c>
       <c r="H58" s="3">
-        <v>0.58899999999999997</v>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="I58" s="3">
-        <v>0.70679999999999998</v>
+        <v>9.5999999999999992E-3</v>
       </c>
       <c r="J58" s="3"/>
       <c r="K58" s="3" t="s">
@@ -2855,130 +2852,130 @@
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" s="3" t="s">
-        <v>144</v>
+        <v>118</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C59" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="E59" s="3">
-        <v>8.0000000000000002E-3</v>
+        <v>67</v>
+      </c>
+      <c r="E59" s="5">
+        <v>9.9999999999999995E-7</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="G59" s="3">
-        <v>6.4000000000000003E-3</v>
-      </c>
-      <c r="H59" s="3">
-        <v>8.0000000000000002E-3</v>
-      </c>
-      <c r="I59" s="3">
-        <v>9.5999999999999992E-3</v>
+        <v>66</v>
+      </c>
+      <c r="G59" s="5">
+        <v>7.9999999999999996E-7</v>
+      </c>
+      <c r="H59" s="5">
+        <v>9.9999999999999995E-7</v>
+      </c>
+      <c r="I59" s="5">
+        <v>1.1999999999999999E-6</v>
       </c>
       <c r="J59" s="3"/>
       <c r="K59" s="3" t="s">
-        <v>81</v>
+        <v>101</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" s="3" t="s">
-        <v>120</v>
+        <v>143</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C60" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E60" s="5">
-        <v>9.9999999999999995E-7</v>
+        <v>65</v>
+      </c>
+      <c r="E60" s="3">
+        <v>7.51E-2</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="G60" s="5">
-        <v>7.9999999999999996E-7</v>
-      </c>
-      <c r="H60" s="5">
-        <v>9.9999999999999995E-7</v>
-      </c>
-      <c r="I60" s="5">
-        <v>1.1999999999999999E-6</v>
+        <v>66</v>
+      </c>
+      <c r="G60" s="3">
+        <v>6.0080000000000001E-2</v>
+      </c>
+      <c r="H60" s="3">
+        <v>7.51E-2</v>
+      </c>
+      <c r="I60" s="3">
+        <v>9.0119999999999895E-2</v>
       </c>
       <c r="J60" s="3"/>
       <c r="K60" s="3" t="s">
-        <v>102</v>
+        <v>81</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
-        <v>145</v>
+        <v>119</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C61" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E61" s="3">
-        <v>7.51E-2</v>
+        <v>13</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G61" s="3">
-        <v>6.0080000000000001E-2</v>
+        <v>10.4</v>
       </c>
       <c r="H61" s="3">
-        <v>7.51E-2</v>
+        <v>13</v>
       </c>
       <c r="I61" s="3">
-        <v>9.0119999999999895E-2</v>
+        <v>15.6</v>
       </c>
       <c r="J61" s="3"/>
       <c r="K61" s="3" t="s">
-        <v>82</v>
+        <v>102</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C62" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E62" s="3">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G62" s="3">
-        <v>10.4</v>
+        <v>20</v>
       </c>
       <c r="H62" s="3">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="I62" s="3">
-        <v>15.6</v>
+        <v>30</v>
       </c>
       <c r="J62" s="3"/>
       <c r="K62" s="3" t="s">
@@ -2987,40 +2984,40 @@
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" s="3" t="s">
-        <v>122</v>
+        <v>144</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C63" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E63" s="3">
-        <v>25</v>
+        <v>3.9899999999999996E-3</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G63" s="3">
-        <v>20</v>
+        <v>3.192E-3</v>
       </c>
       <c r="H63" s="3">
-        <v>25</v>
+        <v>3.9899999999999996E-3</v>
       </c>
       <c r="I63" s="3">
-        <v>30</v>
+        <v>4.7879999999999997E-3</v>
       </c>
       <c r="J63" s="3"/>
       <c r="K63" s="3" t="s">
-        <v>104</v>
+        <v>82</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A64" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B64" s="3" t="s">
         <v>156</v>
@@ -3029,22 +3026,22 @@
         <v>21</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E64" s="3">
-        <v>3.9899999999999996E-3</v>
+        <v>0.06</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G64" s="3">
-        <v>3.192E-3</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="H64" s="3">
-        <v>3.9899999999999996E-3</v>
+        <v>0.06</v>
       </c>
       <c r="I64" s="3">
-        <v>4.7879999999999997E-3</v>
+        <v>7.1999999999999995E-2</v>
       </c>
       <c r="J64" s="3"/>
       <c r="K64" s="3" t="s">
@@ -3053,68 +3050,35 @@
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A65" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C65" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E65" s="3">
-        <v>0.06</v>
+        <v>0.02</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G65" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>1.6E-2</v>
       </c>
       <c r="H65" s="3">
-        <v>0.06</v>
+        <v>0.02</v>
       </c>
       <c r="I65" s="3">
-        <v>7.1999999999999995E-2</v>
+        <v>2.4E-2</v>
       </c>
       <c r="J65" s="3"/>
       <c r="K65" s="3" t="s">
         <v>84</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A66" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="B66" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="C66" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D66" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="E66" s="3">
-        <v>0.02</v>
-      </c>
-      <c r="F66" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="G66" s="3">
-        <v>1.6E-2</v>
-      </c>
-      <c r="H66" s="3">
-        <v>0.02</v>
-      </c>
-      <c r="I66" s="3">
-        <v>2.4E-2</v>
-      </c>
-      <c r="J66" s="3"/>
-      <c r="K66" s="3" t="s">
-        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix aeration-related bugs; add new ferm args; plot updates
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saran\Documents\Academia\repository_clones\Bioindustrial-Park\biorefineries\isobutanol\analyses\full\parameter_distributions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38C5CEFF-4B82-48F3-94B3-0E17AD8402FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D65BB55-3593-4ECE-8D2D-1A6E07AF64EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6100" yWindow="2720" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -912,7 +912,7 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="40.81640625" customWidth="1"/>
-    <col min="2" max="2" width="20.6328125" customWidth="1"/>
+    <col min="2" max="2" width="16.7265625" customWidth="1"/>
     <col min="4" max="4" width="12.1796875" customWidth="1"/>
     <col min="6" max="6" width="14.453125" customWidth="1"/>
     <col min="10" max="10" width="10.6328125" customWidth="1"/>
@@ -1307,14 +1307,16 @@
         <v>27</v>
       </c>
       <c r="G12" s="4">
-        <v>0.95</v>
+        <f t="shared" si="0"/>
+        <v>1.1919999999999999</v>
       </c>
       <c r="H12" s="4">
         <f>E12</f>
         <v>1.49</v>
       </c>
       <c r="I12" s="4">
-        <v>1.7250000000000001</v>
+        <f>1.2*E12</f>
+        <v>1.788</v>
       </c>
       <c r="J12" s="4"/>
       <c r="K12" s="4" t="s">

</xml_diff>

<commit_message>
rollback corn updates for isobutanol compatibility; minor isobutanol updates
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saran\Documents\Academia\repository_clones\Bioindustrial-Park\biorefineries\isobutanol\analyses\full\parameter_distributions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D65BB55-3593-4ECE-8D2D-1A6E07AF64EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6EDC3A7-2A4F-4EA9-B5B1-0964BDF6A7DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="2490" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="166">
   <si>
     <t>Parameter name</t>
   </si>
@@ -512,15 +512,9 @@
     <t>Kinetics: Acetaldehyde compartment degradation</t>
   </si>
   <si>
-    <t>V514.isobutanol_price = x</t>
-  </si>
-  <si>
     <t>DDGS.price =x</t>
   </si>
   <si>
-    <t>makeup_isopentyl_acetate.price = x</t>
-  </si>
-  <si>
     <t>Feedstock starch content</t>
   </si>
   <si>
@@ -530,9 +524,6 @@
     <t>feedstock.imass['Starch'] =x * feedstock.imass['Water']</t>
   </si>
   <si>
-    <t>Isopentyl acetate unit price</t>
-  </si>
-  <si>
     <t>Aeration rate safety factor</t>
   </si>
   <si>
@@ -543,9 +534,6 @@
   </si>
   <si>
     <t>DDGS unit price (sale)</t>
-  </si>
-  <si>
-    <t>Isobutanol selling unit price (sale)</t>
   </si>
 </sst>
 </file>
@@ -908,7 +896,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K65"/>
+  <dimension ref="A1:K63"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="40.81640625" customWidth="1"/>
@@ -1109,12 +1097,12 @@
         <v>18</v>
       </c>
       <c r="G6" s="4">
-        <f t="shared" ref="G6:G13" si="0">E6*0.8</f>
+        <f t="shared" ref="G6:G11" si="0">E6*0.8</f>
         <v>0.35920000000000002</v>
       </c>
       <c r="H6" s="4"/>
       <c r="I6" s="4">
-        <f t="shared" ref="I6:I13" si="1">1.2*E6</f>
+        <f t="shared" ref="I6:I11" si="1">1.2*E6</f>
         <v>0.53879999999999995</v>
       </c>
       <c r="J6" s="4"/>
@@ -1256,7 +1244,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>7</v>
@@ -1284,389 +1272,386 @@
       </c>
       <c r="J11" s="4"/>
       <c r="K11" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A12" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="B12" s="4" t="s">
+      <c r="A12" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="4">
-        <v>1.49</v>
-      </c>
-      <c r="F12" s="4" t="s">
+      <c r="E12" s="6">
+        <v>0.28599999999999998</v>
+      </c>
+      <c r="F12" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G12" s="4">
-        <f t="shared" si="0"/>
-        <v>1.1919999999999999</v>
-      </c>
-      <c r="H12" s="4">
-        <f>E12</f>
-        <v>1.49</v>
-      </c>
-      <c r="I12" s="4">
-        <f>1.2*E12</f>
-        <v>1.788</v>
-      </c>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4" t="s">
-        <v>158</v>
+      <c r="G12" s="6">
+        <v>0.17499999999999999</v>
+      </c>
+      <c r="H12" s="6">
+        <v>0.28599999999999998</v>
+      </c>
+      <c r="I12" s="6">
+        <v>0.315</v>
+      </c>
+      <c r="J12" s="6"/>
+      <c r="K12" s="6" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A13" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="B13" s="4" t="s">
+      <c r="A13" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E13" s="4">
-        <v>3.2</v>
-      </c>
-      <c r="F13" s="4" t="s">
+      <c r="E13" s="6">
+        <v>0.10355</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G13" s="6">
+        <f>E13*0.9</f>
+        <v>9.3195E-2</v>
+      </c>
+      <c r="H13" s="6">
+        <f>E13</f>
+        <v>0.10355</v>
+      </c>
+      <c r="I13" s="6">
+        <f>E13*1.1</f>
+        <v>0.11390500000000001</v>
+      </c>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14" s="3">
+        <v>0.21</v>
+      </c>
+      <c r="F14" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G13" s="4">
-        <f t="shared" si="0"/>
-        <v>2.5600000000000005</v>
-      </c>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4">
-        <f t="shared" si="1"/>
-        <v>3.84</v>
-      </c>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A14" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="6" t="s">
+      <c r="G14" s="3">
+        <v>0.15</v>
+      </c>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A15" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C15" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D14" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E14" s="6">
-        <v>0.28599999999999998</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="G14" s="6">
-        <v>0.17499999999999999</v>
-      </c>
-      <c r="H14" s="6">
-        <v>0.28599999999999998</v>
-      </c>
-      <c r="I14" s="6">
-        <v>0.315</v>
-      </c>
-      <c r="J14" s="6"/>
-      <c r="K14" s="6" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A15" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E15" s="6">
-        <v>0.10355</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="G15" s="6">
-        <f>E15*0.9</f>
-        <v>9.3195E-2</v>
-      </c>
-      <c r="H15" s="6">
-        <f>E15</f>
-        <v>0.10355</v>
-      </c>
-      <c r="I15" s="6">
-        <f>E15*1.1</f>
-        <v>0.11390500000000001</v>
-      </c>
-      <c r="J15" s="6"/>
-      <c r="K15" s="6" t="s">
-        <v>86</v>
+      <c r="D15" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="3">
+        <v>0.15</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" s="3">
+        <f>0.8*E15</f>
+        <v>0.12</v>
+      </c>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3">
+        <f>1.2*E15</f>
+        <v>0.18</v>
+      </c>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>31</v>
+        <v>159</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>7</v>
+        <v>39</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>8</v>
+        <v>160</v>
       </c>
       <c r="E16" s="3">
-        <v>0.21</v>
+        <v>4.08</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="G16" s="3">
-        <v>0.15</v>
-      </c>
-      <c r="H16" s="3"/>
+        <f>0.8*H16</f>
+        <v>3.2640000000000002</v>
+      </c>
+      <c r="H16" s="3">
+        <f>E16</f>
+        <v>4.08</v>
+      </c>
       <c r="I16" s="3">
-        <v>0.28000000000000003</v>
+        <f>1.2*H16</f>
+        <v>4.8959999999999999</v>
       </c>
       <c r="J16" s="3"/>
       <c r="K16" s="3" t="s">
-        <v>34</v>
+        <v>161</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>7</v>
+        <v>39</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="E17" s="3">
-        <v>0.15</v>
+        <v>56972</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="G17" s="3">
-        <f>0.8*E17</f>
-        <v>0.12</v>
-      </c>
-      <c r="H17" s="3"/>
+        <f>0.8*H17</f>
+        <v>45577.600000000006</v>
+      </c>
+      <c r="H17" s="3">
+        <f>E17</f>
+        <v>56972</v>
+      </c>
       <c r="I17" s="3">
-        <f>1.2*E17</f>
-        <v>0.18</v>
+        <f>1.2*H17</f>
+        <v>68366.399999999994</v>
       </c>
       <c r="J17" s="3"/>
       <c r="K17" s="3" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>39</v>
+        <v>163</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>162</v>
+        <v>12</v>
       </c>
       <c r="E18" s="3">
-        <v>4.08</v>
+        <v>2</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="G18" s="3">
-        <f>0.8*H18</f>
-        <v>3.2640000000000002</v>
-      </c>
-      <c r="H18" s="3">
-        <f>E18</f>
-        <v>4.08</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H18" s="3"/>
       <c r="I18" s="3">
-        <f>1.2*H18</f>
-        <v>4.8959999999999999</v>
+        <v>3</v>
       </c>
       <c r="J18" s="3"/>
       <c r="K18" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>39</v>
+        <v>13</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="E19" s="3">
-        <v>56972</v>
+        <v>156</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>27</v>
       </c>
       <c r="G19" s="3">
-        <f>0.8*H19</f>
-        <v>45577.600000000006</v>
+        <f>E19*0.8</f>
+        <v>124.80000000000001</v>
       </c>
       <c r="H19" s="3">
         <f>E19</f>
-        <v>56972</v>
+        <v>156</v>
       </c>
       <c r="I19" s="3">
-        <f>1.2*H19</f>
-        <v>68366.399999999994</v>
+        <f>E19*1.2</f>
+        <v>187.2</v>
       </c>
       <c r="J19" s="3"/>
       <c r="K19" s="3" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>165</v>
+        <v>53</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>166</v>
+        <v>13</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E20" s="3">
-        <v>2</v>
+        <v>156</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="G20" s="3">
-        <v>1</v>
-      </c>
-      <c r="H20" s="3"/>
+        <f>E20*0.8</f>
+        <v>124.80000000000001</v>
+      </c>
+      <c r="H20" s="3">
+        <f>E20</f>
+        <v>156</v>
+      </c>
       <c r="I20" s="3">
-        <v>3</v>
+        <f>E20*1.2</f>
+        <v>187.2</v>
       </c>
       <c r="J20" s="3"/>
       <c r="K20" s="3" t="s">
-        <v>167</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>52</v>
+        <v>121</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>13</v>
+        <v>147</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>14</v>
+        <v>65</v>
       </c>
       <c r="E21" s="3">
-        <v>156</v>
+        <v>1.43</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>27</v>
+        <v>66</v>
       </c>
       <c r="G21" s="3">
-        <f>E21*0.8</f>
-        <v>124.80000000000001</v>
+        <v>1.1439999999999999</v>
       </c>
       <c r="H21" s="3">
-        <f>E21</f>
-        <v>156</v>
+        <v>1.43</v>
       </c>
       <c r="I21" s="3">
-        <f>E21*1.2</f>
-        <v>187.2</v>
+        <v>1.716</v>
       </c>
       <c r="J21" s="3"/>
       <c r="K21" s="3" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>53</v>
+        <v>104</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>13</v>
+        <v>147</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>14</v>
+        <v>67</v>
       </c>
       <c r="E22" s="3">
-        <v>156</v>
+        <v>0.94</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>27</v>
+        <v>66</v>
       </c>
       <c r="G22" s="3">
-        <f>E22*0.8</f>
-        <v>124.80000000000001</v>
+        <v>0.752</v>
       </c>
       <c r="H22" s="3">
-        <f>E22</f>
-        <v>156</v>
+        <v>0.94</v>
       </c>
       <c r="I22" s="3">
-        <f>E22*1.2</f>
-        <v>187.2</v>
+        <v>1.1279999999999999</v>
       </c>
       <c r="J22" s="3"/>
       <c r="K22" s="3" t="s">
-        <v>55</v>
+        <v>87</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>147</v>
@@ -1678,28 +1663,28 @@
         <v>65</v>
       </c>
       <c r="E23" s="3">
-        <v>1.43</v>
+        <v>0.58399999999999996</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G23" s="3">
-        <v>1.1439999999999999</v>
+        <v>0.4672</v>
       </c>
       <c r="H23" s="3">
-        <v>1.43</v>
+        <v>0.58399999999999996</v>
       </c>
       <c r="I23" s="3">
-        <v>1.716</v>
+        <v>0.70079999999999998</v>
       </c>
       <c r="J23" s="3"/>
       <c r="K23" s="3" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>147</v>
@@ -1711,28 +1696,28 @@
         <v>67</v>
       </c>
       <c r="E24" s="3">
-        <v>0.94</v>
+        <v>1.1599999999999999E-2</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G24" s="3">
-        <v>0.752</v>
+        <v>9.2800000000000001E-3</v>
       </c>
       <c r="H24" s="3">
-        <v>0.94</v>
+        <v>1.1599999999999999E-2</v>
       </c>
       <c r="I24" s="3">
-        <v>1.1279999999999999</v>
+        <v>1.3919999999999899E-2</v>
       </c>
       <c r="J24" s="3"/>
       <c r="K24" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>147</v>
@@ -1744,28 +1729,28 @@
         <v>65</v>
       </c>
       <c r="E25" s="3">
-        <v>0.58399999999999996</v>
+        <v>47.1</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G25" s="3">
-        <v>0.4672</v>
+        <v>37.68</v>
       </c>
       <c r="H25" s="3">
-        <v>0.58399999999999996</v>
+        <v>47.1</v>
       </c>
       <c r="I25" s="3">
-        <v>0.70079999999999998</v>
+        <v>56.52</v>
       </c>
       <c r="J25" s="3"/>
       <c r="K25" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>147</v>
@@ -1777,28 +1762,28 @@
         <v>67</v>
       </c>
       <c r="E26" s="3">
-        <v>1.1599999999999999E-2</v>
+        <v>14.2</v>
       </c>
       <c r="F26" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G26" s="3">
-        <v>9.2800000000000001E-3</v>
+        <v>11.36</v>
       </c>
       <c r="H26" s="3">
-        <v>1.1599999999999999E-2</v>
+        <v>14.2</v>
       </c>
       <c r="I26" s="3">
-        <v>1.3919999999999899E-2</v>
+        <v>17.04</v>
       </c>
       <c r="J26" s="3"/>
       <c r="K26" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>123</v>
+        <v>107</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>147</v>
@@ -1807,31 +1792,31 @@
         <v>21</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E27" s="3">
-        <v>47.1</v>
+        <v>0.12</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G27" s="3">
-        <v>37.68</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="H27" s="3">
-        <v>47.1</v>
+        <v>0.12</v>
       </c>
       <c r="I27" s="3">
-        <v>56.52</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="J27" s="3"/>
       <c r="K27" s="3" t="s">
-        <v>57</v>
+        <v>90</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>106</v>
+        <v>124</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>147</v>
@@ -1840,31 +1825,31 @@
         <v>21</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E28" s="3">
-        <v>14.2</v>
+        <v>0.04</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G28" s="3">
-        <v>11.36</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H28" s="3">
-        <v>14.2</v>
+        <v>0.04</v>
       </c>
       <c r="I28" s="3">
-        <v>17.04</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J28" s="3"/>
       <c r="K28" s="3" t="s">
-        <v>89</v>
+        <v>59</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>107</v>
+        <v>125</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>147</v>
@@ -1873,7 +1858,7 @@
         <v>21</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E29" s="3">
         <v>0.12</v>
@@ -1892,12 +1877,12 @@
       </c>
       <c r="J29" s="3"/>
       <c r="K29" s="3" t="s">
-        <v>90</v>
+        <v>60</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>147</v>
@@ -1925,15 +1910,15 @@
       </c>
       <c r="J30" s="3"/>
       <c r="K30" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>21</v>
@@ -1942,61 +1927,61 @@
         <v>65</v>
       </c>
       <c r="E31" s="3">
-        <v>0.12</v>
+        <v>0.501</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G31" s="3">
-        <v>9.6000000000000002E-2</v>
+        <v>0.40079999999999999</v>
       </c>
       <c r="H31" s="3">
-        <v>0.12</v>
+        <v>0.501</v>
       </c>
       <c r="I31" s="3">
-        <v>0.14399999999999999</v>
+        <v>0.60119999999999996</v>
       </c>
       <c r="J31" s="3"/>
       <c r="K31" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
-        <v>126</v>
+        <v>108</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="E32" s="3">
-        <v>0.04</v>
+        <v>67</v>
+      </c>
+      <c r="E32" s="5">
+        <v>2.0000000000000002E-5</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="G32" s="3">
-        <v>3.2000000000000001E-2</v>
-      </c>
-      <c r="H32" s="3">
-        <v>0.04</v>
-      </c>
-      <c r="I32" s="3">
-        <v>4.8000000000000001E-2</v>
+      <c r="G32" s="5">
+        <v>1.5999999999999999E-5</v>
+      </c>
+      <c r="H32" s="5">
+        <v>2.0000000000000002E-5</v>
+      </c>
+      <c r="I32" s="5">
+        <v>2.4000000000000001E-5</v>
       </c>
       <c r="J32" s="3"/>
       <c r="K32" s="3" t="s">
-        <v>61</v>
+        <v>91</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
-        <v>127</v>
+        <v>109</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>148</v>
@@ -2005,67 +1990,67 @@
         <v>21</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E33" s="3">
-        <v>0.501</v>
+        <v>0.10100000000000001</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G33" s="3">
-        <v>0.40079999999999999</v>
+        <v>8.0799999999999997E-2</v>
       </c>
       <c r="H33" s="3">
-        <v>0.501</v>
+        <v>0.10100000000000001</v>
       </c>
       <c r="I33" s="3">
-        <v>0.60119999999999996</v>
+        <v>0.1212</v>
       </c>
       <c r="J33" s="3"/>
       <c r="K33" s="3" t="s">
-        <v>56</v>
+        <v>92</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="E34" s="5">
-        <v>2.0000000000000002E-5</v>
+        <v>65</v>
+      </c>
+      <c r="E34" s="3">
+        <v>5.81</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="G34" s="5">
-        <v>1.5999999999999999E-5</v>
-      </c>
-      <c r="H34" s="5">
-        <v>2.0000000000000002E-5</v>
-      </c>
-      <c r="I34" s="5">
-        <v>2.4000000000000001E-5</v>
+      <c r="G34" s="3">
+        <v>4.6479999999999997</v>
+      </c>
+      <c r="H34" s="3">
+        <v>5.81</v>
+      </c>
+      <c r="I34" s="3">
+        <v>6.9719999999999898</v>
       </c>
       <c r="J34" s="3"/>
       <c r="K34" s="3" t="s">
-        <v>91</v>
+        <v>63</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>21</v>
@@ -2073,32 +2058,32 @@
       <c r="D35" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E35" s="3">
-        <v>0.10100000000000001</v>
+      <c r="E35" s="5">
+        <v>4.9999999999999998E-7</v>
       </c>
       <c r="F35" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="G35" s="3">
-        <v>8.0799999999999997E-2</v>
-      </c>
-      <c r="H35" s="3">
-        <v>0.10100000000000001</v>
-      </c>
-      <c r="I35" s="3">
-        <v>0.1212</v>
+      <c r="G35" s="5">
+        <v>3.9999999999999998E-7</v>
+      </c>
+      <c r="H35" s="5">
+        <v>4.9999999999999998E-7</v>
+      </c>
+      <c r="I35" s="5">
+        <v>5.9999999999999997E-7</v>
       </c>
       <c r="J35" s="3"/>
       <c r="K35" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>21</v>
@@ -2107,61 +2092,61 @@
         <v>65</v>
       </c>
       <c r="E36" s="3">
-        <v>5.81</v>
+        <v>4.8</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G36" s="3">
-        <v>4.6479999999999997</v>
+        <v>3.84</v>
       </c>
       <c r="H36" s="3">
-        <v>5.81</v>
+        <v>4.8</v>
       </c>
       <c r="I36" s="3">
-        <v>6.9719999999999898</v>
+        <v>5.76</v>
       </c>
       <c r="J36" s="3"/>
       <c r="K36" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="E37" s="5">
-        <v>4.9999999999999998E-7</v>
+        <v>65</v>
+      </c>
+      <c r="E37" s="3">
+        <v>0.04</v>
       </c>
       <c r="F37" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="G37" s="5">
-        <v>3.9999999999999998E-7</v>
-      </c>
-      <c r="H37" s="5">
-        <v>4.9999999999999998E-7</v>
-      </c>
-      <c r="I37" s="5">
-        <v>5.9999999999999997E-7</v>
+      <c r="G37" s="3">
+        <v>3.2000000000000001E-2</v>
+      </c>
+      <c r="H37" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="I37" s="3">
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J37" s="3"/>
       <c r="K37" s="3" t="s">
-        <v>93</v>
+        <v>68</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>150</v>
@@ -2173,28 +2158,28 @@
         <v>65</v>
       </c>
       <c r="E38" s="3">
-        <v>4.8</v>
+        <v>0.12</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G38" s="3">
-        <v>3.84</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="H38" s="3">
-        <v>4.8</v>
+        <v>0.12</v>
       </c>
       <c r="I38" s="3">
-        <v>5.76</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="J38" s="3"/>
       <c r="K38" s="3" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>150</v>
@@ -2222,12 +2207,12 @@
       </c>
       <c r="J39" s="3"/>
       <c r="K39" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
-        <v>131</v>
+        <v>111</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>150</v>
@@ -2236,34 +2221,34 @@
         <v>21</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E40" s="3">
-        <v>0.12</v>
+        <v>2.6400000000000002E-4</v>
       </c>
       <c r="F40" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G40" s="3">
-        <v>9.6000000000000002E-2</v>
+        <v>2.1120000000000001E-4</v>
       </c>
       <c r="H40" s="3">
-        <v>0.12</v>
+        <v>2.6400000000000002E-4</v>
       </c>
       <c r="I40" s="3">
-        <v>0.14399999999999999</v>
+        <v>3.168E-4</v>
       </c>
       <c r="J40" s="3"/>
       <c r="K40" s="3" t="s">
-        <v>69</v>
+        <v>94</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>21</v>
@@ -2272,31 +2257,31 @@
         <v>65</v>
       </c>
       <c r="E41" s="3">
-        <v>0.04</v>
+        <v>1.04E-2</v>
       </c>
       <c r="F41" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G41" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>8.3199999999999993E-3</v>
       </c>
       <c r="H41" s="3">
-        <v>0.04</v>
+        <v>1.04E-2</v>
       </c>
       <c r="I41" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>1.248E-2</v>
       </c>
       <c r="J41" s="3"/>
       <c r="K41" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>21</v>
@@ -2305,28 +2290,28 @@
         <v>67</v>
       </c>
       <c r="E42" s="3">
-        <v>2.6400000000000002E-4</v>
+        <v>1.0200000000000001E-2</v>
       </c>
       <c r="F42" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G42" s="3">
-        <v>2.1120000000000001E-4</v>
+        <v>8.1600000000000006E-3</v>
       </c>
       <c r="H42" s="3">
-        <v>2.6400000000000002E-4</v>
+        <v>1.0200000000000001E-2</v>
       </c>
       <c r="I42" s="3">
-        <v>3.168E-4</v>
+        <v>1.2239999999999999E-2</v>
       </c>
       <c r="J42" s="3"/>
       <c r="K42" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>155</v>
@@ -2338,28 +2323,28 @@
         <v>65</v>
       </c>
       <c r="E43" s="3">
-        <v>1.04E-2</v>
+        <v>0.77500000000000002</v>
       </c>
       <c r="F43" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G43" s="3">
-        <v>8.3199999999999993E-3</v>
+        <v>0.62</v>
       </c>
       <c r="H43" s="3">
-        <v>1.04E-2</v>
+        <v>0.77500000000000002</v>
       </c>
       <c r="I43" s="3">
-        <v>1.248E-2</v>
+        <v>0.92999999999999905</v>
       </c>
       <c r="J43" s="3"/>
       <c r="K43" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>155</v>
@@ -2371,28 +2356,28 @@
         <v>67</v>
       </c>
       <c r="E44" s="3">
-        <v>1.0200000000000001E-2</v>
+        <v>0.1</v>
       </c>
       <c r="F44" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G44" s="3">
-        <v>8.1600000000000006E-3</v>
+        <v>0.08</v>
       </c>
       <c r="H44" s="3">
-        <v>1.0200000000000001E-2</v>
+        <v>0.1</v>
       </c>
       <c r="I44" s="3">
-        <v>1.2239999999999999E-2</v>
+        <v>0.12</v>
       </c>
       <c r="J44" s="3"/>
       <c r="K44" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" s="3" t="s">
-        <v>134</v>
+        <v>114</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>155</v>
@@ -2401,97 +2386,97 @@
         <v>21</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E45" s="3">
-        <v>0.77500000000000002</v>
+        <v>440</v>
       </c>
       <c r="F45" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G45" s="3">
-        <v>0.62</v>
+        <v>352</v>
       </c>
       <c r="H45" s="3">
-        <v>0.77500000000000002</v>
+        <v>440</v>
       </c>
       <c r="I45" s="3">
-        <v>0.92999999999999905</v>
+        <v>528</v>
       </c>
       <c r="J45" s="3"/>
       <c r="K45" s="3" t="s">
-        <v>72</v>
+        <v>97</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
-        <v>113</v>
+        <v>135</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E46" s="3">
-        <v>0.1</v>
+        <v>2.82</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G46" s="3">
-        <v>0.08</v>
+        <v>2.2559999999999998</v>
       </c>
       <c r="H46" s="3">
-        <v>0.1</v>
+        <v>2.82</v>
       </c>
       <c r="I46" s="3">
-        <v>0.12</v>
+        <v>3.3839999999999999</v>
       </c>
       <c r="J46" s="3"/>
       <c r="K46" s="3" t="s">
-        <v>96</v>
+        <v>73</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" s="3" t="s">
-        <v>114</v>
+        <v>136</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E47" s="3">
-        <v>440</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="F47" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G47" s="3">
-        <v>352</v>
+        <v>0.01</v>
       </c>
       <c r="H47" s="3">
-        <v>440</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="I47" s="3">
-        <v>528</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="J47" s="3"/>
       <c r="K47" s="3" t="s">
-        <v>97</v>
+        <v>74</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" s="3" t="s">
-        <v>135</v>
+        <v>115</v>
       </c>
       <c r="B48" s="3" t="s">
         <v>151</v>
@@ -2500,31 +2485,31 @@
         <v>21</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E48" s="3">
-        <v>2.82</v>
+        <v>3.4000000000000002E-2</v>
       </c>
       <c r="F48" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G48" s="3">
-        <v>2.2559999999999998</v>
+        <v>2.7199999999999998E-2</v>
       </c>
       <c r="H48" s="3">
-        <v>2.82</v>
+        <v>3.4000000000000002E-2</v>
       </c>
       <c r="I48" s="3">
-        <v>3.3839999999999999</v>
+        <v>4.0800000000000003E-2</v>
       </c>
       <c r="J48" s="3"/>
       <c r="K48" s="3" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" s="3" t="s">
-        <v>136</v>
+        <v>116</v>
       </c>
       <c r="B49" s="3" t="s">
         <v>151</v>
@@ -2533,97 +2518,97 @@
         <v>21</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E49" s="3">
-        <v>1.2500000000000001E-2</v>
+        <v>5.7000000000000002E-2</v>
       </c>
       <c r="F49" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G49" s="3">
-        <v>0.01</v>
+        <v>4.5600000000000002E-2</v>
       </c>
       <c r="H49" s="3">
-        <v>1.2500000000000001E-2</v>
+        <v>5.7000000000000002E-2</v>
       </c>
       <c r="I49" s="3">
-        <v>1.4999999999999999E-2</v>
+        <v>6.8400000000000002E-2</v>
       </c>
       <c r="J49" s="3"/>
       <c r="K49" s="3" t="s">
-        <v>74</v>
+        <v>99</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" s="3" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E50" s="3">
-        <v>3.4000000000000002E-2</v>
+        <v>1.2030000000000001</v>
       </c>
       <c r="F50" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G50" s="3">
-        <v>2.7199999999999998E-2</v>
+        <v>0.96240000000000003</v>
       </c>
       <c r="H50" s="3">
-        <v>3.4000000000000002E-2</v>
+        <v>1.2030000000000001</v>
       </c>
       <c r="I50" s="3">
-        <v>4.0800000000000003E-2</v>
+        <v>1.4436</v>
       </c>
       <c r="J50" s="3"/>
       <c r="K50" s="3" t="s">
-        <v>98</v>
+        <v>75</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
-        <v>116</v>
+        <v>138</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E51" s="3">
-        <v>5.7000000000000002E-2</v>
+        <v>0.04</v>
       </c>
       <c r="F51" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G51" s="3">
-        <v>4.5600000000000002E-2</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="H51" s="3">
-        <v>5.7000000000000002E-2</v>
+        <v>0.04</v>
       </c>
       <c r="I51" s="3">
-        <v>6.8400000000000002E-2</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J51" s="3"/>
       <c r="K51" s="3" t="s">
-        <v>99</v>
+        <v>76</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B52" s="3" t="s">
         <v>152</v>
@@ -2635,28 +2620,28 @@
         <v>65</v>
       </c>
       <c r="E52" s="3">
-        <v>1.2030000000000001</v>
+        <v>0.12</v>
       </c>
       <c r="F52" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G52" s="3">
-        <v>0.96240000000000003</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="H52" s="3">
-        <v>1.2030000000000001</v>
+        <v>0.12</v>
       </c>
       <c r="I52" s="3">
-        <v>1.4436</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="J52" s="3"/>
       <c r="K52" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>152</v>
@@ -2684,12 +2669,12 @@
       </c>
       <c r="J53" s="3"/>
       <c r="K53" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" s="3" t="s">
-        <v>139</v>
+        <v>117</v>
       </c>
       <c r="B54" s="3" t="s">
         <v>152</v>
@@ -2698,34 +2683,34 @@
         <v>21</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E54" s="3">
-        <v>0.12</v>
+        <v>1.01E-2</v>
       </c>
       <c r="F54" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G54" s="3">
-        <v>9.6000000000000002E-2</v>
+        <v>8.0800000000000004E-3</v>
       </c>
       <c r="H54" s="3">
-        <v>0.12</v>
+        <v>1.01E-2</v>
       </c>
       <c r="I54" s="3">
-        <v>0.14399999999999999</v>
+        <v>1.21199999999999E-2</v>
       </c>
       <c r="J54" s="3"/>
       <c r="K54" s="3" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C55" s="3" t="s">
         <v>21</v>
@@ -2734,94 +2719,94 @@
         <v>65</v>
       </c>
       <c r="E55" s="3">
-        <v>0.04</v>
+        <v>0.58899999999999997</v>
       </c>
       <c r="F55" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G55" s="3">
-        <v>3.2000000000000001E-2</v>
+        <v>0.47120000000000001</v>
       </c>
       <c r="H55" s="3">
-        <v>0.04</v>
+        <v>0.58899999999999997</v>
       </c>
       <c r="I55" s="3">
-        <v>4.8000000000000001E-2</v>
+        <v>0.70679999999999998</v>
       </c>
       <c r="J55" s="3"/>
       <c r="K55" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
-        <v>117</v>
+        <v>142</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C56" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E56" s="3">
-        <v>1.01E-2</v>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="F56" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G56" s="3">
-        <v>8.0800000000000004E-3</v>
+        <v>6.4000000000000003E-3</v>
       </c>
       <c r="H56" s="3">
-        <v>1.01E-2</v>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="I56" s="3">
-        <v>1.21199999999999E-2</v>
+        <v>9.5999999999999992E-3</v>
       </c>
       <c r="J56" s="3"/>
       <c r="K56" s="3" t="s">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" s="3" t="s">
-        <v>141</v>
+        <v>118</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C57" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="E57" s="3">
-        <v>0.58899999999999997</v>
+        <v>67</v>
+      </c>
+      <c r="E57" s="5">
+        <v>9.9999999999999995E-7</v>
       </c>
       <c r="F57" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="G57" s="3">
-        <v>0.47120000000000001</v>
-      </c>
-      <c r="H57" s="3">
-        <v>0.58899999999999997</v>
-      </c>
-      <c r="I57" s="3">
-        <v>0.70679999999999998</v>
+      <c r="G57" s="5">
+        <v>7.9999999999999996E-7</v>
+      </c>
+      <c r="H57" s="5">
+        <v>9.9999999999999995E-7</v>
+      </c>
+      <c r="I57" s="5">
+        <v>1.1999999999999999E-6</v>
       </c>
       <c r="J57" s="3"/>
       <c r="K57" s="3" t="s">
-        <v>79</v>
+        <v>101</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B58" s="3" t="s">
         <v>154</v>
@@ -2833,28 +2818,28 @@
         <v>65</v>
       </c>
       <c r="E58" s="3">
-        <v>8.0000000000000002E-3</v>
+        <v>7.51E-2</v>
       </c>
       <c r="F58" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G58" s="3">
-        <v>6.4000000000000003E-3</v>
+        <v>6.0080000000000001E-2</v>
       </c>
       <c r="H58" s="3">
-        <v>8.0000000000000002E-3</v>
+        <v>7.51E-2</v>
       </c>
       <c r="I58" s="3">
-        <v>9.5999999999999992E-3</v>
+        <v>9.0119999999999895E-2</v>
       </c>
       <c r="J58" s="3"/>
       <c r="K58" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B59" s="3" t="s">
         <v>154</v>
@@ -2865,29 +2850,29 @@
       <c r="D59" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E59" s="5">
-        <v>9.9999999999999995E-7</v>
+      <c r="E59" s="3">
+        <v>13</v>
       </c>
       <c r="F59" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="G59" s="5">
-        <v>7.9999999999999996E-7</v>
-      </c>
-      <c r="H59" s="5">
-        <v>9.9999999999999995E-7</v>
-      </c>
-      <c r="I59" s="5">
-        <v>1.1999999999999999E-6</v>
+      <c r="G59" s="3">
+        <v>10.4</v>
+      </c>
+      <c r="H59" s="3">
+        <v>13</v>
+      </c>
+      <c r="I59" s="3">
+        <v>15.6</v>
       </c>
       <c r="J59" s="3"/>
       <c r="K59" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" s="3" t="s">
-        <v>143</v>
+        <v>120</v>
       </c>
       <c r="B60" s="3" t="s">
         <v>154</v>
@@ -2896,31 +2881,31 @@
         <v>21</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E60" s="3">
-        <v>7.51E-2</v>
+        <v>25</v>
       </c>
       <c r="F60" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G60" s="3">
-        <v>6.0080000000000001E-2</v>
+        <v>20</v>
       </c>
       <c r="H60" s="3">
-        <v>7.51E-2</v>
+        <v>25</v>
       </c>
       <c r="I60" s="3">
-        <v>9.0119999999999895E-2</v>
+        <v>30</v>
       </c>
       <c r="J60" s="3"/>
       <c r="K60" s="3" t="s">
-        <v>81</v>
+        <v>103</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
-        <v>119</v>
+        <v>144</v>
       </c>
       <c r="B61" s="3" t="s">
         <v>154</v>
@@ -2929,67 +2914,67 @@
         <v>21</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E61" s="3">
-        <v>13</v>
+        <v>3.9899999999999996E-3</v>
       </c>
       <c r="F61" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G61" s="3">
-        <v>10.4</v>
+        <v>3.192E-3</v>
       </c>
       <c r="H61" s="3">
-        <v>13</v>
+        <v>3.9899999999999996E-3</v>
       </c>
       <c r="I61" s="3">
-        <v>15.6</v>
+        <v>4.7879999999999997E-3</v>
       </c>
       <c r="J61" s="3"/>
       <c r="K61" s="3" t="s">
-        <v>102</v>
+        <v>82</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" s="3" t="s">
-        <v>120</v>
+        <v>145</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C62" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E62" s="3">
-        <v>25</v>
+        <v>0.06</v>
       </c>
       <c r="F62" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G62" s="3">
-        <v>20</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="H62" s="3">
-        <v>25</v>
+        <v>0.06</v>
       </c>
       <c r="I62" s="3">
-        <v>30</v>
+        <v>7.1999999999999995E-2</v>
       </c>
       <c r="J62" s="3"/>
       <c r="K62" s="3" t="s">
-        <v>103</v>
+        <v>83</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="C63" s="3" t="s">
         <v>21</v>
@@ -2998,88 +2983,22 @@
         <v>65</v>
       </c>
       <c r="E63" s="3">
-        <v>3.9899999999999996E-3</v>
+        <v>0.02</v>
       </c>
       <c r="F63" s="3" t="s">
         <v>66</v>
       </c>
       <c r="G63" s="3">
-        <v>3.192E-3</v>
+        <v>1.6E-2</v>
       </c>
       <c r="H63" s="3">
-        <v>3.9899999999999996E-3</v>
+        <v>0.02</v>
       </c>
       <c r="I63" s="3">
-        <v>4.7879999999999997E-3</v>
+        <v>2.4E-2</v>
       </c>
       <c r="J63" s="3"/>
       <c r="K63" s="3" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A64" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="B64" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="C64" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D64" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="E64" s="3">
-        <v>0.06</v>
-      </c>
-      <c r="F64" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="G64" s="3">
-        <v>4.8000000000000001E-2</v>
-      </c>
-      <c r="H64" s="3">
-        <v>0.06</v>
-      </c>
-      <c r="I64" s="3">
-        <v>7.1999999999999995E-2</v>
-      </c>
-      <c r="J64" s="3"/>
-      <c r="K64" s="3" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A65" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="B65" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="C65" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D65" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="E65" s="3">
-        <v>0.02</v>
-      </c>
-      <c r="F65" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="G65" s="3">
-        <v>1.6E-2</v>
-      </c>
-      <c r="H65" s="3">
-        <v>0.02</v>
-      </c>
-      <c r="I65" s="3">
-        <v>2.4E-2</v>
-      </c>
-      <c r="J65" s="3"/>
-      <c r="K65" s="3" t="s">
         <v>84</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: starch content load function
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saran\Documents\Academia\repository_clones\Bioindustrial-Park\biorefineries\isobutanol\analyses\full\parameter_distributions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6EDC3A7-2A4F-4EA9-B5B1-0964BDF6A7DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EEB212C-82B1-4CCC-BF55-6EB86BD9AD25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="2490" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -518,12 +518,6 @@
     <t>Feedstock starch content</t>
   </si>
   <si>
-    <t>kg/kg-water</t>
-  </si>
-  <si>
-    <t>feedstock.imass['Starch'] =x * feedstock.imass['Water']</t>
-  </si>
-  <si>
     <t>Aeration rate safety factor</t>
   </si>
   <si>
@@ -534,6 +528,12 @@
   </si>
   <si>
     <t>DDGS unit price (sale)</t>
+  </si>
+  <si>
+    <t>kg/dry-kg</t>
+  </si>
+  <si>
+    <t>fixed_F_mass = feedstock.F_mass; feedstock.imass['Starch'] = x * (fixed_F_mass - feedstock.imass['Water']); feedstock.F_mass = fixed_F_mass</t>
   </si>
 </sst>
 </file>
@@ -1244,7 +1244,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>7</v>
@@ -1419,29 +1419,29 @@
         <v>21</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="E16" s="3">
-        <v>4.08</v>
+        <v>0.72</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>27</v>
       </c>
       <c r="G16" s="3">
         <f>0.8*H16</f>
-        <v>3.2640000000000002</v>
+        <v>0.57599999999999996</v>
       </c>
       <c r="H16" s="3">
         <f>E16</f>
-        <v>4.08</v>
+        <v>0.72</v>
       </c>
       <c r="I16" s="3">
         <f>1.2*H16</f>
-        <v>4.8959999999999999</v>
+        <v>0.86399999999999999</v>
       </c>
       <c r="J16" s="3"/>
       <c r="K16" s="3" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">
@@ -1482,10 +1482,10 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>21</v>
@@ -1508,7 +1508,7 @@
       </c>
       <c r="J18" s="3"/>
       <c r="K18" s="3" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
default to 80-120% uniform for uncertainty in raw material purchase prices
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saran\Documents\Academia\repository_clones\Bioindustrial-Park\biorefineries\isobutanol\analyses\full\parameter_distributions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EEB212C-82B1-4CCC-BF55-6EB86BD9AD25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D34303BB-A1B5-46C8-9072-A86A70FA1727}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1325,19 +1325,19 @@
         <v>0.10355</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="G13" s="6">
-        <f>E13*0.9</f>
-        <v>9.3195E-2</v>
+        <f>E13*0.8</f>
+        <v>8.2840000000000011E-2</v>
       </c>
       <c r="H13" s="6">
         <f>E13</f>
         <v>0.10355</v>
       </c>
       <c r="I13" s="6">
-        <f>E13*1.1</f>
-        <v>0.11390500000000001</v>
+        <f>E13*1.2</f>
+        <v>0.12426</v>
       </c>
       <c r="J13" s="6"/>
       <c r="K13" s="6" t="s">

</xml_diff>

<commit_message>
update for nsk reset call refactor
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saran\Documents\Academia\repository_clones\Bioindustrial-Park\biorefineries\isobutanol\analyses\full\parameter_distributions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D34303BB-A1B5-46C8-9072-A86A70FA1727}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11D9513E-CA76-42FF-9D18-367610097181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1331,10 +1331,7 @@
         <f>E13*0.8</f>
         <v>8.2840000000000011E-2</v>
       </c>
-      <c r="H13" s="6">
-        <f>E13</f>
-        <v>0.10355</v>
-      </c>
+      <c r="H13" s="6"/>
       <c r="I13" s="6">
         <f>E13*1.2</f>
         <v>0.12426</v>

</xml_diff>

<commit_message>
update for nskinetics rename of kinetic_reaction_system to nsk_kinetic_model
Rename attribute references across system, utils, analyses, and the
scenario A/B parameter-distributions xlsx setter statements; matches
nskinetics a0f7c11. Smoke tests validated (A ~0.745, B ~0.991, 2x each).
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
@@ -206,31 +206,31 @@
     <t>V514.tau = x</t>
   </si>
   <si>
-    <t>V406.kinetic_reaction_system._te.k_2 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_1e = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_1h = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_1ie = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_1ia = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_1ii = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_1l = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_3 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_4 = x</t>
+    <t>V406.nsk_kinetic_model._te.k_2 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_1e = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_1h = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_1ie = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_1ia = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_1ii = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_1l = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_3 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_4 = x</t>
   </si>
   <si>
     <t>g_per_l_per_h</t>
@@ -242,55 +242,55 @@
     <t>g_per_l</t>
   </si>
   <si>
-    <t>V406.kinetic_reaction_system._te.k_4ie = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_4ia = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_4ii = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_5 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_5e = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_6 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_6r = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_7 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_7ie = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_7ia = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_7ii = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_8 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_9 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_9e = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_9c = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_10 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_11 = x</t>
+    <t>V406.nsk_kinetic_model._te.k_4ie = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_4ia = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_4ii = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_5 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_5e = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_6 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_6r = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_7 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_7ie = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_7ia = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_7ii = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_8 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_9 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_9e = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_9c = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_10 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_11 = x</t>
   </si>
   <si>
     <t>lime.price = x</t>
@@ -299,55 +299,55 @@
     <t>sulfuric_acid.price = x</t>
   </si>
   <si>
-    <t>V406.kinetic_reaction_system._te.K_1l = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_1h = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_1i = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_1e = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_2 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_2i = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_3 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_4 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_5 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_5e = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_5i = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_6 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_6e = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_7 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_9 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_9e = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_9i = x</t>
+    <t>V406.nsk_kinetic_model._te.K_1l = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_1h = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_1i = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_1e = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_2 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_2i = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_3 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_4 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_5 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_5e = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_5i = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_6 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_6e = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_7 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_9 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_9e = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_9i = x</t>
   </si>
   <si>
     <t>K_1l</t>

</xml_diff>

<commit_message>
data(distributions): price rows in 2023 dollars in both scenario workbooks
The 2026-09-02 price-year indexing (432943d1) rewrote the baseline price
rows of the A and B parameter-distribution workbooks in 2023$ (feedstock
0.139 -> 0.174 $/wet-kg, electricity 0.07 -> 0.093 $/kWh, ammonia, yeast,
amylases, denaturant, DDGS, lime, sulfuric acid; B's isobutanol 1.49 ->
1.50 $/kg) but the workbooks themselves were left uncommitted.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.139</v>
+        <v>0.17414</v>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
@@ -621,15 +621,19 @@
         </is>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.127</v>
+        <v>0.15911</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0.139</v>
+        <v>0.17414</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="J4" s="6" t="n"/>
+        <v>0.18792</v>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>2023$ = source value x 1.2528 (BLS PPI WPU06 2023/2017); source: USDA NASS 2015-2019 mean 3.543 $/bu (0.139 $/kg; 5th/95th pct 0.127/0.150), nominal, taken as 2017$</t>
+        </is>
+      </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
           <t>feedstock.price = x</t>
@@ -658,7 +662,7 @@
         </is>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.09289600000000001</v>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
@@ -666,15 +670,19 @@
         </is>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.067</v>
+        <v>0.08891499999999999</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.09289600000000001</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>0.074</v>
-      </c>
-      <c r="J5" s="6" t="n"/>
+        <v>0.098204</v>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>2023$ = source value x 1.3271 (BLS PPI WPU06 2023/2016); source: EIA AEO 2010-2019 average 0.070 $/kWh (0.067-0.074), 2016$ per HP/process_settings</t>
+        </is>
+      </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
           <t>PowerUtility.price = x</t>
@@ -703,7 +711,7 @@
         </is>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0.449</v>
+        <v>0.53521</v>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
@@ -711,13 +719,17 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.3592</v>
+        <v>0.42817</v>
       </c>
       <c r="H6" s="4" t="n"/>
       <c r="I6" s="4" t="n">
-        <v>0.5387999999999999</v>
-      </c>
-      <c r="J6" s="4" t="n"/>
+        <v>0.64225</v>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>2023$ = source value x 1.1920 (BLS PPI WPU06 2023/2018); source: corn package default 0.449 $/kg (Kurambhatti et al. 2019), 2018$</t>
+        </is>
+      </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
           <t>ammonia.price = x</t>
@@ -746,7 +758,7 @@
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>1.86</v>
+        <v>2.2171</v>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
@@ -754,13 +766,17 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>1.488</v>
+        <v>1.7737</v>
       </c>
       <c r="H7" s="4" t="n"/>
       <c r="I7" s="4" t="n">
-        <v>2.232</v>
-      </c>
-      <c r="J7" s="4" t="n"/>
+        <v>2.6606</v>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>2023$ = source value x 1.1920 (BLS PPI WPU06 2023/2018); source: corn package default 1.86 $/kg (Kurambhatti et al. 2019), 2018$</t>
+        </is>
+      </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
           <t>yeast.price = x</t>
@@ -789,7 +805,7 @@
         </is>
       </c>
       <c r="E8" s="4" t="n">
-        <v>2.25</v>
+        <v>2.682</v>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
@@ -797,13 +813,17 @@
         </is>
       </c>
       <c r="G8" s="4" t="n">
-        <v>1.8</v>
+        <v>2.1456</v>
       </c>
       <c r="H8" s="4" t="n"/>
       <c r="I8" s="4" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="J8" s="4" t="n"/>
+        <v>3.2184</v>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>2023$ = source value x 1.1920 (BLS PPI WPU06 2023/2018); source: corn package default 2.25 $/kg (Kurambhatti et al. 2019), 2018$</t>
+        </is>
+      </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
           <t>alpha_amylase.price = x</t>
@@ -832,7 +852,7 @@
         </is>
       </c>
       <c r="E9" s="4" t="n">
-        <v>2.25</v>
+        <v>2.682</v>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
@@ -840,13 +860,17 @@
         </is>
       </c>
       <c r="G9" s="4" t="n">
-        <v>1.8</v>
+        <v>2.1456</v>
       </c>
       <c r="H9" s="4" t="n"/>
       <c r="I9" s="4" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="J9" s="4" t="n"/>
+        <v>3.2184</v>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>2023$ = source value x 1.1920 (BLS PPI WPU06 2023/2018); source: corn package default 2.25 $/kg (Kurambhatti et al. 2019), 2018$</t>
+        </is>
+      </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
           <t>gluco_amylase.price = x</t>
@@ -875,7 +899,7 @@
         </is>
       </c>
       <c r="E10" s="4" t="n">
-        <v>0.436</v>
+        <v>0.51972</v>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
@@ -883,13 +907,17 @@
         </is>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.3488</v>
+        <v>0.41577</v>
       </c>
       <c r="H10" s="4" t="n"/>
       <c r="I10" s="4" t="n">
-        <v>0.5232</v>
-      </c>
-      <c r="J10" s="4" t="n"/>
+        <v>0.62366</v>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>2023$ = source value x 1.1920 (BLS PPI WPU06 2023/2018); source: corn package default 0.436 $/kg (Kurambhatti et al. 2019), 2018$</t>
+        </is>
+      </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
           <t>denaturant.price = x</t>
@@ -918,7 +946,7 @@
         </is>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0.12</v>
+        <v>0.14304</v>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
@@ -926,13 +954,17 @@
         </is>
       </c>
       <c r="G11" s="4" t="n">
-        <v>0.096</v>
+        <v>0.11443</v>
       </c>
       <c r="H11" s="4" t="n"/>
       <c r="I11" s="4" t="n">
-        <v>0.144</v>
-      </c>
-      <c r="J11" s="4" t="n"/>
+        <v>0.17165</v>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>2023$ = source value x 1.1920 (BLS PPI WPU06 2023/2018); source: corn package default 0.12 $/kg (Kurambhatti et al. 2019), 2018$</t>
+        </is>
+      </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
           <t>DDGS.price =x</t>
@@ -961,7 +993,7 @@
         </is>
       </c>
       <c r="E12" s="6" t="n">
-        <v>0.286</v>
+        <v>0.34802</v>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
@@ -969,15 +1001,19 @@
         </is>
       </c>
       <c r="G12" s="6" t="n">
-        <v>0.175</v>
+        <v>0.21295</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>0.286</v>
+        <v>0.34802</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>0.315</v>
-      </c>
-      <c r="J12" s="6" t="n"/>
+        <v>0.38331</v>
+      </c>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>2023$ = source value x 1.2168 (BLS PPI WPU06 2023/2019); source: HP/process_settings 0.286 $/kg (0.175-0.315), 2019$</t>
+        </is>
+      </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
           <t>lime.price = x</t>
@@ -1006,7 +1042,7 @@
         </is>
       </c>
       <c r="E13" s="6" t="n">
-        <v>0.10355</v>
+        <v>0.126</v>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
@@ -1014,13 +1050,17 @@
         </is>
       </c>
       <c r="G13" s="6" t="n">
-        <v>0.08284000000000001</v>
+        <v>0.1008</v>
       </c>
       <c r="H13" s="6" t="n"/>
       <c r="I13" s="6" t="n">
-        <v>0.12426</v>
-      </c>
-      <c r="J13" s="6" t="n"/>
+        <v>0.15121</v>
+      </c>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>2023$ = source value x 1.2168 (BLS PPI WPU06 2023/2019); source: HP/process_settings 0.10355 $/kg (+/-20%), 2019$</t>
+        </is>
+      </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
           <t>sulfuric_acid.price = x</t>

</xml_diff>

<commit_message>
data(distributions): exclude physically-constrained kinetic params from the uncertainty sweep
Remove parameters that should not carry a flat +/-20% band because they are fixed by thermodynamics or model structure rather than measured:
- k_6r (both), k_16r (B): reverse-rate ratios (thermodynamic; Haldane). Independent perturbation is inconsistent and can flip the ADH/Ehrlich net-flux sign.
- K_2, K_9 (both): structural always-saturated constants (>=3 orders below their substrate pools); no empirical band, null sensitivity. K_2i/K_3/K_4/K_13 kept (near-operating).
- P_10e/P_10a (both), P_10i (B): piecewise death-onset thresholds (switch, not gain -> discontinuous sensitivity).
Kinetic set: A 45->40, B 63->56. Ehrlich block otherwise unchanged. Rationale + citations in docs/reports/kinetic-parameter-exclusions.md (gitignored).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K64"/>
+  <dimension ref="A1:K59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="40.81640625" customWidth="1" min="1" max="1"/>
@@ -1786,7 +1786,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>K_2</t>
+          <t>K_2i</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1804,39 +1804,39 @@
           <t>g_per_l</t>
         </is>
       </c>
-      <c r="E30" s="5" t="n">
-        <v>2e-05</v>
+      <c r="E30" s="3" t="n">
+        <v>0.101</v>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
           <t>triangular</t>
         </is>
       </c>
-      <c r="G30" s="5" t="n">
-        <v>1.6e-05</v>
-      </c>
-      <c r="H30" s="5" t="n">
-        <v>2e-05</v>
-      </c>
-      <c r="I30" s="5" t="n">
-        <v>2.4e-05</v>
+      <c r="G30" s="3" t="n">
+        <v>0.08080000000000001</v>
+      </c>
+      <c r="H30" s="3" t="n">
+        <v>0.101</v>
+      </c>
+      <c r="I30" s="3" t="n">
+        <v>0.1212</v>
       </c>
       <c r="J30" s="3" t="n"/>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.K_2 = x</t>
+          <t>V406.nsk_kinetic_model._te.K_2i = x</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>K_2i</t>
+          <t>._k_3</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Kinetics: TCA Cycle</t>
+          <t>Kinetics: Pyruvate-to-Acetaldehyde</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -1846,11 +1846,11 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>g_per_l</t>
+          <t>g_per_l_per_h</t>
         </is>
       </c>
       <c r="E31" s="3" t="n">
-        <v>0.101</v>
+        <v>5.81</v>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
@@ -1858,25 +1858,25 @@
         </is>
       </c>
       <c r="G31" s="3" t="n">
-        <v>0.08080000000000001</v>
+        <v>4.648</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>0.101</v>
+        <v>5.81</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>0.1212</v>
+        <v>6.972</v>
       </c>
       <c r="J31" s="3" t="n"/>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.K_2i = x</t>
+          <t>V406.nsk_kinetic_model._te.k_3 = x</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>._k_3</t>
+          <t>K_3</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1891,42 +1891,42 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>g_per_l_per_h</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="n">
-        <v>5.81</v>
+          <t>g_per_l</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>5e-07</v>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
           <t>triangular</t>
         </is>
       </c>
-      <c r="G32" s="3" t="n">
-        <v>4.648</v>
-      </c>
-      <c r="H32" s="3" t="n">
-        <v>5.81</v>
-      </c>
-      <c r="I32" s="3" t="n">
-        <v>6.972</v>
+      <c r="G32" s="5" t="n">
+        <v>4e-07</v>
+      </c>
+      <c r="H32" s="5" t="n">
+        <v>5e-07</v>
+      </c>
+      <c r="I32" s="5" t="n">
+        <v>6e-07</v>
       </c>
       <c r="J32" s="3" t="n"/>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.k_3 = x</t>
+          <t>V406.nsk_kinetic_model._te.K_3 = x</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>K_3</t>
+          <t>._k_4</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Kinetics: Pyruvate-to-Acetaldehyde</t>
+          <t>Kinetics: Acetaldehyde-to-Acetate</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -1936,37 +1936,37 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>g_per_l</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="n">
-        <v>5e-07</v>
+          <t>g_per_l_per_h</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>4.8</v>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
           <t>triangular</t>
         </is>
       </c>
-      <c r="G33" s="5" t="n">
-        <v>4e-07</v>
-      </c>
-      <c r="H33" s="5" t="n">
-        <v>5e-07</v>
-      </c>
-      <c r="I33" s="5" t="n">
-        <v>6e-07</v>
+      <c r="G33" s="3" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="H33" s="3" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="I33" s="3" t="n">
+        <v>5.76</v>
       </c>
       <c r="J33" s="3" t="n"/>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.K_3 = x</t>
+          <t>V406.nsk_kinetic_model._te.k_4 = x</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>._k_4</t>
+          <t>._k_4ie</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1985,7 +1985,7 @@
         </is>
       </c>
       <c r="E34" s="3" t="n">
-        <v>4.8</v>
+        <v>0.04</v>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
@@ -1993,25 +1993,25 @@
         </is>
       </c>
       <c r="G34" s="3" t="n">
-        <v>3.84</v>
+        <v>0.032</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>4.8</v>
+        <v>0.04</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>5.76</v>
+        <v>0.048</v>
       </c>
       <c r="J34" s="3" t="n"/>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.k_4 = x</t>
+          <t>V406.nsk_kinetic_model._te.k_4ie = x</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>._k_4ie</t>
+          <t>._k_4ia</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -2030,7 +2030,7 @@
         </is>
       </c>
       <c r="E35" s="3" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
@@ -2038,25 +2038,25 @@
         </is>
       </c>
       <c r="G35" s="3" t="n">
-        <v>0.032</v>
+        <v>0.096</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>0.048</v>
+        <v>0.144</v>
       </c>
       <c r="J35" s="3" t="n"/>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.k_4ie = x</t>
+          <t>V406.nsk_kinetic_model._te.k_4ia = x</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>._k_4ia</t>
+          <t>K_4</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -2071,11 +2071,11 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>g_per_l_per_h</t>
+          <t>g_per_l</t>
         </is>
       </c>
       <c r="E36" s="3" t="n">
-        <v>0.12</v>
+        <v>0.000264</v>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
@@ -2083,30 +2083,30 @@
         </is>
       </c>
       <c r="G36" s="3" t="n">
-        <v>0.096</v>
+        <v>0.0002112</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>0.12</v>
+        <v>0.000264</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>0.144</v>
+        <v>0.0003168</v>
       </c>
       <c r="J36" s="3" t="n"/>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.k_4ia = x</t>
+          <t>V406.nsk_kinetic_model._te.K_4 = x</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>K_4</t>
+          <t>._k_5</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Kinetics: Acetaldehyde-to-Acetate</t>
+          <t>Kinetics: Acetate respiration</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -2116,11 +2116,11 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>g_per_l</t>
+          <t>g_per_l_per_h</t>
         </is>
       </c>
       <c r="E37" s="3" t="n">
-        <v>0.000264</v>
+        <v>0.0104</v>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
@@ -2128,25 +2128,25 @@
         </is>
       </c>
       <c r="G37" s="3" t="n">
-        <v>0.0002112</v>
+        <v>0.008319999999999999</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>0.000264</v>
+        <v>0.0104</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>0.0003168</v>
+        <v>0.01248</v>
       </c>
       <c r="J37" s="3" t="n"/>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.K_4 = x</t>
+          <t>V406.nsk_kinetic_model._te.k_5 = x</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>._k_5</t>
+          <t>K_5</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -2161,11 +2161,11 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>g_per_l_per_h</t>
+          <t>g_per_l</t>
         </is>
       </c>
       <c r="E38" s="3" t="n">
-        <v>0.0104</v>
+        <v>0.0102</v>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
@@ -2173,25 +2173,25 @@
         </is>
       </c>
       <c r="G38" s="3" t="n">
-        <v>0.008319999999999999</v>
+        <v>0.008160000000000001</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>0.0104</v>
+        <v>0.0102</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>0.01248</v>
+        <v>0.01224</v>
       </c>
       <c r="J38" s="3" t="n"/>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.k_5 = x</t>
+          <t>V406.nsk_kinetic_model._te.K_5 = x</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>K_5</t>
+          <t>._k_5e</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -2206,11 +2206,11 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>g_per_l</t>
+          <t>g_per_l_per_h</t>
         </is>
       </c>
       <c r="E39" s="3" t="n">
-        <v>0.0102</v>
+        <v>0.775</v>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
@@ -2218,25 +2218,25 @@
         </is>
       </c>
       <c r="G39" s="3" t="n">
-        <v>0.008160000000000001</v>
+        <v>0.6200000000000001</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>0.0102</v>
+        <v>0.775</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>0.01224</v>
+        <v>0.9299999999999999</v>
       </c>
       <c r="J39" s="3" t="n"/>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.K_5 = x</t>
+          <t>V406.nsk_kinetic_model._te.k_5e = x</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>._k_5e</t>
+          <t>K_5e</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -2251,11 +2251,11 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>g_per_l_per_h</t>
+          <t>g_per_l</t>
         </is>
       </c>
       <c r="E40" s="3" t="n">
-        <v>0.775</v>
+        <v>0.1</v>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
@@ -2263,25 +2263,25 @@
         </is>
       </c>
       <c r="G40" s="3" t="n">
-        <v>0.6200000000000001</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>0.775</v>
+        <v>0.1</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>0.9299999999999999</v>
+        <v>0.12</v>
       </c>
       <c r="J40" s="3" t="n"/>
       <c r="K40" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.k_5e = x</t>
+          <t>V406.nsk_kinetic_model._te.K_5e = x</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>K_5e</t>
+          <t>K_5i</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -2300,7 +2300,7 @@
         </is>
       </c>
       <c r="E41" s="3" t="n">
-        <v>0.1</v>
+        <v>440</v>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
@@ -2308,30 +2308,30 @@
         </is>
       </c>
       <c r="G41" s="3" t="n">
-        <v>0.08000000000000002</v>
+        <v>352</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>0.1</v>
+        <v>440</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>0.12</v>
+        <v>528</v>
       </c>
       <c r="J41" s="3" t="n"/>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.K_5e = x</t>
+          <t>V406.nsk_kinetic_model._te.K_5i = x</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>K_5i</t>
+          <t>._k_6</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Kinetics: Acetate respiration</t>
+          <t>Kinetics: Acetaldyhede-to-Ethanol</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -2341,11 +2341,11 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>g_per_l</t>
+          <t>g_per_l_per_h</t>
         </is>
       </c>
       <c r="E42" s="3" t="n">
-        <v>440</v>
+        <v>2.82</v>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
@@ -2353,25 +2353,25 @@
         </is>
       </c>
       <c r="G42" s="3" t="n">
-        <v>352</v>
+        <v>2.256</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>440</v>
+        <v>2.82</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>528</v>
+        <v>3.384</v>
       </c>
       <c r="J42" s="3" t="n"/>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.K_5i = x</t>
+          <t>V406.nsk_kinetic_model._te.k_6 = x</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>._k_6</t>
+          <t>K_6</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -2386,11 +2386,11 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>g_per_l_per_h</t>
+          <t>g_per_l</t>
         </is>
       </c>
       <c r="E43" s="3" t="n">
-        <v>2.82</v>
+        <v>0.034</v>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
@@ -2398,25 +2398,25 @@
         </is>
       </c>
       <c r="G43" s="3" t="n">
-        <v>2.256</v>
+        <v>0.0272</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>2.82</v>
+        <v>0.034</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>3.384</v>
+        <v>0.0408</v>
       </c>
       <c r="J43" s="3" t="n"/>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.k_6 = x</t>
+          <t>V406.nsk_kinetic_model._te.K_6 = x</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>._k_6r</t>
+          <t>K_6e</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -2431,11 +2431,11 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>g_per_l_per_h</t>
+          <t>g_per_l</t>
         </is>
       </c>
       <c r="E44" s="3" t="n">
-        <v>0.0125</v>
+        <v>0.057</v>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
@@ -2443,75 +2443,74 @@
         </is>
       </c>
       <c r="G44" s="3" t="n">
-        <v>0.01</v>
+        <v>0.0456</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>0.0125</v>
+        <v>0.057</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>0.015</v>
+        <v>0.0684</v>
       </c>
       <c r="J44" s="3" t="n"/>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.k_6r = x</t>
+          <t>V406.nsk_kinetic_model._te.K_6e = x</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>K_6</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>._k_6ia</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
         <is>
           <t>Kinetics: Acetaldyhede-to-Ethanol</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>coupled</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>g_per_l</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="n">
-        <v>0.034</v>
-      </c>
-      <c r="F45" s="3" t="inlineStr">
-        <is>
-          <t>triangular</t>
-        </is>
-      </c>
-      <c r="G45" s="3" t="n">
-        <v>0.0272</v>
-      </c>
-      <c r="H45" s="3" t="n">
-        <v>0.034</v>
-      </c>
-      <c r="I45" s="3" t="n">
-        <v>0.0408</v>
-      </c>
-      <c r="J45" s="3" t="n"/>
-      <c r="K45" s="3" t="inlineStr">
-        <is>
-          <t>V406.nsk_kinetic_model._te.K_6 = x</t>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>coupled</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>g_per_l_per_h</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>triangular</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0.07199999999999999</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>V406.nsk_kinetic_model._te.k_6ia = x</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>K_6e</t>
+          <t>._k_7</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Kinetics: Acetaldyhede-to-Ethanol</t>
+          <t>Kinetics: Glucose-to-Biomass</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -2521,11 +2520,11 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>g_per_l</t>
+          <t>g_per_l_per_h</t>
         </is>
       </c>
       <c r="E46" s="3" t="n">
-        <v>0.057</v>
+        <v>1.203</v>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
@@ -2533,69 +2532,70 @@
         </is>
       </c>
       <c r="G46" s="3" t="n">
-        <v>0.0456</v>
+        <v>0.9624000000000001</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>0.057</v>
+        <v>1.203</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>0.0684</v>
+        <v>1.4436</v>
       </c>
       <c r="J46" s="3" t="n"/>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.K_6e = x</t>
+          <t>V406.nsk_kinetic_model._te.k_7 = x</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>._k_6ia</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Kinetics: Acetaldyhede-to-Ethanol</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>coupled</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>._k_7ie</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Kinetics: Glucose-to-Biomass</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>coupled</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>g_per_l_per_h</t>
         </is>
       </c>
-      <c r="E47" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>triangular</t>
-        </is>
-      </c>
-      <c r="G47" t="n">
+      <c r="E47" s="3" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>triangular</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="H47" s="3" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="I47" s="3" t="n">
         <v>0.048</v>
       </c>
-      <c r="H47" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="I47" t="n">
-        <v>0.07199999999999999</v>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>V406.nsk_kinetic_model._te.k_6ia = x</t>
+      <c r="J47" s="3" t="n"/>
+      <c r="K47" s="3" t="inlineStr">
+        <is>
+          <t>V406.nsk_kinetic_model._te.k_7ie = x</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>._k_7</t>
+          <t>._k_7ia</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -2614,7 +2614,7 @@
         </is>
       </c>
       <c r="E48" s="3" t="n">
-        <v>1.203</v>
+        <v>0.12</v>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
@@ -2622,25 +2622,25 @@
         </is>
       </c>
       <c r="G48" s="3" t="n">
-        <v>0.9624000000000001</v>
+        <v>0.096</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>1.203</v>
+        <v>0.12</v>
       </c>
       <c r="I48" s="3" t="n">
-        <v>1.4436</v>
+        <v>0.144</v>
       </c>
       <c r="J48" s="3" t="n"/>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.k_7 = x</t>
+          <t>V406.nsk_kinetic_model._te.k_7ia = x</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>._k_7ie</t>
+          <t>K_7</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -2655,11 +2655,11 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>g_per_l_per_h</t>
+          <t>g_per_l</t>
         </is>
       </c>
       <c r="E49" s="3" t="n">
-        <v>0.04</v>
+        <v>0.0101</v>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
@@ -2667,30 +2667,30 @@
         </is>
       </c>
       <c r="G49" s="3" t="n">
-        <v>0.032</v>
+        <v>0.00808</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>0.04</v>
+        <v>0.0101</v>
       </c>
       <c r="I49" s="3" t="n">
-        <v>0.048</v>
+        <v>0.01212</v>
       </c>
       <c r="J49" s="3" t="n"/>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.k_7ie = x</t>
+          <t>V406.nsk_kinetic_model._te.K_7 = x</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>._k_7ia</t>
+          <t>._k_8</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Kinetics: Glucose-to-Biomass</t>
+          <t>Kinetics: Acetate-to-Biomass</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -2704,7 +2704,7 @@
         </is>
       </c>
       <c r="E50" s="3" t="n">
-        <v>0.12</v>
+        <v>0.589</v>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
@@ -2712,30 +2712,30 @@
         </is>
       </c>
       <c r="G50" s="3" t="n">
-        <v>0.096</v>
+        <v>0.4712</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>0.12</v>
+        <v>0.589</v>
       </c>
       <c r="I50" s="3" t="n">
-        <v>0.144</v>
+        <v>0.7068</v>
       </c>
       <c r="J50" s="3" t="n"/>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.k_7ia = x</t>
+          <t>V406.nsk_kinetic_model._te.k_8 = x</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>K_7</t>
+          <t>._k_9</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Kinetics: Glucose-to-Biomass</t>
+          <t>Kinetics: Acetalhdyde compartment formation</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -2745,11 +2745,11 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>g_per_l</t>
+          <t>g_per_l_per_h</t>
         </is>
       </c>
       <c r="E51" s="3" t="n">
-        <v>0.0101</v>
+        <v>0.008</v>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
@@ -2757,30 +2757,30 @@
         </is>
       </c>
       <c r="G51" s="3" t="n">
-        <v>0.00808</v>
+        <v>0.0064</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>0.0101</v>
+        <v>0.008</v>
       </c>
       <c r="I51" s="3" t="n">
-        <v>0.01212</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="J51" s="3" t="n"/>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.K_7 = x</t>
+          <t>V406.nsk_kinetic_model._te.k_9 = x</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>._k_8</t>
+          <t>._k_9e</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Kinetics: Acetate-to-Biomass</t>
+          <t>Kinetics: Acetalhdyde compartment formation</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -2794,7 +2794,7 @@
         </is>
       </c>
       <c r="E52" s="3" t="n">
-        <v>0.589</v>
+        <v>0.0751</v>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
@@ -2802,25 +2802,25 @@
         </is>
       </c>
       <c r="G52" s="3" t="n">
-        <v>0.4712</v>
+        <v>0.06008</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>0.589</v>
+        <v>0.0751</v>
       </c>
       <c r="I52" s="3" t="n">
-        <v>0.7068</v>
+        <v>0.09011999999999999</v>
       </c>
       <c r="J52" s="3" t="n"/>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.k_8 = x</t>
+          <t>V406.nsk_kinetic_model._te.k_9e = x</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>._k_9</t>
+          <t>K_9e</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -2835,11 +2835,11 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>g_per_l_per_h</t>
+          <t>g_per_l</t>
         </is>
       </c>
       <c r="E53" s="3" t="n">
-        <v>0.008</v>
+        <v>13</v>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
@@ -2847,25 +2847,25 @@
         </is>
       </c>
       <c r="G53" s="3" t="n">
-        <v>0.0064</v>
+        <v>10.4</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>0.008</v>
+        <v>13</v>
       </c>
       <c r="I53" s="3" t="n">
-        <v>0.009599999999999999</v>
+        <v>15.6</v>
       </c>
       <c r="J53" s="3" t="n"/>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.k_9 = x</t>
+          <t>V406.nsk_kinetic_model._te.K_9e = x</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>K_9</t>
+          <t>K_9i</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -2883,34 +2883,34 @@
           <t>g_per_l</t>
         </is>
       </c>
-      <c r="E54" s="5" t="n">
-        <v>1e-06</v>
+      <c r="E54" s="3" t="n">
+        <v>25</v>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
           <t>triangular</t>
         </is>
       </c>
-      <c r="G54" s="5" t="n">
-        <v>8e-07</v>
-      </c>
-      <c r="H54" s="5" t="n">
-        <v>1e-06</v>
-      </c>
-      <c r="I54" s="5" t="n">
-        <v>1.2e-06</v>
+      <c r="G54" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H54" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="I54" s="3" t="n">
+        <v>30</v>
       </c>
       <c r="J54" s="3" t="n"/>
       <c r="K54" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.K_9 = x</t>
+          <t>V406.nsk_kinetic_model._te.K_9i = x</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>._k_9e</t>
+          <t>._k_9c</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="E55" s="3" t="n">
-        <v>0.0751</v>
+        <v>0.00399</v>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
@@ -2937,30 +2937,30 @@
         </is>
       </c>
       <c r="G55" s="3" t="n">
-        <v>0.06008</v>
+        <v>0.003192</v>
       </c>
       <c r="H55" s="3" t="n">
-        <v>0.0751</v>
+        <v>0.00399</v>
       </c>
       <c r="I55" s="3" t="n">
-        <v>0.09011999999999999</v>
+        <v>0.004788</v>
       </c>
       <c r="J55" s="3" t="n"/>
       <c r="K55" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.k_9e = x</t>
+          <t>V406.nsk_kinetic_model._te.k_9c = x</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>K_9e</t>
+          <t>._k_10</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Kinetics: Acetalhdyde compartment formation</t>
+          <t>Kinetics: Active compartment degradation</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -2970,11 +2970,11 @@
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>g_per_l</t>
+          <t>g_per_l_per_h</t>
         </is>
       </c>
       <c r="E56" s="3" t="n">
-        <v>13</v>
+        <v>0.06</v>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
@@ -2982,120 +2982,118 @@
         </is>
       </c>
       <c r="G56" s="3" t="n">
-        <v>10.4</v>
+        <v>0.048</v>
       </c>
       <c r="H56" s="3" t="n">
-        <v>13</v>
+        <v>0.06</v>
       </c>
       <c r="I56" s="3" t="n">
-        <v>15.6</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="J56" s="3" t="n"/>
       <c r="K56" s="3" t="inlineStr">
         <is>
-          <t>V406.nsk_kinetic_model._te.K_9e = x</t>
+          <t>V406.nsk_kinetic_model._te.k_10 = x</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="3" t="inlineStr">
-        <is>
-          <t>K_9i</t>
-        </is>
-      </c>
-      <c r="B57" s="3" t="inlineStr">
-        <is>
-          <t>Kinetics: Acetalhdyde compartment formation</t>
-        </is>
-      </c>
-      <c r="C57" s="3" t="inlineStr">
-        <is>
-          <t>coupled</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>g_per_l</t>
-        </is>
-      </c>
-      <c r="E57" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="F57" s="3" t="inlineStr">
-        <is>
-          <t>triangular</t>
-        </is>
-      </c>
-      <c r="G57" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="H57" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="I57" s="3" t="n">
-        <v>30</v>
-      </c>
-      <c r="J57" s="3" t="n"/>
-      <c r="K57" s="3" t="inlineStr">
-        <is>
-          <t>V406.nsk_kinetic_model._te.K_9i = x</t>
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>._k_10ie</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Kinetics: Active compartment degradation</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>coupled</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>g_per_l_per_h</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>triangular</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="H57" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="I57" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>V406.nsk_kinetic_model._te.k_10ie = x</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>._k_9c</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="inlineStr">
-        <is>
-          <t>Kinetics: Acetalhdyde compartment formation</t>
-        </is>
-      </c>
-      <c r="C58" s="3" t="inlineStr">
-        <is>
-          <t>coupled</t>
-        </is>
-      </c>
-      <c r="D58" s="3" t="inlineStr">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>._k_10ia</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Kinetics: Active compartment degradation</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>coupled</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
         <is>
           <t>g_per_l_per_h</t>
         </is>
       </c>
-      <c r="E58" s="3" t="n">
-        <v>0.00399</v>
-      </c>
-      <c r="F58" s="3" t="inlineStr">
-        <is>
-          <t>triangular</t>
-        </is>
-      </c>
-      <c r="G58" s="3" t="n">
-        <v>0.003192</v>
-      </c>
-      <c r="H58" s="3" t="n">
-        <v>0.00399</v>
-      </c>
-      <c r="I58" s="3" t="n">
-        <v>0.004788</v>
-      </c>
-      <c r="J58" s="3" t="n"/>
-      <c r="K58" s="3" t="inlineStr">
-        <is>
-          <t>V406.nsk_kinetic_model._te.k_9c = x</t>
+      <c r="E58" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>triangular</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I58" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>V406.nsk_kinetic_model._te.k_10ia = x</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>._k_10</t>
+          <t>._k_11</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Kinetics: Active compartment degradation</t>
+          <t>Kinetics: Acetaldehyde compartment degradation</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -3109,7 +3107,7 @@
         </is>
       </c>
       <c r="E59" s="3" t="n">
-        <v>0.06</v>
+        <v>0.02</v>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
@@ -3117,237 +3115,16 @@
         </is>
       </c>
       <c r="G59" s="3" t="n">
-        <v>0.048</v>
+        <v>0.016</v>
       </c>
       <c r="H59" s="3" t="n">
-        <v>0.06</v>
+        <v>0.02</v>
       </c>
       <c r="I59" s="3" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.024</v>
       </c>
       <c r="J59" s="3" t="n"/>
       <c r="K59" s="3" t="inlineStr">
-        <is>
-          <t>V406.nsk_kinetic_model._te.k_10 = x</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>._k_10ie</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Kinetics: Active compartment degradation</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>coupled</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>g_per_l_per_h</t>
-        </is>
-      </c>
-      <c r="E60" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>triangular</t>
-        </is>
-      </c>
-      <c r="G60" t="n">
-        <v>0.032</v>
-      </c>
-      <c r="H60" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="I60" t="n">
-        <v>0.048</v>
-      </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>V406.nsk_kinetic_model._te.k_10ie = x</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>._k_10ia</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Kinetics: Active compartment degradation</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>coupled</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>g_per_l_per_h</t>
-        </is>
-      </c>
-      <c r="E61" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>triangular</t>
-        </is>
-      </c>
-      <c r="G61" t="n">
-        <v>0.096</v>
-      </c>
-      <c r="H61" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="I61" t="n">
-        <v>0.144</v>
-      </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>V406.nsk_kinetic_model._te.k_10ia = x</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>P_10e</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Kinetics: Active compartment degradation</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>coupled</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>g_per_l</t>
-        </is>
-      </c>
-      <c r="E62" t="n">
-        <v>100</v>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>triangular</t>
-        </is>
-      </c>
-      <c r="G62" t="n">
-        <v>80</v>
-      </c>
-      <c r="H62" t="n">
-        <v>100</v>
-      </c>
-      <c r="I62" t="n">
-        <v>120</v>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>V406.nsk_kinetic_model._te.P_10e = x</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>P_10a</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Kinetics: Active compartment degradation</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>coupled</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>g_per_l</t>
-        </is>
-      </c>
-      <c r="E63" t="n">
-        <v>5</v>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>triangular</t>
-        </is>
-      </c>
-      <c r="G63" t="n">
-        <v>4</v>
-      </c>
-      <c r="H63" t="n">
-        <v>5</v>
-      </c>
-      <c r="I63" t="n">
-        <v>6</v>
-      </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>V406.nsk_kinetic_model._te.P_10a = x</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="3" t="inlineStr">
-        <is>
-          <t>._k_11</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>Kinetics: Acetaldehyde compartment degradation</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="inlineStr">
-        <is>
-          <t>coupled</t>
-        </is>
-      </c>
-      <c r="D64" s="3" t="inlineStr">
-        <is>
-          <t>g_per_l_per_h</t>
-        </is>
-      </c>
-      <c r="E64" s="3" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="F64" s="3" t="inlineStr">
-        <is>
-          <t>triangular</t>
-        </is>
-      </c>
-      <c r="G64" s="3" t="n">
-        <v>0.016</v>
-      </c>
-      <c r="H64" s="3" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="I64" s="3" t="n">
-        <v>0.024</v>
-      </c>
-      <c r="J64" s="3" t="n"/>
-      <c r="K64" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_11 = x</t>
         </is>

</xml_diff>